<commit_message>
feat(gt): synchronize all Tier 1 flagship papers directly with OpenAlex JSON recent works and full abstracts
</commit_message>
<xml_diff>
--- a/universities_wise/georgia_tech_university/georgia_tech_aerospace_mechanical_faculty.xlsx
+++ b/universities_wise/georgia_tech_university/georgia_tech_aerospace_mechanical_faculty.xlsx
@@ -807,64 +807,64 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>High-fidelity LES of supercritical-pressure reacting flows -- combining real-fluid thermodynamics, finite-rate chemistry, and subgrid turbulence closures to resolve transcritical LOX/CH4 injection, flame stabilization, and combustion instability in rocket and gas-turbine combustors.</t>
+          <t>Lagrangian coherent structures (LCS), finite-time Lyapunov exponent (FTLE) ridges, and adjoint-based receptivity/biorthogonal decomposition in compressible turbulent reacting shear layers.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>LES (Peng-Robinson real-fluid EOS), Finite-rate GRI-Mech 3.0 chemistry, Dynamic Smagorinsky subgrid, Transcritical jet DNS, RAPTOR high-performance CFD solver</t>
+          <t>Direct Numerical Simulation (DNS), Forward/backward FTLE ridges, Hyperbolic geodesic LCS, Cauchy-Green deformation tensors, Direct/adjoint biorthogonal eigenmode projection</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Large eddy simulation of a supercritical LOX/CH4 round jet flame</t>
+          <t>Planar Lagrangian transport and scalar-gradient organization in a turbulent reacting shear layer</t>
         </is>
       </c>
       <c r="P2" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2022.112183", "https://doi.org/10.1016/j.combustflame.2022.112183")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2606.20352", "https://doi.org/10.48550/arxiv.2606.20352")</f>
         <v/>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>performing real-fluid LES with Peng-Robinson EOS in a supercritical LOX/CH4 jet flame at 6 MPa, demonstrating that transcritical pseudoboiling produces a LOX core of L_c/D = 4.8 and anchors the diffusion flame within 2 jet diameters at the pseudoboiling interface.</t>
+          <t>analyzing 3D DNS of a supersonic reacting H2-air temporal mixing layer via hyperbolic geodesic LCS and FTLE ridges, demonstrating that forward/backward ridge intersections govern localized scalar-gradient enrichment and strain-dominated transport skeletons.</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>LES of a turbulent supercritical LOX/CH4 round jet flame at 6 MPa using RAPTOR with Peng-Robinson real-fluid EOS. The pseudoboiling transition of LOX injected at 120 K into supercritical methane at 300 K produces a dense LOX core of L_c/D = 4.8. Flame stabilization occurs within 2 jet diameters at the highest-density-gradient pseudoboiling interface.</t>
+          <t>We analyze planar Lagrangian transport and scalar-gradient organization in a supersonic, reacting hydrogen-air temporal mixing layer using time-resolved mid-plane data from a three-dimensional direct numerical simulation. The analysis combines forward/backward finite-time Lyapunov exponent (FTLE) fields, operational FTLE-ridge skeletons, Cauchy-Green deformation measures, shear-LCS metrics, and planar hyperbolic geodesic-LCS extraction to examine how finite-time stretching structures the reacting shear layer. The time-resolved FTLE ridges identify repelling and attracting finite-time transport skeletons in the constrained two-dimensional slice, from which ridge geometry, intersection occupancy, persistence, and scalar-conditioned transport are quantified. Hyperbolic geodesic LCS are extracted from Cauchy-Green tensors reconstructed from planar flow maps as strainlines seeded at high-$λ_{\max}$ normal maxima, providing a variational counterpart to the operational FTLE-ridge skeleton. We then relate the transport skeleton to temperature, mixture fraction, and a reaction intermediate. The results show localized forward/backward ridge overlap, strong scalar-gradient enrichment, fini...</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>Analysis of Mixing, Thermodynamic, and Combustion Characteristics of Turbulent Supercritical Flows</t>
+          <t>Receptivity and Biorthogonal Decomposition in a Reacting Temporal Mixing Layer</t>
         </is>
       </c>
       <c r="T2" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.J059845", "https://doi.org/10.2514/1.J059845")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2606.20819", "https://doi.org/10.48550/arxiv.2606.20819")</f>
         <v/>
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>combining DNS and LES with Peng-Robinson real-fluid EOS across three supercritical configurations at 6-10 MPa, demonstrating that density stratification suppresses scalar dissipation rate by 23% near the critical point and sustains sub-centimeter density gradients through the reacting zone.</t>
+          <t>applying energy-weighted adjoint projections and biorthogonal decomposition to a compressible reacting mixing layer, demonstrating that finite-thickness base states sustain unstable Kelvin-Helmholtz modes across low wavenumbers where vortex-sheet approximations remain neutral.</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>DNS and LES with Peng-Robinson EOS study three supercritical configurations: a N2 jet, LOX/H2 shear layer, and LOX/CH4 injector at 10 MPa. Density stratification produces 23% reduction in scalar dissipation rate at the critical point. Sub-centimeter density gradients persist through the reaction zone in the LOX/CH4 injector LES.</t>
+          <t>We examine receptivity and biorthogonal decomposition in a reacting temporal mixing layer using direct and adjoint eigenmodes of a finite-thickness compressible linearized operator built from the mean reacting base state. The analysis focuses on the Kelvin--Helmholtz branch and asks how the reacting base state modifies the selected temporal instability, where localized forcing most efficiently excites it, and how strongly the associated modal family is represented in time-resolved planar simulation data. Receptivity maps are constructed for mass, momentum, thermal, and mixture-fraction forcing channels using an energy-weighted adjoint projection, with biorthogonality enforced by the corresponding direct--adjoint inner product. A complementary biorthogonal decomposition provides modal amplitudes and cumulative few-mode reconstructions at the fundamental streamwise wavenumber. The finite-thickness branch is interpreted against a compressible vortex-sheet reference built from the outer-stream states. The reacting layer supports an unstable finite-thickness Kelvin--Helmholtz family over low-to-moderate wavenumbers even though the discontinuous reference is essentially neutral. Mass ...</t>
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>1. LES of a supercritical LOX/CH4 round jet flame (Combustion and Flame, 2022) | 2. Analysis of Mixing, Thermodynamic, and Combustion Characteristics of Turbulent Supercritical Flows (AIAA J., 2021)</t>
+          <t>1. Planar Lagrangian transport and scalar-gradient organization in a turbulent reacting shear layer (arXiv, 2026) | 2. Receptivity and Biorthogonal Decomposition in a Reacting Temporal Mixing Layer (arXiv, 2026)</t>
         </is>
       </c>
       <c r="X2" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2022.112183 | https://doi.org/10.2514/1.J059845", "https://doi.org/10.1016/j.combustflame.2022.112183 | https://doi.org/10.2514/1.J059845")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2606.20352 | https://doi.org/10.48550/arxiv.2606.20819", "https://doi.org/10.48550/arxiv.2606.20352 | https://doi.org/10.48550/arxiv.2606.20819")</f>
         <v/>
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>performing real-fluid LES with Peng-Robinson EOS in a supercritical LOX/CH4 jet flame at 6 MPa, demonstrating that transcritical pseudoboiling produces a LOX core of L_c/D = 4.8 and anchors the diffusion flame within 2 jet diameters at the pseudoboiling interface.</t>
+          <t>analyzing 3D DNS of a supersonic reacting H2-air temporal mixing layer via hyperbolic geodesic LCS and FTLE ridges, demonstrating that forward/backward ridge intersections govern localized scalar-gradient enrichment and strain-dominated transport skeletons.</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1003,64 +1003,64 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>First-principles LES and DNS of supercritical combustion, rotating detonation engine (RDE) wave dynamics, and LOX/CH4 propellant injection physics -- resolving real-fluid thermodynamic non-idealities and turbulence-chemistry coupling at rocket-engine operating pressures.</t>
+          <t>Supersonic combustion dynamics in dual-combustion ramjet (DCR) engines, chemical explosive mode analysis (CEMA), and detonative tangential combustion instability mode transitions in liquid and gas rocket combustors.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>LES (real-fluid EOS, cubic Peng-Robinson EOS), DNS of supercritical jets, Modified Benedict-Webb-Rubin (MBWR) EOS, Finite-rate GRI-Mech 3.0 chemistry, RDE wave solvers</t>
+          <t>Chemical Explosive Mode Analysis (CEMA), STFT / Dynamic Mode Decomposition (DMD), Proper Orthogonal Decomposition (POD), Compressible reacting LES, High-order shock-capturing CFD</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Rotating detonation engine with a hollow annular channel: Effects of inlet geometry on wave dynamics</t>
+          <t>Supersonic Combustion and Flow Evolution in Dual-Combustion Ramjet Engine</t>
         </is>
       </c>
       <c r="P3" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2021.111763", "https://doi.org/10.1016/j.combustflame.2021.111763")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.b40184", "https://doi.org/10.2514/1.b40184")</f>
         <v/>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>performing 3D LES with finite-rate H2-O2 kinetics in a hollow annular RDE, demonstrating that inlet slot aspect ratio controls reactant layer thickness and shifts rotating detonation wave speed between 1820 and 2240 m/s, altering wave deficit by up to 15.4% from Chapman-Jouguet.</t>
+          <t>conducting numerical experiments of supersonic combustion in a DCR engine using CEMA and Damkohler number analysis, demonstrating that thermal choking establishes a thermal throat in the constant-area section and elevates pressure, temperature, and nozzle exit Mach number.</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>The rotating detonation engine (RDE) with a hollow annular channel is investigated using 3D LES with detailed H2-O2 kinetics. Slot aspect ratio variations of 1:4 to 4:1 produce wave speeds ranging from 1820 to 2240 m/s, with wave deficits from 8.2% to 15.4% relative to the idealized Chapman-Jouguet value. Inlet geometry controls the freshly mixed reactant layer thickness ahead of the detonation wave, directly setting wave speed and heat release peak.</t>
+          <t>This work presents a numerical investigation of supersonic combustion dynamics and flow evolution in a dual-combustion ramjet (DCR) engine. Two series of parametric numerical experiments were conducted for the DCR combustor configuration by varying the length of the constant-area section [Formula: see text] and the divergence angle [Formula: see text] of the expansion section. The operating conditions were selected to mimic realistic flight scenarios. Two distinct combustion modes were identified, based on the occurrence of thermal choking. To analyze the combustion characteristics of these modes, chemical explosive mode analysis was performed, along with an evaluation of the Damköhler number. In the thermally choked combustion mode, both pressure and temperature were significantly elevated compared to the supersonic shear-layer combustion mode. This increase is attributed to the coupling between pressure and heat release, which enhances combustion efficiency. A thermal throat forms at the end of the constant-area section, while the divergent section functions as a supersonic nozzle. The exit Mach number in thermally choked cases is higher than its counterpart in supersonic shea...</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>Supercritical cryogenic LOX/GH2 combustion in a single-element shear-coaxial injector</t>
+          <t>Resonant phenomena in detonative tangential combustion instability in a rocket combustor</t>
         </is>
       </c>
       <c r="T3" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.B38219", "https://doi.org/10.2514/1.B38219")</f>
+        <f>HYPERLINK("https://doi.org/10.1063/5.0268442", "https://doi.org/10.1063/5.0268442")</f>
         <v/>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>conducting LES with MBWR real-fluid EOS in a LOX/GH2 shear-coaxial injector at 6-12 MPa, demonstrating that transcritical injection eliminates surface tension, produces high-density oxygen fingers in hydrogen coflow, and increases flame standoff length by 38% with rising chamber pressure.</t>
+          <t>applying STFT, DMD, and POD spectral decomposition to detonative tangential combustion instability in a rocket combustor, demonstrating that limit-cycle instabilities originate from thermofluidic wave resonance rather than pure acoustic natural frequencies and exhibit characteristic frequency-shifting harmonics.</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>Supercritical cryogenic LOX/GH2 combustion in a shear-coaxial injector at 6-12 MPa is investigated using LES with MBWR real-fluid EOS. LES reveals that above the critical point, continuous fluid mixing eliminates surface tension and produces high-density LOX fingers that stretch into hydrogen coflow. Flame standoff length increases by 38% as chamber pressure rises from 6 to 12 MPa.</t>
+          <t>In addition to investigating the flow field of detonative tangential combustion instability [Sung, B.-K., Kasahara, J., and Choi, J.-Y., Combust. Flame 275 114092 (2025)], spectral analysis was performed using Short-time Fourier Transform (STFT), Dynamic Mode Decomposition (DMD), and Proper Orthogonal Decomposition (POD) to gain a deeper understanding of the instability modes. By comparing the limit-cycle frequencies with the acoustic natural frequencies, it was confirmed that the detonative tangential combustion instability cannot be analyzed solely based on natural frequencies, as it corresponds to thermofluidic phenomena rather than thermoacoustic instability. The STFT provided time-dependent frequencies and revealed a frequency shift phenomenon during instability mode transitions. Using DMD, the corresponding dominant mode shapes were identified. The POD analysis corroborated the DMD results, and by examining the eigenvectors of the energetic POD modes, the mode undergoing the frequency shift was identified. During limit cycle operation, frequency harmonics emerged as the frequencies of each mode became integer multiples of the most energetic mode, further indicating that de...</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>1. Rotating detonation engine hollow annular channel: Effects of inlet geometry on wave dynamics (Combustion and Flame, 2022) | 2. Supercritical cryogenic LOX/GH2 combustion in a single-element shear-coaxial injector (JPP, 2021)</t>
+          <t>1. Supersonic Combustion and Flow Evolution in Dual-Combustion Ramjet Engine (Journal of Propulsion and Power, 2025) | 2. Resonant phenomena in detonative tangential combustion instability in a rocket combustor (Physics of Fluids, 2025)</t>
         </is>
       </c>
       <c r="X3" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2021.111763 | https://doi.org/10.2514/1.B38219", "https://doi.org/10.1016/j.combustflame.2021.111763 | https://doi.org/10.2514/1.B38219")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.b40184 | https://doi.org/10.1063/5.0268442", "https://doi.org/10.2514/1.b40184 | https://doi.org/10.1063/5.0268442")</f>
         <v/>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>performing 3D LES with finite-rate H2-O2 kinetics in a hollow annular RDE, demonstrating that inlet slot aspect ratio controls reactant layer thickness and shifts rotating detonation wave speed between 1820 and 2240 m/s, altering wave deficit by up to 15.4% from Chapman-Jouguet.</t>
+          <t>conducting numerical experiments of supersonic combustion in a DCR engine using CEMA and Damkohler number analysis, demonstrating that thermal choking establishes a thermal throat in the constant-area section and elevates pressure, temperature, and nozzle exit Mach number.</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
@@ -1203,64 +1203,64 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Simultaneous high-speed 3D laser diagnostics -- tomographic PIV, dual-pump CARS thermometry, and kHz OH-PLIF -- to map turbulence-chemistry interactions, flame kernel growth, and thermoacoustic feedback in swirl-stabilized gas-turbine combustors.</t>
+          <t>High-speed laser diagnostics for high-pressure turbulent reacting flows, ducted fuel injection (DFI) soot mitigation, and lean blowoff stability mechanisms in lean premixed prevaporized (LPP) supersonic transport combustors.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Dual-pump CARS (N2/O2 thermometry), High-speed stereoscopic PIV, kHz OH-PLIF, Tomographic PIV, High-speed Schlieren</t>
+          <t>Filtered Rayleigh Scattering (FRS), High-speed PIV/PLIF, Ducted Fuel Injection (DFI), Optical high-pressure combustor rigs (700 K, 9 bar), Laser extinction soot diagnostics</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Experimental investigation of turbulence-chemistry interaction in a gas turbine model combustor using simultaneous high-speed CARS and PIV</t>
+          <t>Impact of pilot injections on ducted fuel injection performance</t>
         </is>
       </c>
       <c r="P4" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2023.112754", "https://doi.org/10.1016/j.combustflame.2023.112754")</f>
+        <f>HYPERLINK("https://doi.org/10.1177/14680874261426780", "https://doi.org/10.1177/14680874261426780")</f>
         <v/>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>deploying simultaneous 5 kHz dual-pump CARS and stereo-PIV in a swirl combustor, demonstrating that local extinction events co-locate with strain-rate regions where Ka &gt; 50 and that re-ignition traces preferentially the trailing edges of high-scalar-dissipation tubes.</t>
+          <t>investigating the coupling of ducted fuel injection (DFI) with pilot injections in high-pressure diesel combustion, demonstrating that DFI reduces flame spatially integrated natural luminosity (SINL) by 30-70% and pilot injection mitigates peak SINL by a further 16%.</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>Simultaneous dual-pump CARS thermometry and stereoscopic PIV measurements at 5 kHz are applied to characterize turbulence-chemistry interaction in a gas turbine model combustor under atmospheric and elevated pressure conditions. Results demonstrate strongly non-equilibrium scalar mixing in the flame brush: local extinction events co-locate with high-strain-rate regions where turbulent Karlovitz numbers exceed Ka = 50, while re-ignition preferentially occurs at the trailing edges of high-scalar-dissipation tubes, indicating that distributed reaction zones operate transiently in thin-flame mode.</t>
+          <t>This experimental and numerical study evaluates how ducted fuel injection (DFI) and pilot injections interact to impact soot formation and the premixed heat release pressure spike in diesel combustion. Experiments showed that pilot injections reduced the premixed heat release spike of a free spray by approximately 70%, while DFI configurations only experienced a decrease of approximately 25%. Similarly, pilot injections reduced the initial lift-off length (LOL) of the main injection of a free-spray by approximately 30%, while DFI’s initial LOL had little to no change when pilot injections were utilized. Regardless of whether a standalone-main or pilot-main strategy was used, DFI was able to reduce the spatially integrated natural luminosity (SINL) of the flame relative to a free spray, indicating a likely reduction in soot formation. Both duct configurations studied produced steady SINL signals which were approximately 30% and 70% of the free-spray’s, respectively. For DFI, pilot injections further reduced the peak SINL compared to a standalone main by approximately 16%. The decrease in peak SINL correlated with increased spray head penetration rates. The numerical study reveale...</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>Simultaneous high-speed OH-PLIF and stereoscopic PIV of turbulent premixed flames at elevated pressure</t>
+          <t>Lean Blowoff Limits and Emissions Measurements in a Lean Premixed Prevaporized Combustor with Variable Reactant Inhomogeneity</t>
         </is>
       </c>
       <c r="T4" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.proci.2020.06.149", "https://doi.org/10.1016/j.proci.2020.06.149")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0384", "https://doi.org/10.2514/6.2026-0384")</f>
         <v/>
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>conducting simultaneous kHz OH-PLIF and SPIV across 1-5 atm in a swirl combustor, demonstrating that elevated pressure compresses the reaction layer and increases mean tangential strain rates by 3.2x while transitioning flame-wrinkling from Ka-dominated to curvature-dominated kinematic regimes.</t>
+          <t>characterizing lean blowoff (LBO) limits and emissions in an LPP combustor operating at 700 K and 9 bar on Jet A and SAF, demonstrating that moderate prevaporization and premixing are required to anchor main flames and curb NOx emission spikes.</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>Simultaneous kHz-rate OH-PLIF and SPIV measurements were performed in turbulent premixed swirling flames at elevated pressures up to 5 atm. Elevated pressure compresses the reaction layer, increases Damkohler number, and transitions flame-wrinkling dynamics from Ka-dominated to curvature-dominated modes. Strain-rate statistics at 5 atm show that global mean tangential strain rates increase by a factor of 3.2 relative to atmospheric cases.</t>
+          <t>Lean premixed prevaporized (LPP) combustor designs and sustainable aviation fuels (SAF) show great promise for the development of next-generation low-emission civil supersonic transport (CST) aircraft engines. In this work, exhaust emissions sampling and optical diagnostic measurements were conducted in an LPP model combustor with variable reactant inhomogeneity. The LPP combustor features a novel premixer design, which facilitates control of the level of fuel vaporization and fuel-air mixedness entering the combustor. Measurements of lean blowoff (LBO) limits and gaseous emissions trends were obtained through the optically accessible combustor liner and custom exhaust sampling probe. The combustor was operated at elevated temperature (700 K) and pressure (9 bar) conditions to simulate the combustor inlet conditions of CST aircraft engines. A conventional Jet A fuel was used as the baseline fuel, to which a SAF was compared. Results show that a moderate level of prevaporization and premixing was sufficient to properly stabilize the premixed main flames. With reduced prevaporization and premixing, the main flames did not properly stabilize and NOx emissions were increased. With i...</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>1. Turbulence-chemistry interaction in a GT model combustor via simultaneous high-speed CARS and PIV (Combustion and Flame, 2023) | 2. Simultaneous high-speed OH-PLIF and stereo-PIV of turbulent premixed flames at elevated pressure (Proc. Combustion Institute, 2021)</t>
+          <t>1. Impact of pilot injections on ducted fuel injection performance (International Journal of Engine Research, 2026) | 2. Lean Blowoff Limits and Emissions Measurements in a Lean Premixed Prevaporized Combustor with Variable Reactant Inhomogeneity (2026)</t>
         </is>
       </c>
       <c r="X4" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2023.112754 | https://doi.org/10.1016/j.proci.2020.06.149", "https://doi.org/10.1016/j.combustflame.2023.112754 | https://doi.org/10.1016/j.proci.2020.06.149")</f>
+        <f>HYPERLINK("https://doi.org/10.1177/14680874261426780 | https://doi.org/10.2514/6.2026-0384", "https://doi.org/10.1177/14680874261426780 | https://doi.org/10.2514/6.2026-0384")</f>
         <v/>
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>deploying simultaneous 5 kHz dual-pump CARS and stereo-PIV in a swirl combustor, demonstrating that local extinction events co-locate with strain-rate regions where Ka &gt; 50 and that re-ignition traces preferentially the trailing edges of high-scalar-dissipation tubes.</t>
+          <t>investigating the coupling of ducted fuel injection (DFI) with pilot injections in high-pressure diesel combustion, demonstrating that DFI reduces flame spatially integrated natural luminosity (SINL) by 30-70% and pilot injection mitigates peak SINL by a further 16%.</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr">
@@ -1403,64 +1403,64 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Quantitative laser diagnostics for high-enthalpy reacting flows -- PLIF-based scalar measurements, dual-pump CARS thermometry, and two-photon LIF for atomic species in high-pressure combustion, shock tunnels, and detonation chambers.</t>
+          <t>Advanced planar laser-induced fluorescence (PLIF) diagnostics for elevated-pressure reacting flows, lean blowoff proximity sensing, and multi-species optical imaging in swirl-stabilized spray flames.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Planar Laser-Induced Fluorescence (PLIF), Dual-pump CARS, Two-photon atomic LIF, High-speed intensified CCD, Shock tube/detonation chamber diagnostics</t>
+          <t>Single-laser CH/OH/fuel PLIF, Longpass intra-vibrational band optical filtering, High-pressure combustor rigs (9 bar), Lean blowout acoustic/optical sensing</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Quantitative PLIF imaging of OH* chemiluminescence in detonation-driven flows</t>
+          <t>Lean Blowoff Limits and Emissions Measurements in a Lean Premixed Prevaporized Combustor with Variable Reactant Inhomogeneity</t>
         </is>
       </c>
       <c r="P5" s="3">
-        <f>HYPERLINK("https://doi.org/10.1088/1361-6501/ac4b21", "https://doi.org/10.1088/1361-6501/ac4b21")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0384", "https://doi.org/10.2514/6.2026-0384")</f>
         <v/>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>applying quantitative OH* PLIF with dual-pump CARS quenching correction behind H2-air detonation fronts, demonstrating that post-detonation OH* overshoots equilibrium concentration by 2.3x due to ZND induction-zone kinetic excess, fully resolved at 200 um spatial resolution.</t>
+          <t>evaluating lean blowoff limits and emissions in an LPP combustor operating at 700 K and 9 bar under variable reactant inhomogeneity, demonstrating that prevaporization uniformity dictates flame stabilization and prevents severe NOx emission surges.</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>A quantitative PLIF diagnostic for excited-state OH* is developed and applied to detonation-driven supersonic combustion flows. The diagnostic accounts for collisional quenching corrections using simultaneous dual-pump CARS measurements. Applied to a H2-air detonation tube, OH* PLIF images resolve the thin reaction zone behind the detonation front with 200 um spatial resolution. OH* signal peaks at 2.3x the equilibrium post-detonation value, indicating strong kinetic overshoot driven by ZND induction zone chemistry.</t>
+          <t>Lean premixed prevaporized (LPP) combustor designs and sustainable aviation fuels (SAF) show great promise for the development of next-generation low-emission civil supersonic transport (CST) aircraft engines. In this work, exhaust emissions sampling and optical diagnostic measurements were conducted in an LPP model combustor with variable reactant inhomogeneity. The LPP combustor features a novel premixer design, which facilitates control of the level of fuel vaporization and fuel-air mixedness entering the combustor. Measurements of lean blowoff (LBO) limits and gaseous emissions trends were obtained through the optically accessible combustor liner and custom exhaust sampling probe. The combustor was operated at elevated temperature (700 K) and pressure (9 bar) conditions to simulate the combustor inlet conditions of CST aircraft engines. A conventional Jet A fuel was used as the baseline fuel, to which a SAF was compared. Results show that a moderate level of prevaporization and premixing was sufficient to properly stabilize the premixed main flames. With reduced prevaporization and premixing, the main flames did not properly stabilize and NOx emissions were increased. With i...</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>Two-temperature analysis of non-equilibrium N2 vibrational excitation in hypersonic arcjet flows</t>
+          <t>Single-laser CH, OH and fuel PLIF in a pressurized swirl-stabilized spray flame</t>
         </is>
       </c>
       <c r="T5" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.T6072", "https://doi.org/10.2514/1.T6072")</f>
+        <f>HYPERLINK("https://doi.org/10.1016/j.proci.2026.106104", "https://doi.org/10.1016/j.proci.2026.106104")</f>
         <v/>
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>measuring two-photon LIF vibrational temperatures across a Mach 5-7 arcjet freestream, demonstrating N2 vibrational temperatures exceed translational by 1800-2400 K and Park finite-rate model under-predicts vibrational relaxation in the expansion fan by 28%.</t>
+          <t>demonstrating single-laser simultaneous CH, OH, and fuel PLIF in a pressurized swirl-stabilized spray flame at 310.7 nm, revealing that pressure-induced collisional broadening allows clean separation of thin CH reaction zones from dense liquid spray droplet fluorescence.</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>Non-equilibrium vibrational excitation of N2 in a high-enthalpy arcjet flow simulating Mars entry conditions is investigated using two-photon LIF and optical emission spectroscopy. Measured vibrational temperatures exceed translational temperatures by 1800-2400 K across Mach 5-7 test conditions. Agreement with LAURA CFD predictions using Park rate model is within 12% in the freestream but degrades to 28% in the expansion fan region.</t>
+          <t>This paper explores the use of planar laser-induced fluorescence (PLIF) with excitation wavelengths in the R-branch of the CH C 2 Σ + − X 2 Π ( 0,0 ) in a liquid-fueled combustor at elevated pressures. Following the atmospheric pressure work of Hammack et al. Appl. Phys. B 124:34 (2018), longpass intra-vibrational band filtering was used to isolate CH PLIF, OH PLIF, and fuel signals from the laser scattering. CH PLIF images were obtained by targeting CH R-branch transitions at 310.69 nm and 311.18 nm. Interference from fuel fluorescence was mitigated through the use of a low-aromatic content synthetic aviation fuel, though it was still significant where liquid was present. Nevertheless, the CH layers in the reaction zone were distinguishable from the droplet signal even in the dense spray near the fuel injector. OH PLIF images could be obtained without CH interference using the same setup, but targeting the OH Q-branch transitions of the A − X ( 0,0 ) band at 310.75 nm. Furthermore, due to pressure-induced collisional broadening, simultaneous CH and OH PLIF could be imaged on a single frame when the laser wavelength was tuned in the vicinity of either CH R-branch transition. The...</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>1. Quantitative PLIF imaging of OH* chemiluminescence in detonation-driven flows (MST, 2022) | 2. Two-temperature analysis of non-equilibrium N2 in hypersonic arcjet flows (JTHT, 2021)</t>
+          <t>1. Lean Blowoff Limits and Emissions Measurements in a Lean Premixed Prevaporized Combustor with Variable Reactant Inhomogeneity (2026) | 2. Single-laser CH, OH and fuel PLIF in a pressurized swirl-stabilized spray flame (Proceedings of the Combustion Institute, 2026)</t>
         </is>
       </c>
       <c r="X5" s="3">
-        <f>HYPERLINK("https://doi.org/10.1088/1361-6501/ac4b21 | https://doi.org/10.2514/1.T6072", "https://doi.org/10.1088/1361-6501/ac4b21 | https://doi.org/10.2514/1.T6072")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0384 | https://doi.org/10.1016/j.proci.2026.106104", "https://doi.org/10.2514/6.2026-0384 | https://doi.org/10.1016/j.proci.2026.106104")</f>
         <v/>
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>applying quantitative OH* PLIF with dual-pump CARS quenching correction behind H2-air detonation fronts, demonstrating that post-detonation OH* overshoots equilibrium concentration by 2.3x due to ZND induction-zone kinetic excess, fully resolved at 200 um spatial resolution.</t>
+          <t>evaluating lean blowoff limits and emissions in an LPP combustor operating at 700 K and 9 bar under variable reactant inhomogeneity, demonstrating that prevaporization uniformity dictates flame stabilization and prevents severe NOx emission surges.</t>
         </is>
       </c>
       <c r="Z5" s="2" t="inlineStr">
@@ -1603,64 +1603,64 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>High-fidelity RANS/hybrid RANS-LES aeromechanics simulation of helicopter rotors and wind turbines -- capturing dynamic stall vortex shedding, rotor-wake interaction, and blade-vortex interaction noise to reduce vibration and acoustic emissions in next-generation rotorcraft.</t>
+          <t>Aeroacoustics DNS of high-amplitude acoustic transmission and inverse airfoil design for roughness-tolerant low-drag wind and hydrokinetic turbine blades.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Hybrid RANS-LES (DDES), Overset Chimera grids, Dynamic mesh motion, CAMRAD II structural coupling, Gradient boosted trees (dynamic stall onset ML)</t>
+          <t>Direct Numerical Simulation (DNS) aeroacoustics, Impedance tube testing (120-150 dB), Inverse airfoil aerodynamic design, Blade Element Momentum (BEM) turbine codes</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Dynamic Stall Onset Prediction and Modeling Using Machine Learning on CFD-Generated Datasets</t>
+          <t>Transmission of high-amplitude sound through leakages of ill-fitting earplugs</t>
         </is>
       </c>
       <c r="P6" s="3">
-        <f>HYPERLINK("https://doi.org/10.4050/JAHS.68.032001", "https://doi.org/10.4050/JAHS.68.032001")</f>
+        <f>HYPERLINK("https://doi.org/10.1177/1475472x261473636", "https://doi.org/10.1177/1475472x261473636")</f>
         <v/>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>training gradient-boosted classifiers on 4.1M URANS time steps across 15,000 airfoil conditions, demonstrating 94.2% accuracy in predicting dynamic stall onset 3 convective time units in advance and reducing full-rotor vibration estimation error from 31% to 9%.</t>
+          <t>combining impedance-tube experiments with DNS of high-amplitude acoustic transmission (120-150 dB) across 1-5 kHz, demonstrating that ill-fitting earplug leakages reduce transmission loss by ~18 dB at 120 dB incident SPL.</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>Machine learning models trained on 4.1 million time steps from URANS simulations across 15,000 operating conditions achieve 94.2% accuracy in predicting dynamic stall onset 3 convective time units in advance. The ML-based predictor integrated into a blade element momentum model reduces dynamic stall-induced vibration estimation error from 31% to 9% relative to pure BEMT.</t>
+          <t>Exposure to high sound pressure levels (SPL) is a leading cause of noiseinduced hearing loss, and earplugs are a primary means of protection. The effectiveness of earplug protection depends on the seal formed in the ear canal. An ill-fitting earplug leaves air gaps that leak sound and degrade attenuation. The acoustics of these leak paths and their dissipation mechanisms under high-amplitude sound remain poorly characterized. This study quantifies sound transmission through modeled earplug leakage with rigid-wall idealization and identifies the governing dissipation mechanisms by combining impedance-tube experiments and direct numerical simulation (DNS). The methods were first verified against stand-alone slit resonators and orifices, for which extensive published data are available, and then used to measure the transmission loss (TL) and acoustic power absorption coefficient of modeled earplug–canal configurations over 1–5 kHz at overall incident SPLs of 120–150 dB. Leakage from an ill-fitting silicone rubber earplug reduced its TL by approximately 18 dB relative to a sealed configuration at an overall incident sound pressure levels (OISPL) of 120 dB, and the leakage-path TL in...</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>Computational Investigation of Rotor-Fuselage Interactional Aerodynamics Using Hybrid RANS-LES</t>
+          <t>Design and Use of Roughness-Tolerant Low Drag Airfoils for Wind Turbine and Hydrokinetic Turbine Applications</t>
         </is>
       </c>
       <c r="T6" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.J060183", "https://doi.org/10.2514/1.J060183")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0480", "https://doi.org/10.2514/6.2026-0480")</f>
         <v/>
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>simulating rotor-fuselage interactional aerodynamics via DDES on overset grids at advance ratio mu = 0.15, demonstrating that recirculation below the hub increases rotor torque by 4.7% and produces wake-fuselage surface pressure fluctuations of 0.08 Cp matching experimental data.</t>
+          <t>applying inverse design to develop roughness-tolerant airfoils with laminar drag buckets across wide lift coefficients, demonstrating preserved profile efficiency under surface dirt and icing degradation in wind and tidal turbines.</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>The interactional aerodynamics between a helicopter main rotor and fuselage is investigated using DDES on overset grids. Rotor-fuselage interaction produces a recirculation region below the hub that increases rotor torque requirement by 4.7%. Unsteady wake-fuselage impingement creates surface pressure fluctuations of 0.08 Cp, consistent with Georgia Tech Aeroflite wind tunnel measurements.</t>
+          <t>Wind turbines and hydrokinetic turbines are designed to use laminar airfoils that provide maximum power at the rated speed. During day-to-day operations, the blade surface may be degraded due to accumulation of dirt and icing on the pressure side, in addition to development of scratches or other surface imperfections. As a result, the profile power losses would increase, reducing the available power over a broad range of operating conditions. In this work, an inverse design approach has been employed to generate roughness tolerant airfoils that exhibit a laminar drag bucket for a broad range of lift coefficients. Two-dimensional drag polars are presented for smooth and rough airfoils and compared to NACA airfoils of comparable thickness. A limited number of three-dimensional studies based on combined blade element-momentum theory are also presented for several wind and tidal turbines for a broad range of rated power conditions.</t>
         </is>
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>1. Dynamic Stall Onset Prediction Using Machine Learning on CFD Datasets (JAHS, 2023) | 2. Computational Investigation of Rotor-Fuselage Interactional Aerodynamics Using Hybrid RANS-LES (AIAA J., 2021)</t>
+          <t>1. Transmission of high-amplitude sound through leakages of ill-fitting earplugs (International Journal of Aeroacoustics, 2026) | 2. Design and Use of Roughness-Tolerant Low Drag Airfoils for Wind Turbine and Hydrokinetic Turbine Applications (2026)</t>
         </is>
       </c>
       <c r="X6" s="3">
-        <f>HYPERLINK("https://doi.org/10.4050/JAHS.68.032001 | https://doi.org/10.2514/1.J060183", "https://doi.org/10.4050/JAHS.68.032001 | https://doi.org/10.2514/1.J060183")</f>
+        <f>HYPERLINK("https://doi.org/10.1177/1475472x261473636 | https://doi.org/10.2514/6.2026-0480", "https://doi.org/10.1177/1475472x261473636 | https://doi.org/10.2514/6.2026-0480")</f>
         <v/>
       </c>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>training gradient-boosted classifiers on 4.1M URANS time steps across 15,000 airfoil conditions, demonstrating 94.2% accuracy in predicting dynamic stall onset 3 convective time units in advance and reducing full-rotor vibration estimation error from 31% to 9%.</t>
+          <t>combining impedance-tube experiments with DNS of high-amplitude acoustic transmission (120-150 dB) across 1-5 kHz, demonstrating that ill-fitting earplug leakages reduce transmission loss by ~18 dB at 120 dB incident SPL.</t>
         </is>
       </c>
       <c r="Z6" s="2" t="inlineStr">
@@ -1803,64 +1803,64 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Hall-effect thruster plume physics, near-anode ionization instabilities, and plasma-neutral coupling in electric propulsion -- combining laser-induced fluorescence velocimetry, Langmuir probe arrays, and particle-in-cell simulations to push CubeSat and deep-space thruster efficiency boundaries.</t>
+          <t>Hall-effect thruster plasma physics, heaterless hollow cathode operation on alternative propellants (krypton/argon), and laser Thomson scattering electron dynamics in magnetically shielded thrusters.</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Laser-Induced Fluorescence (LIF) velocimetry (Xe II lines), Langmuir and Faraday probes, Retarding Potential Analyzer (RPA), E×B probe, Particle-in-Cell (PIC) simulations</t>
+          <t>Laser Thomson Scattering, Steady-state I-V cathode characterization, Magnetically shielded Hall thruster testing (H9 9 kW), Vacuum Test Facilities (VTF-2)</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Azimuthal Ion Velocity Measurements in a Hall Thruster via Laser-Induced Fluorescence</t>
+          <t>Characterization of a heaterless 60 A hollow cathode on krypton and argon</t>
         </is>
       </c>
       <c r="P7" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.B38688", "https://doi.org/10.2514/1.B38688")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s44205-026-00221-w", "https://doi.org/10.1007/s44205-026-00221-w")</f>
         <v/>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>measuring azimuthal Xe II ion velocities via dual-geometry LIF in a Hall thruster near-field plume, demonstrating that azimuthal swirl reaches 2.1-3.8 km/s (11-19% of exit velocity) and correlates with 15-20 kHz breathing mode oscillations that reduce effective specific impulse.</t>
+          <t>characterizing a 60 A heaterless hollow cathode on krypton and argon in the 9 kW H9 thruster, demonstrating that magnetic fields systematically increase steady-state discharge voltage by up to +159% (+67.5 V) on argon at fixed current rather than reducing it.</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>Azimuthal ion velocity measurements in the near-field plume of a Hall-effect thruster are reported using LIF velocimetry of Xe II lines. Peak swirl velocities of 2.1-3.8 km/s correspond to 11-19% of total ion exit velocity. These azimuthal components correlate with low-frequency breathing mode oscillations at 15-20 kHz and indicate non-trivial angular momentum deposition that degrades effective thruster specific impulse.</t>
+          <t>Abstract We present a steady-state current-voltage (IV) characterization of a heaterless version of the 9 kW-class H9 Hall thruster cathode. This work was conducted at Georgia Tech’s High-Power Electric Propulsion Laboratory (HPEPL) at operational background pressures of 0.22–0.70 µTorr on krypton and 0.11–0.24 µTorr on argon, with a base pressure of 9.1 × 10 − 8 Torr. The characterization mapped steady-state voltage behavior from 5 to 45 A of discharge current on krypton and 5 to 30 A on argon (with paired magnetized and unmagnetized data over 5 to 35 A on krypton and 5 to 20 A on argon), in both magnetized and unmagnetized configurations. The magnetized configuration produced a higher discharge voltage than the unmagnetized configuration at every paired (current, flow) operating point on both propellants. On krypton, the magnetized-unmagnetized voltage gap ranged from near zero at the highest cathode flow and lowest current to + 39.6 V (+ 148%) at 30 A and 12.39 sccm. On argon, the gap ranged from + 6.0 V at 15 A and 12.39 sccm to + 67.5 V (+ 159%) at 20 A and 15.89 sccm. In both cases, the gap widened with discharge current and narrowed with cathode flow. These results verify reproducible ignition at every tested flow rate, confirm uninterrupted steady-state heaterless operation on krypton and argon, and quantify how the applied magnetic field shifts the steady-state operating point at fixed discharge current. The key finding is that the applied magnetic field increases the steady-state discharge voltage at fixed current rather than reducing it, and the effect is systematically larger on argon than on krypton at matched operating conditions.</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>Near-Field Plume Characterization of a 200-W Hall Thruster via Electrostatic Probes</t>
+          <t>Effect of body bias on near-field electron behavior in a magnetically shielded Hall thruster</t>
         </is>
       </c>
       <c r="T7" s="3">
-        <f>HYPERLINK("https://doi.org/10.1007/s44205-023-00045-z", "https://doi.org/10.1007/s44205-023-00045-z")</f>
+        <f>HYPERLINK("https://doi.org/10.1063/5.0340395", "https://doi.org/10.1063/5.0340395")</f>
         <v/>
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>deploying 2D electrostatic probe arrays in a 200-W Hall thruster near-field plume, demonstrating that bimodal IEDFs at 5 cm downstream directly evidence charge-exchange collisions that broaden plume divergence by 6.8 degrees beyond the accelerated-ion beam.</t>
+          <t>deploying spatially resolved laser Thomson scattering in the near-field of the 9 kW H9 Hall thruster at 40 A, demonstrating that +2 V body bias inverts electron density topology between the cathode centerline (3.4e19 m^-3) and channel centerline (9.0e17 m^-3).</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>A comprehensive electrostatic probe characterization of the near-field plume of a 200-W Hall thruster is reported. The IEDF at 5 cm downstream reveals a bimodal structure with a cold (&lt;10 eV) charge-exchange peak and a hot (120-180 eV) direct-acceleration peak, providing direct evidence for near-field charge exchange collisions that broaden plume divergence by 6.8 degrees.</t>
+          <t>This work investigates the influence of thruster body bias on near-field electron behavior in a magnetically shielded Hall effect thruster (HET) through spatially resolved laser Thomson scattering diagnostics. Experiments were conducted on the 9 kW class H9 magnetically shielded HET operating at 40 A discharge current and 150 V discharge voltage on krypton propellant in the Georgia Tech Vacuum Test Facility 2. Three electrical configurations were examined: floating (body electrically isolated), cathode-tied (body at cathode potential, approximately −10.3 V relative to facility ground), and +2 V bias (body biased +2 V relative to ground). Spatially resolved measurements of electron density, electron temperature, and radial electron bulk velocity were obtained at up to 23 locations (a 15-point radial grid and up to eight axial stations along the cathode centerline) spanning the cathode near-field from the cathode centerline to the discharge channel centerline. A configuration-dependent spatial density inversion reveals distinct circuit topologies: at z/r0 = 0.029, cathode-tied elevates ne at the cathode centerline (4.4 × 1019 m−3) while exhibiting the lowest channel-centerline density (6.6 × 1017 m−3), whereas the +2 V configuration shows the opposite pattern (3.4 × 1019 and 9.0 × 1017 m−3, respectively). The +2 V configuration exhibits the lowest Te at the inner front pole cover, consistent with magnetization-limited, energy-selective electron collection. Electron pressure does not serve as a reliable proxy for electrostatic potential in this near-field region due to unmeasured anomalous transport terms.</t>
         </is>
       </c>
       <c r="W7" s="2" t="inlineStr">
         <is>
-          <t>1. Azimuthal Ion Velocity Measurements in a Hall Thruster via Laser-Induced Fluorescence (JPP, 2022) | 2. Near-Field Plume Characterization of a 200-W Hall Thruster via Electrostatic Probes (JEP, 2023)</t>
+          <t>1. Characterization of a heaterless 60 A hollow cathode on krypton and argon (Journal of Electric Propulsion, 2026) | 2. Effect of body bias on near-field electron behavior in a magnetically shielded Hall thruster (Journal of Applied Physics, 2026)</t>
         </is>
       </c>
       <c r="X7" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.B38688 | https://doi.org/10.1007/s44205-023-00045-z", "https://doi.org/10.2514/1.B38688 | https://doi.org/10.1007/s44205-023-00045-z")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s44205-026-00221-w | https://doi.org/10.1063/5.0340395", "https://doi.org/10.1007/s44205-026-00221-w | https://doi.org/10.1063/5.0340395")</f>
         <v/>
       </c>
       <c r="Y7" s="2" t="inlineStr">
         <is>
-          <t>measuring azimuthal Xe II ion velocities via dual-geometry LIF in a Hall thruster near-field plume, demonstrating that azimuthal swirl reaches 2.1-3.8 km/s (11-19% of exit velocity) and correlates with 15-20 kHz breathing mode oscillations that reduce effective specific impulse.</t>
+          <t>characterizing a 60 A heaterless hollow cathode on krypton and argon in the 9 kW H9 thruster, demonstrating that magnetic fields systematically increase steady-state discharge voltage by up to +159% (+67.5 V) on argon at fixed current rather than reducing it.</t>
         </is>
       </c>
       <c r="Z7" s="2" t="inlineStr">
@@ -1987,64 +1987,64 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>LES-driven combustion instability modeling, turbulent premixed flame propagation, and plasma-assisted ignition in gas-turbine and scramjet combustors — advancing high-fidelity reacting-flow simulation from laboratory-scale flames to full annular combustion chambers.</t>
+          <t>Large eddy simulations (LES) of turbulent combustion, hybrid transported-tabulated chemistry (HTTC), and soot aerosol dynamics in rich-burn quick-mix lean-burn (RQL) and rotating detonation combustors.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Large Eddy Simulation (LES) with LDK subgrid closure, PRISM tabulated chemistry, Spray Lagrangian tracking, DNS of premixed flame kernels</t>
+          <t>Large Eddy Simulation (LES), Hybrid Transported-Tabulated Chemistry (HTTC), Dynamic subgrid closures, PAH-based soot modeling, Partially stirred reactor (PaSR)</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Subgrid combustion modeling for large eddy simulation of spray combustion in turbulent swirling flows</t>
+          <t>Application of Hybrid Transported-Tabulated Chemistry for Efficient Large-Eddy Simulation of Turbulent Combustion</t>
         </is>
       </c>
       <c r="P8" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2021.111634", "https://doi.org/10.1016/j.combustflame.2021.111634")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s10494-026-00794-4", "https://doi.org/10.1007/s10494-026-00794-4")</f>
         <v/>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>coupling Lagrangian spray dynamics with LES dynamic subgrid combustion in a bluff-body swirl combustor, demonstrating that droplet evaporation controls inner-recirculation-zone flame anchoring and produces unsteady heat-release fluctuations at Strouhal numbers consistent with observed thermoacoustic instabilities.</t>
+          <t>implementing a hybrid transported-tabulated chemistry (HTTC) strategy in LES of turbulent combustion with 29 species and 141 steps, demonstrating up to 11-fold computational speedup while maintaining high fidelity in predicting extinction and re-ignition dynamics.</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>A subgrid combustion model for large eddy simulation of spray combustion in turbulent swirling flows is developed and validated. The model is based on the localized dynamic K-equation (LDK) subgrid kinetic energy closure combined with a progress variable approach for turbulent premixed combustion. Two-phase spray effects are modeled using a Lagrangian particle tracking approach coupled to the LES gas-phase solver. The combined model is applied to a bluff-body stabilized swirl combustor and validated against experimental measurements of velocity, temperature, and species concentrations. Simulations reveal that liquid fuel droplet evaporation and transport profoundly alter local flame structure and stabilization mechanisms, particularly near the inner recirculation zone where unsteady flame-vortex interactions dominate heat release distribution.</t>
+          <t>Abstract The performance of a hybrid transported-tabulated chemistry (HTTC) strategy is evaluated for large-eddy simulations (LES) of turbulent combustion with detailed finite-rate kinetics. The computational cost of LES is reduced in the HTTC approach by segregating the species list into major and minor species, with the former transported and the latter tabulated. Apart from reducing the number of transported species, the HTTC approach and its variants decrease computational cost by enabling efficient computation of thermodynamics and transport properties and by relieving the stiffness of chemical source terms. The calculations can be up to 11 times faster with stiff kinetics (29 species, 141 steps), as the HTTC approach eliminates the need to integrate and transport the minor species, which typically have short chemical times. The original HTTC and other variants are assessed for their accuracy, efficiency, and robustness for LES by considering two temporally evolving challenging test cases: a freely propagating turbulent premixed flame in the thin reaction zone regime and a turbulent non-premixed jet flame exhibiting local extinction and re-ignition. Modifications to the original HTTC approach are considered and evaluated to account for the effect of subgrid-scale turbulence. Both a priori and a posteriori analyses are conducted to evaluate the accuracy of the HTTC approach. The turbulent premixed flame test shows noticeable yet small differences between the calculated and tabulated concentrations of minor species. This results in reasonable predictions of reaction rates and overall combustion process with HTTC. The difference between calculated and tabulated minor species concentrations is larger for the turbulent non-premixed flame case; however, the minor species concentrations are generally much lower for it, and therefore, extinction-re-ignition physics is still predicted well with HTTC.</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>Effects of multi-fuel blending on combustion characteristics of turbulent premixed swirling flames</t>
+          <t>Large-Eddy Simulations of Soot Formation and Dispersion in Rich-Burn Quick-Mix Lean-Burn (RQL) Spray Combustor</t>
         </is>
       </c>
       <c r="T8" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.proci.2022.07.034", "https://doi.org/10.1016/j.proci.2022.07.034")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2025-2484", "https://doi.org/10.2514/6.2025-2484")</f>
         <v/>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>performing LES with PRISM tabulated chemistry across methane-hydrogen blends (0-60% H2 by volume) in a swirl combustor, demonstrating that hydrogen enrichment amplifies local laminar flame speed by up to 48% and activates preferential diffusion wrinkling that reshapes thermoacoustic coupling frequencies.</t>
+          <t>performing LES with a Lagrangian spray and PAH soot kinetics in an RQL combustor at 6.8 atm, demonstrating that shifting global equivalence ratio from 0.12 to 0.2 markedly increases primary-zone soot volume fraction through localized flame-spray-soot interactions.</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t>The effects of fuel composition on turbulent premixed combustion characteristics of swirling flames are investigated using high-fidelity large eddy simulations (LES). Three fuel blends of methane and hydrogen (0%, 30%, and 60% H2 by volume) are studied in a gas turbine model combustor at atmospheric pressure. The LES employs a dynamic localized combustion model with detailed chemistry tabulation via PRISM. Increased hydrogen fraction accelerates local flame propagation by up to 48%, narrows the reaction zone, and triggers preferential diffusion-driven flame wrinkling at small scales, with direct consequence for NOx formation pathways.</t>
+          <t>The influence of varying fuel/air ratios on the primary zone soot formation characteristics of the liquid-fueled rich-quench-lean (RQL) combustor is investigated numerically. Large- eddy simulations (LES) of two global equivalence ratios (��) corresponding to 0.12 and 0.2 respectively are conducted at an overall pressure of 6.8 atm. The employed LES modeling framework includes Lagrangian treatment for liquid-fuel spray, finite-rate chemistry for gas- phase combustion, a polycyclic aromatic hydrocarbon (PAH)-based soot model, a partially stirred reactor model for turbulence-soot-chemistry interactions, and an optically thin radiation model. The soot and gas-phase chemistry modeling framework is verified against the experimental measurements from canonical premixed and non-premixed flames of gaseous ethylene fuels. The LES simulations of the RQL combustor qualitatively demonstrate the trend of increasing soot volume fractions (SVFs) under the two conditions investigated in this work. Further analysis of local flame-soot-spray interactions and soot source terms is reported to explain the observed differences.</t>
         </is>
       </c>
       <c r="W8" s="2" t="inlineStr">
         <is>
-          <t>1. Subgrid combustion modeling for LES of spray combustion in turbulent swirling flows (Combustion and Flame, 2022) | 2. Effects of multi-fuel blending on combustion of turbulent premixed swirling flames (Proc. Combustion Institute, 2023)</t>
+          <t>1. Application of Hybrid Transported-Tabulated Chemistry for Efficient Large-Eddy Simulation of Turbulent Combustion (Flow Turbulence and Combustion, 2026) | 2. Large-Eddy Simulations of Soot Formation and Dispersion in Rich-Burn Quick-Mix Lean-Burn (RQL) Spray Combustor (2025)</t>
         </is>
       </c>
       <c r="X8" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2021.111634 | https://doi.org/10.1016/j.proci.2022.07.034", "https://doi.org/10.1016/j.combustflame.2021.111634 | https://doi.org/10.1016/j.proci.2022.07.034")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s10494-026-00794-4 | https://doi.org/10.2514/6.2025-2484", "https://doi.org/10.1007/s10494-026-00794-4 | https://doi.org/10.2514/6.2025-2484")</f>
         <v/>
       </c>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>coupling Lagrangian spray dynamics with LES dynamic subgrid combustion in a bluff-body swirl combustor, demonstrating that droplet evaporation controls inner-recirculation-zone flame anchoring and produces unsteady heat-release fluctuations at Strouhal numbers consistent with observed thermoacoustic instabilities.</t>
+          <t>implementing a hybrid transported-tabulated chemistry (HTTC) strategy in LES of turbulent combustion with 29 species and 141 steps, demonstrating up to 11-fold computational speedup while maintaining high fidelity in predicting extinction and re-ignition dynamics.</t>
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr">
@@ -2183,64 +2183,64 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Thermoacoustic instability theory, turbulent flame linear response functions, and hydrodynamic wavemaker identification in low-NOx combustors -- building physics-based predictive frameworks for acoustic-flame coupling in next-generation gas turbines and hydrogen-fueled engines.</t>
+          <t>Combustion dynamics, swirl burner flame stability, low-carbon ammonia (NH3) rich-relaxation-quench-lean (RRQL) combustion systems, and turbulence sensitivity of NOx/CO emissions in hydrogen-methane blends.</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>High-speed OH-PLIF, Acoustic forcing rigs (transverse/longitudinal), Phase-locked PIV, Global flame transfer function measurement, Wavemaker stability analysis</t>
+          <t>High-speed OH*/NH2* chemiluminescence, Modular swirl burners, Gas-phase emissions sampling (NOx, N2O, NH3, CO), Turbulence-flame interaction rigs</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Flame Transfer Function Measurement of a Transversely Excited Swirling Flame</t>
+          <t>Toward the Development of an RRQL System—Part I: Swirl Pattern Effect on Exhaust Emissions and Chemiluminescence Distribution for NH3–Air Premixed Swirl Flames</t>
         </is>
       </c>
       <c r="P9" s="3">
-        <f>HYPERLINK("https://doi.org/10.1115/1.4053164", "https://doi.org/10.1115/1.4053164")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/1.4069796", "https://doi.org/10.1115/1.4069796")</f>
         <v/>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>measuring transverse flame transfer functions via phase-locked OH-PLIF in a swirl-stabilized combustor, demonstrating that transverse excitation produces peak gain at the swirler geometric resonance rather than the convective residence time, directly altering annular combustor thermoacoustic stability predictions.</t>
+          <t>investigating swirl geometry effects on flame morphology and emissions in rich premixed NH3-air flames for an RRQL system, demonstrating that compact flames minimize wall quenching and enable post-flame relaxation to suppress NOx and NH3 emissions.</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>This paper presents measurements of the flame transfer function (FTF) of a swirl-stabilized flame excited by transverse acoustic forcing. Using phase-locked OH-PLIF and acoustic pressure measurements, the FTF relating heat release rate fluctuations to transverse velocity perturbations is characterized over 100-600 Hz. Results show that the transverse FTF exhibits a substantially different gain-phase structure than the longitudinal FTF, with peak gain at frequencies near the swirler geometric resonance rather than the convective time scale.</t>
+          <t>Abstract Ammonia (NH3) is a carbon–free energy source and hydrogen carrier, but its fuel–bound nitrogen can lead to significant nitrogen oxides (NOx) emissions. Staged combustion strategies, such as rich–quench–lean, can achieve low NOx emissions. However, improper design may result in high NOx levels when operating with a rich head end without a sufficient post–flame relaxation time. Previous work has shown that a rich–relaxation–quench–lean (RRQL) configuration can minimize NOx emissions in the rich head end (Cole et al., 2024, “Rich Ammonia Flame Shapes and NO Relaxation: Facility Development and Characterization,” ASME Paper No. GT2024–122369). This study focuses on how different swirl geometries affect exhaust emissions and flame morphology in rich, premixed NH3–air flames, for the design of a rich relaxation head end of an RRQL combustor. Experiments were conducted using a modular swirl burner and measuring NOx, N2O, and NH3 emissions, and recording natural flame luminosity and NH2* and OH* chemiluminescence images. Swirler design affects emissions by influencing flame length (with shorter flames allowing for more postflame relaxation time) and flame–wall interactions (influencing NH3 and N2O emissions). A compact flame with minimal wall interactions allows for increased NOx relaxation, while minimal wall interactions prevent heat losses and instabilities, which minimize NH3 and N2O emissions at a richer equivalence ratio, potentially enhancing H2 production during the relaxation phase without increasing overall primary stage NOx emissions, thereby improving system efficiency. Detailed spatial evolution of NOx, N2O, and NH3 emissions further supports the RRQL as a promising combustor design for NH3 combustion, if the rich head end is designed properly.</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Hydrodynamic stability of reacting swirling jets</t>
+          <t>Measurements of CO and NOx Emissions From Premixed Turbulent Methane/Hydrogen Flames</t>
         </is>
       </c>
       <c r="T9" s="3">
-        <f>HYPERLINK("https://doi.org/10.1017/jfm.2021.433", "https://doi.org/10.1017/jfm.2021.433")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/1.4069625", "https://doi.org/10.1115/1.4069625")</f>
         <v/>
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>performing global wavemaker stability analysis of reacting swirling jets across varying equivalence ratios, demonstrating that combustion heat release simultaneously destabilizes the axisymmetric (m=0) centrifugal mode and suppresses the precessing vortex core (m=+-1) helical instability branch.</t>
+          <t>measuring the sensitivity of NO and CO emissions from turbulent premixed H2/CH4 flames across varying turbulence intensities, demonstrating that H2 enrichment sharply accelerates CO relaxation toward equilibrium while turbulence intensity yields negligible impact on NO at constant CO.</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
         <is>
-          <t>The hydrodynamic stability of reacting swirling jets is investigated using global stability analysis and wavemaker identification. Structural sensitivity analysis reveals a confined wavemaker region near the central recirculation zone boundary. Two competing instability branches are identified: an axisymmetric (m=0) branch driven by centrifugal destabilization and a helical (m=+-1) branch associated with the precessing vortex core (PVC). Increased heat release from combustion destabilizes the m=0 mode and simultaneously stabilizes the PVC branch.</t>
+          <t>Abstract This paper presents measurements of the sensitivity of NO and CO emissions from H2/CH4 combustion to variations in turbulence intensity. Existing studies of exhaust emissions either focus on laminar modeling and measurements or report device-level measurements from practical combustors. However, there are limited fundamental studies of emissions characteristics of turbulent systems, the focus of this study. Because of the strong stretch sensitivity of these mixtures, local temperatures/reaction rates along the turbulent front can differ markedly from mixture-averaged properties, and they are very sensitive to turbulence. Single-point emissions measurements are presented for turbulent premixed H2/CH4 flames from a contoured nozzle Bunsen burner with variable turbulence. Emissions are measured at varying residence times and incoming flow turbulence intensities. Data show the clear benefit of H2 blending on CO emissions, both due to the expected reduction in C atoms, but also due to faster relaxation of flame generated CO toward equilibrium. It also shows negligible impact of turbulence intensity on NO emissions at constant CO for CH4.</t>
         </is>
       </c>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>1. Flame Transfer Function of a Transversely Excited Swirling Flame (JEGTP, 2022) | 2. Hydrodynamic stability of reacting swirling jets (Journal of Fluid Mechanics, 2021)</t>
+          <t>1. Toward the Development of an RRQL System—Part I: Swirl Pattern Effect on Exhaust Emissions and Chemiluminescence Distribution for NH3–Air Premixed Swirl Flames (Journal of Engineering for Gas Turbines and Power, 2025) | 2. Measurements of CO and NOx Emissions From Premixed Turbulent Methane/Hydrogen Flames (Journal of Engineering for Gas Turbines and Power, 2025)</t>
         </is>
       </c>
       <c r="X9" s="3">
-        <f>HYPERLINK("https://doi.org/10.1115/1.4053164 | https://doi.org/10.1017/jfm.2021.433", "https://doi.org/10.1115/1.4053164 | https://doi.org/10.1017/jfm.2021.433")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/1.4069796 | https://doi.org/10.1115/1.4069625", "https://doi.org/10.1115/1.4069796 | https://doi.org/10.1115/1.4069625")</f>
         <v/>
       </c>
       <c r="Y9" s="2" t="inlineStr">
         <is>
-          <t>measuring transverse flame transfer functions via phase-locked OH-PLIF in a swirl-stabilized combustor, demonstrating that transverse excitation produces peak gain at the swirler geometric resonance rather than the convective residence time, directly altering annular combustor thermoacoustic stability predictions.</t>
+          <t>investigating swirl geometry effects on flame morphology and emissions in rich premixed NH3-air flames for an RRQL system, demonstrating that compact flames minimize wall quenching and enable post-flame relaxation to suppress NOx and NH3 emissions.</t>
         </is>
       </c>
       <c r="Z9" s="2" t="inlineStr">
@@ -2363,64 +2363,64 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Computational soft-matter and mesoscale fluid mechanics -- lattice Boltzmann / immersed boundary simulations of active elastic filaments, magnetically controlled microswimmers, elastic capsule deformation in microchannel flow, and interfacial transport in patterned soft-wetting surfaces.</t>
+          <t>Quantum lattice Boltzmann methods (QLBM) for phase-change heat transfer and mesoscale modeling of responsive hydrogel interfaces and fluid-structure interaction.</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Lattice-Boltzmann Method (LBM), Immersed Boundary Method (IBM), Elastic network membrane model, Magnetic dipole actuator model, Finite element structural coupling</t>
+          <t>Quantum Lattice Boltzmann Method (QLBM), Dissipative Particle Dynamics (DPD), Quantum circuit state storage (53 qubits), Immersed Boundary Method (IBM)</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Magnetic soft robot locomotion across unstructured terrains</t>
+          <t>Neutron Reflectometry and Compression of Graded Hydrogel Surfaces</t>
         </is>
       </c>
       <c r="P10" s="3">
-        <f>HYPERLINK("https://doi.org/10.1002/adma.202307002", "https://doi.org/10.1002/adma.202307002")</f>
+        <f>HYPERLINK("https://doi.org/10.1002/admi.70580", "https://doi.org/10.1002/admi.70580")</f>
         <v/>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>simulating magnetic soft robot locomotion with IBM-coupled elastic shell mechanics across terrain roughness Ra/L = 0-0.3, demonstrating undulatory gaits outperform rolling by 2.8x on irregular substrates with gait switching at critical roughness threshold Ra/L = 0.12.</t>
+          <t>investigating depth-wise graded hydrogel layers via neutron reflectometry and DPD mesoscale simulations, demonstrating that near-surface polymer network collapse under compression dictates contact stress modulation and effective elastic modulus.</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>IBM-coupled elastic shell finite element mechanics simulates magnetic soft robot locomotion across substrates with random height perturbations up to 30% of body length. Undulatory gaits outperform rolling gaits by 2.8x on irregular substrates. Gait switching occurs at a terrain roughness threshold of Ra/L = 0.12.</t>
+          <t>ABSTRACT Polyacrylamide hydrogels with depth‐wise gradients in polymer density (i.e., surface gel layers) are ideal synthetic models to understand stress modulation in hierarchical, compositionally‐graded biological tissues, including articular cartilage, in part, due to their similarities in water content and network structure. This work investigated surface gel layer thickness and crosslinker mobility (e.g., covalent crosslinks vs. physical entanglements) in polyacrylamide hydrogels and their impact on mechanical properties via confocal microscopy, indentation and compression measurements, neutron reflectivity, and mesoscale modeling. Hydrogels polymerized against oxygen‐permeable polydimethylsiloxane exhibited thicker surface gel layers and significantly lower elastic modulus compared to hydrogels polymerized against oxygen‐impermeable glass. Physical entanglements lowered the hydrogel elastic modulus within the surface gel layer and throughout the bulk. Neutron reflectivity revealed the collapse of near‐surface polymer networks under compressive loads, in good agreement with dissipative particle dynamics (DPD) simulations. Our results suggested that both the hydrogel elastic...</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>Elastic capsules in shear flow near a planar wall: Numerical simulation</t>
+          <t>Quantum lattice Boltzmann algorithm for heat transfer with phase change</t>
         </is>
       </c>
       <c r="T10" s="3">
-        <f>HYPERLINK("https://doi.org/10.1063/5.0078753", "https://doi.org/10.1063/5.0078753")</f>
+        <f>HYPERLINK("https://doi.org/10.1088/2058-9565/ae7b7c", "https://doi.org/10.1088/2058-9565/ae7b7c")</f>
         <v/>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>simulating elastic capsule wall migration via IB-LBM at Ca=0.1-0.5 and h/a=0.1-2.0, demonstrating near-wall membrane amplifies principal strain by 45-68% relative to far-field and lateral migration velocity scales as Ca*(h/a)^-3.</t>
+          <t>implementing a quantum lattice Boltzmann method (QLBM) on 17 lattice nodes using 53 qubits for phase-change heat transfer, demonstrating accurate moving interface tracking with temperature RMS errors of order 0.01 relative to classical analytical solutions.</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>IB-LBM simulates elastic capsule dynamics in shear flow near a rigid wall. Near-wall membrane deformation is amplified by 45-68% relative to far-field, with maximum principal strain of 0.42 at Ca=0.5, h/a=0.15. Lateral migration velocity scales as Ca*(h/a)^-3.</t>
+          <t>Abstract Heat transfer involving phase change is computationally intensive due to moving phase boundaries, nonlinear computations, and time step restrictions. This paper presents a quantum lattice Boltzmann method (QLBM) for simulating heat transfer with phase change. The approach leverages the statistical nature of the lattice Boltzmann method (LBM) while addressing the challenges of discontinuous phase transitions in quantum computing. The method implements an interface-tracking strategy that partitions the problem into separate solid and liquid domains, enabling the algorithm to handle the discontinuity in the enthalpy–temperature relationship. We store phase change information in the quantum circuit to reduce information exchange between classical and quantum hardware, a bottleneck in many quantum applications. Results from the implementation agree with both classical LBM and analytical solutions, demonstrating QLBM as an effective approach for analyzing thermal systems with phase transitions. Simulations using 17 lattice nodes with 53 qubits demonstrate temperature root-mean-square errors of order 0.01 when compared against classical solutions. The method accurately tracks ...</t>
         </is>
       </c>
       <c r="W10" s="2" t="inlineStr">
         <is>
-          <t>1. Magnetic soft robot locomotion across unstructured terrains (Advanced Materials, 2023) | 2. Elastic capsules in shear flow near a planar wall: Numerical simulation (Biomicrofluidics, 2022)</t>
+          <t>1. Neutron Reflectometry and Compression of Graded Hydrogel Surfaces (Advanced Materials Interfaces, 2026) | 2. Quantum lattice Boltzmann algorithm for heat transfer with phase change (Quantum Science and Technology, 2026)</t>
         </is>
       </c>
       <c r="X10" s="3">
-        <f>HYPERLINK("https://doi.org/10.1002/adma.202307002 | https://doi.org/10.1063/5.0078753", "https://doi.org/10.1002/adma.202307002 | https://doi.org/10.1063/5.0078753")</f>
+        <f>HYPERLINK("https://doi.org/10.1002/admi.70580 | https://doi.org/10.1088/2058-9565/ae7b7c", "https://doi.org/10.1002/admi.70580 | https://doi.org/10.1088/2058-9565/ae7b7c")</f>
         <v/>
       </c>
       <c r="Y10" s="2" t="inlineStr">
         <is>
-          <t>simulating magnetic soft robot locomotion with IBM-coupled elastic shell mechanics across terrain roughness Ra/L = 0-0.3, demonstrating undulatory gaits outperform rolling by 2.8x on irregular substrates with gait switching at critical roughness threshold Ra/L = 0.12.</t>
+          <t>investigating depth-wise graded hydrogel layers via neutron reflectometry and DPD mesoscale simulations, demonstrating that near-surface polymer network collapse under compression dictates contact stress modulation and effective elastic modulus.</t>
         </is>
       </c>
       <c r="Z10" s="2" t="inlineStr">
@@ -2428,11 +2428,7 @@
           <t>Skip To Keyboard Navigation Toggle navigation George W. Woodruff School of Mechanical Engineering Main navigation Home About Ch...</t>
         </is>
       </c>
-      <c r="AA10" s="2" t="inlineStr">
-        <is>
-          <t>"Neutron Reflectometry and Compression of Graded Hydrogel Surfaces" [Advanced Materials Interfaces] (2026) [DOI: https://doi.org/10.1002/admi.70580] | "Quantum lattice Boltzmann algorithm for heat transfer with phase change" [Quantum Science and Technology] (2026) [DOI: https://doi.org/10.1088/2058-9565/ae7b7c] | "Undulatory hydrodynamics of tapered elastic plates in viscous fluid" [Journal of Fluid Mechanics] (2026) [DOI: https://doi.org/10.1017/jfm.2026.11157] | "MEASUREMENT TECHNIQUE MEASUREMENT OF ABSORBED DOSE IN WATER DURING IRRADIATION IN CARBON ION AND PROTON BEAMS USING THERMAL LUMINESCENCE DOSIMETERS номер в ФИФ: ФР.1.38.2025.52532" (2026) [DOI: https://doi.org/10.13140/rg.2.2.36020.51847] | "Mesoscale Modeling of Hydrogels Under Frictional Shear Stress" [Macromolecules] (2025) [DOI: https://doi.org/10.1021/acs.macromol.5c01748]</t>
-        </is>
-      </c>
+      <c r="AA10" s="2" t="inlineStr"/>
       <c r="AB10" s="2" t="inlineStr">
         <is>
           <t>"Deformations in Si−Li Anodes Upon Electrochemical Alloying in Nano-Confined Space" [Journal of the American Chemical Society] (2010, 324 cites) [DOI: https://doi.org/10.1021/ja1031997] | "Ultrasoft microgels displaying emergent platelet-like behaviours" [Nature Materials] (2014, 221 cites) [DOI: https://doi.org/10.1038/nmat4066] | "Harnessing Janus Nanoparticles to Create Controllable Pores in Membranes" [ACS Nano] (2008, 198 cites) [DOI: https://doi.org/10.1021/nn8000998]</t>
@@ -2563,64 +2559,64 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Lattice-Boltzmann and fluctuating lattice-Boltzmann methods for multiphase suspension flows, deformable capsule dynamics in microcirculation, and turbulent fiber suspensions -- bridging colloidal-scale stochastic physics with engineering-scale flow predictions.</t>
+          <t>Direct numerical simulation (DNS) and experimental scaling of bubble interactions in decaying dynamic turbulence, Hinze-scale evolution, and microbubble mass-transfer control.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Lattice-Boltzmann Method (LBM), Fluctuating Lattice-Boltzmann (FLB), Immersed Boundary Method (IBM), Spectral Element DNS, Capsule membrane finite-element models</t>
+          <t>DNS of bubble-laden homogeneous isotropic turbulence, Particle Shadow Velocimetry (PSV), High-speed back-lit shadowgraphy, Lattice Boltzmann suspension modeling</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>Lattice Boltzmann simulation of the dynamics of capsule suspensions in shear flow</t>
+          <t>On the scaling of bubble interactions in dynamic turbulence: theoretical, numerical, and experimental study</t>
         </is>
       </c>
       <c r="P11" s="3">
-        <f>HYPERLINK("https://doi.org/10.1103/PhysRevFluids.7.054302", "https://doi.org/10.1103/PhysRevFluids.7.054302")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2607.25251", "https://doi.org/10.48550/arxiv.2607.25251")</f>
         <v/>
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>coupling LBM with finite-element capsule membrane models for volume fractions up to 0.40, demonstrating hydrodynamic capsule interactions produce shear-induced diffusivity of 3.2e-3 and drive a 340% viscosity increase from dilute to concentrated regimes.</t>
+          <t>investigating bubbly decaying homogeneous isotropic turbulence via DNS and experiments, demonstrating that when dissipation decays rapidly the Hinze scale overtakes bubble diameter, driving a transition from super-Hinze to capillary-dominated sub-Hinze scaling.</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>LBM coupled with finite-element membrane models studies capsule suspensions in shear flow at volume fractions up to 0.40. Shear-induced diffusion coefficient D_s/gamma_dot*a^2 = 3.2e-3, comparable to experimental hard-sphere measurements. Bulk suspension viscosity increases by 340% from dilute to concentrated regime at the same capillary number.</t>
+          <t>This study investigates dilute bubbly decaying homogeneous isotropic turbulence at high Reynolds number using theory, direct numerical simulation, and experiments. The turbulent kinetic energy and dissipation rate follow power-law decay, while the bubble population reorganizes relative to the evolving Hinze scale. When the dissipation decays sufficiently rapidly, the Hinze scale grows faster than the characteristic bubble diameter, driving the population from super-Hinze toward sub-Hinze sizes. The system passes through a mixed regime in which coalescence dominates but breakup remains active, followed by a pure-coalescence regime. Residual breakup in the mixed regime increases the number of small bubbles and enhances coalescence, leading to faster growth of the characteristic bubble size. DNS of dilute bubble-laden turbulence shows decay exponents close to single-phase turbulence and a bubble-size distribution that shifts toward smaller diameter relative to the Hinze scale. Before the transition, the distribution exhibits two power-law ranges associated with capillary effects and inertial breakup; after the transition, it approaches a single capillary-dominated scaling. Theory a...</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>Fluctuating lattice Boltzmann method for complex fluids and dense suspensions</t>
+          <t>Mass-Transfer Control With Microbubbles in Highly Turbulent Decaying Flows</t>
         </is>
       </c>
       <c r="T11" s="3">
-        <f>HYPERLINK("https://doi.org/10.1017/jfm.2021.432", "https://doi.org/10.1017/jfm.2021.432")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2604.24520", "https://doi.org/10.48550/arxiv.2604.24520")</f>
         <v/>
       </c>
       <c r="U11" s="2" t="inlineStr">
         <is>
-          <t>extending fluctuating LBM to dense suspensions at volume fractions 0.35-0.55, demonstrating sub-diffusive caging dynamics with MSD ~ t^0.72 and predicting viscosity divergence at 0.63 consistent with Krieger-Dougherty theory.</t>
+          <t>combining extreme turbulence (Re_lambda ~ 10^3) with minute surfactant addition (~0.01% CMC) in a straight duct, demonstrating that interfacial tuning arrests bubble coalescence and dictates micron-scale bubble size distributions.</t>
         </is>
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>The fluctuating LBM is extended to dense suspensions with thermodynamically consistent Langevin noise. At volume fractions 0.35-0.55, the model captures sub-diffusive dynamics with MSD scaling as t^0.72, consistent with colloidal glass transition theories. Suspension viscosity diverges at volume fraction 0.63, consistent with Krieger-Dougherty theory.</t>
+          <t>We hypothesize that combining extreme turbulence with a minute reduction in surface tension $σ$ (surface tension of the liquid) using surfactant provides a simple and scalable route for controlling micron scale bubble size in gas--liquid systems. To test this, we generate high-intensity turbulence using a multiphase pump [turbulent intensity $\ge 40\%$; Taylor Reynolds number $Re_λ=\mathcal{O}(10^3)$; bulk Reynolds number $Re=\mathcal{O}(10^5)$] feeding a straight duct, which produces a decaying turbulent flow where, without additives, bubble coalescence dominates and causes monotonic downstream growth in the mean diameter $d_\mathrm{avg}$ of the bubbles. This growth is governed by the turbulent dissipation rate $\varepsilon$. High-speed imaging, back-lit shadowgraph and particle shadow velocimetry (PSV) quantify bubble statistics ($d_\mathrm{avg}$, and the bubble-size distribution) and turbulence metrics (turbulent kinetic energy $k$, turbulence intensity $\mathcal{I}$, and dissipation rate $\varepsilon$). We then introduce a minute amount ($\sim 0.01\%$ critical micelle concentration) of additive that produces a slight reduction in $σ$, used here only as an interfacial tuning ...</t>
         </is>
       </c>
       <c r="W11" s="2" t="inlineStr">
         <is>
-          <t>1. LBM simulation of capsule suspensions in shear flow (Physical Review Fluids, 2022) | 2. Fluctuating LBM for dense suspensions (Journal of Fluid Mechanics, 2021)</t>
+          <t>1. On the scaling of bubble interactions in dynamic turbulence: theoretical, numerical, and experimental study (arXiv, 2026) | 2. Mass-Transfer Control With Microbubbles in Highly Turbulent Decaying Flows (arXiv, 2026)</t>
         </is>
       </c>
       <c r="X11" s="3">
-        <f>HYPERLINK("https://doi.org/10.1103/PhysRevFluids.7.054302 | https://doi.org/10.1017/jfm.2021.432", "https://doi.org/10.1103/PhysRevFluids.7.054302 | https://doi.org/10.1017/jfm.2021.432")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2607.25251 | https://doi.org/10.48550/arxiv.2604.24520", "https://doi.org/10.48550/arxiv.2607.25251 | https://doi.org/10.48550/arxiv.2604.24520")</f>
         <v/>
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>coupling LBM with finite-element capsule membrane models for volume fractions up to 0.40, demonstrating hydrodynamic capsule interactions produce shear-induced diffusivity of 3.2e-3 and drive a 340% viscosity increase from dilute to concentrated regimes.</t>
+          <t>investigating bubbly decaying homogeneous isotropic turbulence via DNS and experiments, demonstrating that when dissipation decays rapidly the Hinze scale overtakes bubble diameter, driving a transition from super-Hinze to capillary-dominated sub-Hinze scaling.</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr">
@@ -2763,64 +2759,64 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Multi-fidelity rotorcraft aeromechanics -- coupling CAMRAD II with CFD/CSD for dynamic stall, blade-vortex interaction, and coaxial rotor-wake aerodynamics to enable next-generation Urban Air Mobility eVTOL vehicle design.</t>
+          <t>Proprotor-wing interactional aerodynamics across tiltrotor conversion maneuvers, mid-to-high-fidelity CFD coupling (Helios / OVERFLOW / ROAM), and reduced-order wake models for Advanced Air Mobility.</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>CAMRAD II, Overset CFD/CSD loose coupling, Unsteady Vortex Lattice Method (UVLM), GT-Hybrid RANS-LES, Aeroflite wind tunnel PIV validation</t>
+          <t>Helios-OVERFLOW overset CFD, Reduced Order Aerodynamic Model (ROAM), Actuator Line Model (ALM), Immersed Boundary Method (IBM), Power spectral density surface pressure analysis</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Validation of an Unsteady Vortex Lattice Method for Coaxial Rotor Wake Interactions</t>
+          <t>Physics of the Proprotor–Wing Interactional Aerodynamics Across the Tiltrotor Conversion Maneuver</t>
         </is>
       </c>
       <c r="P12" s="3">
-        <f>HYPERLINK("https://doi.org/10.4050/JAHS.67.032007", "https://doi.org/10.4050/JAHS.67.032007")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.c038965", "https://doi.org/10.2514/1.c038965")</f>
         <v/>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>validating a free-wake UVLM for coaxial rotor wake mutual induction against Georgia Tech PIV data, demonstrating 6.4% RMS blade normal force accuracy and capturing the figure-8 loading signature in the lower rotor from upper-rotor tip-vortex impingement.</t>
+          <t>simulating two-way coupled proprotor-wing interaction across tilt angles in 15-degree increments using high-fidelity CFD, demonstrating that wing surface pressure PSD reveals dominant wake excitation frequencies during tiltrotor conversion maneuvers.</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>An unsteady vortex lattice method (UVLM) for coaxial rotor aerodynamics is validated against GT Aeroflite wind tunnel PIV data. The UVLM predicts blade normal force within 6.4% RMS error across the azimuth and reproduces the characteristic figure-8 loading signature in the lower rotor due to upper rotor tip vortex impingement.</t>
+          <t>The conversion maneuver is one of the most complex and hazardous aspects of tiltrotor operations. The complex interactions increase pilot workload and vibratory wing loads, making it imperative to further understand and accurately predict this dynamic operation. An extensively correlated high-fidelity computational fluid dynamics (CFD) model elucidates the physics within these two-way coupled aerodynamic interactions for a generic model-scale tractor proprotor–wing configuration. Quasi-static evaluations are conducted for proprotor tilt angles in fifteen degree increments to capture the conversion from low-speed edgewise flight to cruise. To assess and quantify the coupled proprotor–wing interactions, additional assessments of an isolated wing at two relevant wing angles of attack and an isolated proprotor operating at all tilt angles were conducted. Wing thickness and loading were mildly correlated with the proprotor loads due to the large proprotor–wing separation relative to the proprotor radius. The proprotor-to-wing effects were assessed using a power spectral density of the wing surface pressure within the proprotor wake. This novel approach elucidates the dominant frequen...</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>Multi-fidelity aeromechanical analysis of a UH-60A rotor in forward flight using loosely coupled CFD/CSD</t>
+          <t>Mid-Fidelity Investigation of the Proprotor-Wing Aerodynamic Interactions across the Tiltrotor Conversion Maneuver</t>
         </is>
       </c>
       <c r="T12" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.J059977", "https://doi.org/10.2514/1.J059977")</f>
+        <f>HYPERLINK("https://doi.org/10.4050/f-0082-2026-0243", "https://doi.org/10.4050/f-0082-2026-0243")</f>
         <v/>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>loosely coupling overset RANS with CAMRAD II across UH-60A advance ratios from 0.15 to 0.368, demonstrating rotor performance within 4.5% of flight test data and capturing dynamic stall vibratory 4P loads at high-advance-ratio conditions.</t>
+          <t>evaluating the Helios mid-fidelity ROAM actuator line model against OVERFLOW for proprotor-wing conversion, demonstrating that adaptive mesh refinement (AMR) in the off-body Cartesian domain is essential for capturing proprotor vortex trajectory and wing load distribution.</t>
         </is>
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>Loosely coupled CFD/CSD methodology is applied to the UH-60A main rotor across advance ratios from mu = 0.15 to 0.368. Rotor performance including thrust, torque, and blade pitch angles agree with UH-60A flight test data within 4.5%. Dynamic stall at high advance ratios is captured with qualitative agreement to flight test vibratory loads at 4P frequency.</t>
+          <t>This paper assesses the capabilities and limitations of mid-fidelity computational fluid dynamics (CFD) approaches when resolving the complex aerodynamic interactions for a generic model-scale proprotor-wing configuration across the tiltrotor conversion maneuver. The Helios mid-fidelity Reduced Order Aerodynamic Model (ROAM) is evaluated against prior extensively validated high-fidelity Helios-OVERFLOW assessments for the proprotor-wing configuration. The ROAM actuator line model (ALM), which represents the proprotor blade via source terms injected into the off-body Cartesian domain, is assessed for the isolated proprotor configuration at several mesh resolutions to understand the requirements to accurately resolve the proprotor physics across the conversion maneuver. The impact of adaptive mesh refinement (AMR) on ROAM's ability to resolve the proprotor physics is also investigated. Next, the flow characteristics and wing loads are evaluated using the ROAM immersed boundary method (IBM) for the isolated wing. The sensitivity of the ROAM IBM predictions to mesh resolution and boundary condition selection is quantified in these assessments. Leveraging the findings from the isolat...</t>
         </is>
       </c>
       <c r="W12" s="2" t="inlineStr">
         <is>
-          <t>1. Validation of an Unsteady Vortex Lattice Method for Coaxial Rotor Wake Interactions (JAHS, 2022) | 2. Multi-fidelity aeromechanical analysis of UH-60A rotor using loosely coupled CFD/CSD (AIAA J., 2021)</t>
+          <t>1. Physics of the Proprotor–Wing Interactional Aerodynamics Across the Tiltrotor Conversion Maneuver (Journal of Aircraft, 2026) | 2. Mid-Fidelity Investigation of the Proprotor-Wing Aerodynamic Interactions across the Tiltrotor Conversion Maneuver (2026)</t>
         </is>
       </c>
       <c r="X12" s="3">
-        <f>HYPERLINK("https://doi.org/10.4050/JAHS.67.032007 | https://doi.org/10.2514/1.J059977", "https://doi.org/10.4050/JAHS.67.032007 | https://doi.org/10.2514/1.J059977")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.c038965 | https://doi.org/10.4050/f-0082-2026-0243", "https://doi.org/10.2514/1.c038965 | https://doi.org/10.4050/f-0082-2026-0243")</f>
         <v/>
       </c>
       <c r="Y12" s="2" t="inlineStr">
         <is>
-          <t>validating a free-wake UVLM for coaxial rotor wake mutual induction against Georgia Tech PIV data, demonstrating 6.4% RMS blade normal force accuracy and capturing the figure-8 loading signature in the lower rotor from upper-rotor tip-vortex impingement.</t>
+          <t>simulating two-way coupled proprotor-wing interaction across tilt angles in 15-degree increments using high-fidelity CFD, demonstrating that wing surface pressure PSD reveals dominant wake excitation frequencies during tiltrotor conversion maneuvers.</t>
         </is>
       </c>
       <c r="Z12" s="2" t="inlineStr">
@@ -2959,64 +2955,64 @@
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Stochastic optimal control theory, Hamilton-Jacobi-Bellman PDEs, and adaptive numerical methods for diffusion-dominated transport -- developing efficient solvers for high-dimensional control problems in turbulent mixing, ensemble Kalman filtering, and molecular dynamics.</t>
+          <t>Dynamics-guided weighted weak-form identification of differential equations from noisy trajectories and discrete Mean Field Games (Graph MFG) on finite graphs as initial value optimization.</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Hamilton-Jacobi-Bellman (HJB) finite-difference solvers, Policy iteration, Ensemble Kalman Inversion (EKI), Stochastic Runge-Kutta, Adaptive mesh refinement (h-refinement)</t>
+          <t>Dynamics-guided weighted weak form, Feature voting ensembles, Graph Mean Field Games (Graph MFG), Neural network ODE integrators, Hamilton-Jacobi-Bellman optimization</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Efficient numerical methods for high-dimensional stochastic control with application to turbulent diffusion</t>
+          <t>Identification of Differential Equations by Dynamics-Guided Weighted Weak Form with Voting</t>
         </is>
       </c>
       <c r="P13" s="3">
-        <f>HYPERLINK("https://doi.org/10.1137/21M1409124", "https://doi.org/10.1137/21M1409124")</f>
+        <f>HYPERLINK("https://doi.org/10.4208/cicp.oa-2025-0163", "https://doi.org/10.4208/cicp.oa-2025-0163")</f>
         <v/>
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>solving 6D HJB equations via sparse-grid policy iteration for turbulent scalar mixing control at Re_lambda=150, demonstrating 38% scalar variance reduction using 4.2x fewer grid points through dimension-independent O(h^4*|log h|^(d-1)) convergence.</t>
+          <t>developing dynamics-guided weighted weak formulations with voting strategies for PDE discovery from single noisy trajectories, demonstrating robust recovery of governing differential terms and coefficients by weighting high-dynamic regions.</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>Sparse tensor grid HJB solvers with policy iteration applied to 6D turbulent scalar mixing control at Re_lambda=150. The sparse grid achieves dimension-independent convergence O(h^4*|log h|^(d-1)) vs O(h^2) for standard solvers. Controls reduce scalar variance by 38% using 4.2x fewer grid points than full-tensor discretization.</t>
+          <t>In the identification of differential equations from data, significant progresses have been made with the weak/integral formulation. In this paper, we explore the direction of finding more efficient and robust test functions adaptively given the observed data. While this is a difficult task, we propose weighting a collection of localized test functions for better identification of differential equations from a single trajectory of noisy observations on the differential equation. We find that using high dynamic regions is effective in finding the equation as well as the coefficients, and propose a dynamics indicator per differential term and weight the weak form accordingly. For stable identification against noise, we further introduce a voting strategy to identify the active features from an ensemble of recovered results by selecting the features that frequently occur in different weighting of test functions. Systematic numerical experiments are provided to demonstrate the robustness of our method.</t>
         </is>
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>Adaptive mesh refinement for Hamilton-Jacobi-Bellman equations in continuous-time stochastic control</t>
+          <t>Discrete Mean Field Games on Finite Graphs as Initial Value Optimization</t>
         </is>
       </c>
       <c r="T13" s="3">
-        <f>HYPERLINK("https://doi.org/10.4208/jcm.2009-m2019-0214", "https://doi.org/10.4208/jcm.2009-m2019-0214")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2604.05685", "https://doi.org/10.48550/arxiv.2604.05685")</f>
         <v/>
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
-          <t>applying AMR with gradient-discontinuity indicators to HJB solvers for stochastic control, demonstrating 75-82% reduction in degrees of freedom vs uniform grids while maintaining L-inf error below 1% and recovering optimal O(h^2) convergence at the free boundary.</t>
+          <t>reformulating discrete potential Mean Field Games on finite graphs as initial value optimization problems (Graph MFG-IV), demonstrating reduced search space by utilizing coupled Hamilton-Jacobi ODE integrators without full time-discretization.</t>
         </is>
       </c>
       <c r="V13" s="2" t="inlineStr">
         <is>
-          <t>AMR with a posteriori gradient-discontinuity error estimators for HJB PDE solvers in stochastic control. Applied to LQR with state constraints, stopping-time problem, and pursuit-evasion game. AMR reduces degrees of freedom by 75-82% vs uniform grids while maintaining L-inf error below 1%.</t>
+          <t>In this paper, we propose an initial value fomulation of the discrete mean field games on finite graphs (Graph MFG), and design a neural network based approach to solve it. Graph MFG describes infinite, non-cooperative and interactive homogeneous agents move on node states through the edges to optimize their own goals. Nash Equilibrium of the Graph MFG is characterized by a coupled ordinary differential equations (ODE) system, including the discrete forward continuity equation and the discrete backward Hamilton-Jacobi equation. In this paper, we mainly focus on the potential mean field games (Potential MFG) on finite graphs, which has an infinite-dimensional constrained optimization structure. We reformulate Potential MFG as an initial value finite-dimentional optimization problem with dynamics constrains, names Graph MFG-IV. Specifically, the initial condition of the Hamilton-Jacobi equation is regarded as the unique variable, constrained by the coupled Hamilton-Jacobi and continuity equation system as the ODE integrator. This formulation is a reduced-order model, which avoids time-discretization of the infinite-dimensional path and has a much smaller searching space than the g...</t>
         </is>
       </c>
       <c r="W13" s="2" t="inlineStr">
         <is>
-          <t>1. Efficient numerical methods for high-dimensional stochastic control with application to turbulent diffusion (SIAM J. Control Optim., 2022) | 2. Adaptive mesh refinement for HJB equations in stochastic control (J. Computational Mathematics, 2021)</t>
+          <t>1. Identification of Differential Equations by Dynamics-Guided Weighted Weak Form with Voting (Communications in Computational Physics, 2026) | 2. Discrete Mean Field Games on Finite Graphs as Initial Value Optimization (arXiv, 2026)</t>
         </is>
       </c>
       <c r="X13" s="3">
-        <f>HYPERLINK("https://doi.org/10.1137/21M1409124 | https://doi.org/10.4208/jcm.2009-m2019-0214", "https://doi.org/10.1137/21M1409124 | https://doi.org/10.4208/jcm.2009-m2019-0214")</f>
+        <f>HYPERLINK("https://doi.org/10.4208/cicp.oa-2025-0163 | https://doi.org/10.48550/arxiv.2604.05685", "https://doi.org/10.4208/cicp.oa-2025-0163 | https://doi.org/10.48550/arxiv.2604.05685")</f>
         <v/>
       </c>
       <c r="Y13" s="2" t="inlineStr">
         <is>
-          <t>solving 6D HJB equations via sparse-grid policy iteration for turbulent scalar mixing control at Re_lambda=150, demonstrating 38% scalar variance reduction using 4.2x fewer grid points through dimension-independent O(h^4*|log h|^(d-1)) convergence.</t>
+          <t>developing dynamics-guided weighted weak formulations with voting strategies for PDE discovery from single noisy trajectories, demonstrating robust recovery of governing differential terms and coefficients by weighting high-dynamic regions.</t>
         </is>
       </c>
       <c r="Z13" s="2" t="inlineStr">
@@ -3139,64 +3135,64 @@
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Variational image reconstruction, PDE-based level-set methods, and machine-learning-augmented numerical schemes for fluid interface tracking and multiphase flow image segmentation -- bridging applied harmonic analysis with high-order conservative transport methods.</t>
+          <t>Sampled Local WeakIdent (SLW-Ident) for discovering transitioning governing PDEs from single-set data and unified variational Potts frameworks for weakly supervised image segmentation.</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Variational level-set methods (Chan-Vese), Total variation minimization, PDE-constrained optimization, Physics-informed neural networks (PINNs), ADMM</t>
+          <t>Sampled Local WeakIdent (SLW-Ident), Local patch residual error analysis, Simplex-constrained Potts models, RKHS fuzzy membership functions, Weakly supervised deep learning loss</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>A variational framework for exemplar-based image inpainting integrated with level-set interface tracking</t>
+          <t>Identifying changing partial differential equations using Sampled Local WeakIdent</t>
         </is>
       </c>
       <c r="P14" s="3">
-        <f>HYPERLINK("https://doi.org/10.1137/21M1442626", "https://doi.org/10.1137/21M1442626")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2608.12479", "https://doi.org/10.48550/arxiv.2608.12479")</f>
         <v/>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>coupling exemplar-based TV inpainting with Chan-Vese level-set evolution via ADMM for corrupted multiphase flow images, demonstrating SSIM improvement from 0.74 to 0.91 and boundary localization error reduction to 1.2 pixels through joint rather than sequential optimization.</t>
+          <t>proposing Sampled Local WeakIdent (SLW-Ident) to identify changing governing equations from a single dataset, demonstrating that sampling localized patches and tracking residual errors accurately detects spatial transitions between varying-coefficient PDEs.</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>A variational framework couples exemplar-based TV inpainting with Chan-Vese level-set evolution via ADMM for fluid imaging. Applied to synthetic multiphase flow images with 30% corruption, the joint model achieves SSIM = 0.91 and boundary localization error of 1.2 pixels, vs SSIM = 0.74 for sequential inpainting-then-segmentation.</t>
+          <t>We propose Sampled Local WeakIdent (SLW-Ident), a framework for identifying changing governing equations from a single set of given data. Different from a typical approach of using finite element based approximation to represent varying coefficients, this paper explores a local approach in identification of differential equations. First, we present the power of Local WeakIdent which gives good local identification and is also computationally efficient with a small patch size, yet it can be sensitive to local perturbations. We propose SLW-Ident which stabilizes the identification process and also incorporates global information: we first sample patches in the whole given domain, identify equations for each sampled patch, then use residual error of these equations to find the transitions between different equations. We refer to a region where the support of the identified equation does not change to be a region of one equation. Within each region of one equation, we pick the most frequently identified equation as the identified equation, and find constant as well as varying coefficient PDEs within each region of one equation. This is justified by an uncertainty quantification theo...</t>
         </is>
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>Physics-informed neural networks for multiphase flow interface reconstruction from tomographic measurements</t>
+          <t>A Unified Variational Framework for Deep Weakly Supervised Image Segmentation</t>
         </is>
       </c>
       <c r="T14" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.jcp.2023.112086", "https://doi.org/10.1016/j.jcp.2023.112086")</f>
+        <f>HYPERLINK("https://arxiv.org/abs/2607.19669", "https://arxiv.org/abs/2607.19669")</f>
         <v/>
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>embedding incompressible two-phase NS and VOF physics residuals in PINNs for interface reconstruction from 12 tomographic angles, demonstrating interface curvature MAE of 0.08/cm versus 0.31/cm for unphysical FBP and sub-voxel (0.5 mm RMS) accuracy on experimental bubbly-flow CT data.</t>
+          <t>formulating a simplex-constrained Potts model with RKHS fuzzy membership for weakly supervised image segmentation, demonstrating superior accuracy over partial cross-entropy baselines without requiring dense ground-truth segmentation masks.</t>
         </is>
       </c>
       <c r="V14" s="2" t="inlineStr">
         <is>
-          <t>PINNs embedding two-phase incompressible Navier-Stokes and VOF transport in the loss function reconstruct gas-liquid interfaces from 12 tomographic projections. Interface curvature MAE = 0.08/cm vs 0.31/cm for filtered backprojection. Experimental X-ray CT bubbly flow interface located to within 0.5 mm RMS.</t>
+          <t>We propose a unified variational framework for image segmentation under sparse pixel-level supervision. Our method is based on a simplex-constrained Potts model with a smooth perimeter regularizer, yielding a convex, smooth energy functional that can be used as a training loss in weakly supervised deep learning paradigms or optimized efficiently using iterative methods. Sparse labels are incorporated into the data fidelity term by constructing a fuzzy membership function via a function extension problem in a Reproducing Kernel Hilbert Space (RKHS), which can effectively capture inhomogeneous intensity statistics. The derived discrete loss for training standard networks demonstrates robustness and consistent improvements over non-training and partial cross-entropy (PCE) baselines in experiments, achieving comparable performance without requiring ground-truth segmentation images.</t>
         </is>
       </c>
       <c r="W14" s="2" t="inlineStr">
         <is>
-          <t>1. Variational framework for exemplar-based inpainting integrated with level-set interface tracking (SIAM J. Imaging Sci., 2022) | 2. PINNs for multiphase flow interface reconstruction from tomographic measurements (JCP, 2023)</t>
+          <t>1. Identifying changing partial differential equations using Sampled Local WeakIdent (arXiv, 2026) | 2. A Unified Variational Framework for Deep Weakly Supervised Image Segmentation (arXiv, 2026)</t>
         </is>
       </c>
       <c r="X14" s="3">
-        <f>HYPERLINK("https://doi.org/10.1137/21M1442626 | https://doi.org/10.1016/j.jcp.2023.112086", "https://doi.org/10.1137/21M1442626 | https://doi.org/10.1016/j.jcp.2023.112086")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2608.12479 | https://arxiv.org/abs/2607.19669", "https://doi.org/10.48550/arxiv.2608.12479 | https://arxiv.org/abs/2607.19669")</f>
         <v/>
       </c>
       <c r="Y14" s="2" t="inlineStr">
         <is>
-          <t>coupling exemplar-based TV inpainting with Chan-Vese level-set evolution via ADMM for corrupted multiphase flow images, demonstrating SSIM improvement from 0.74 to 0.91 and boundary localization error reduction to 1.2 pixels through joint rather than sequential optimization.</t>
+          <t>proposing Sampled Local WeakIdent (SLW-Ident) to identify changing governing equations from a single dataset, demonstrating that sampling localized patches and tracking residual errors accurately detects spatial transitions between varying-coefficient PDEs.</t>
         </is>
       </c>
       <c r="Z14" s="2" t="inlineStr">
@@ -3319,64 +3315,64 @@
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>High-order Runge-Kutta discontinuous Galerkin (RKDG) schemes, central compact WENO reconstruction, and entropy-stable finite difference methods for hyperbolic conservation laws -- developing structure-preserving schemes for compressible Euler/Navier-Stokes flows.</t>
+          <t>Neural networks with local converging input (NNLCI) for unstructured-grid supersonic CFD and multiphase Euler CFD simulations of bubble-driven fluidization hydrodynamics.</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Runge-Kutta Discontinuous Galerkin (RKDG), Central compact WENO (CC-WENO), Limiter-free high-order reconstruction, Entropy-stable flux schemes, Gauss-Seidel relaxation</t>
+          <t>Neural Network with Local Converging Input (NNLCI), Unstructured-grid supersonic Euler solvers, Multiphase Eulerian CFD, Population Balance Modeling (PBM)</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>A new fifth-order finite difference compact reconstruction unequal-sized WENO scheme for compressible flow</t>
+          <t>Neural Network with Local Converging Input for Unstructured-Grid Computational Fluid Dynamics</t>
         </is>
       </c>
       <c r="P15" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.jcp.2022.111140", "https://doi.org/10.1016/j.jcp.2022.111140")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.j063885", "https://doi.org/10.2514/1.j063885")</f>
         <v/>
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>designing a fifth-order compact-reconstruction unequal-sized WENO scheme for compressible Euler flows, demonstrating 4.2x reduction in L-inf error on smooth wave tests relative to WENO-JS while maintaining ENO-sharp shock capture without parameter tuning.</t>
+          <t>developing neural networks with local converging input (NNLCI) on unstructured grids for supersonic flows with shocks, demonstrating several orders of magnitude reduction in computing wall time with single-network generalization across multiple bump configurations.</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>A new fifth-order finite difference scheme combining compact reconstruction and unequal-sized WENO stencils is proposed for compressible Euler equations. Compared to standard fifth-order WENO-JS, the new scheme reduces L-inf error by a factor of 4.2 on smooth wave tests while maintaining ENO-sharp shock capture without parameter tuning.</t>
+          <t>In recent years, surrogate models based on deep neural networks have been widely used to solve partial differential equations for fluid flow physics. This kind of model focuses on global interpolation of the training data and thus requires a large network structure. The process is both time consuming and computationally costly. In the present study, we develop a neural network with local converging input (NNLCI) for high-fidelity prediction using unstructured data. The framework uses the local domain of dependence with converging coarse solutions as input, thereby greatly reducing computational resource and training time. As a validation case, the NNLCI method is applied to study two-dimensional inviscid supersonic flows in channels with bumps. Different bump geometries and locations are examined to benchmark the effectiveness and versatility of this new approach. The NNLCI method can accurately and efficiently capture the structure and dynamics of the entire flowfield, including regions with shock discontinuities. For a new bump configuration, the method can perform prediction with only one neural network, eliminating the need for repeated training of multiple networks for different geometries. A saving of computing wall time is achieved by several orders of magnitude against the high-fidelity simulation with the same level of accuracy. The demand on training data is modest, and the training data can be allocated sparsely. These features are especially advantageous compared with conventional global-to-global deep learning methods and physics-informed methods.</t>
         </is>
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>Central compact schemes with spectral-like resolution for computational aeroacoustics</t>
+          <t>Euler multiphase‐CFD simulation on a bubble‐driven gas–liquid–solid fluidized bed</t>
         </is>
       </c>
       <c r="T15" s="3">
-        <f>HYPERLINK("https://doi.org/10.1137/20M1371847", "https://doi.org/10.1137/20M1371847")</f>
+        <f>HYPERLINK("https://doi.org/10.1002/cjce.24742", "https://doi.org/10.1002/cjce.24742")</f>
         <v/>
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>constructing Hermite-based central compact schemes that maintain phase error below 0.1% over 75% of the resolved wavenumber band versus 50% for classical 10th-order explicit schemes, with demonstrated superiority on acoustic pulse propagation and Taylor-Green vortex at Re=1600.</t>
+          <t>simulating gas-liquid-solid fluidized beds via Eulerian multiphase CFD and population balance modeling, demonstrating that bubble coalescence shifts bubble diameters from 2-4 mm at the base to 5-10 mm at the top, dictating axial solids holdup.</t>
         </is>
       </c>
       <c r="V15" s="2" t="inlineStr">
         <is>
-          <t>Central compact finite difference schemes with spectral-like resolution are developed using Hermite-based interpolation. The 10th-order compact scheme maintains phase error below 0.1% over 75% of the resolved wavenumber band, compared to 50% for classical 10th-order explicit schemes, with superiority on acoustic pulse propagation and Taylor-Green vortex at Re=1600.</t>
+          <t>Abstract An integrated flow model was developed to simulate the fluidization hydrodynamics in a new bubble‐driven gas–liquid–solid fluidized bed using the computational fluid dynamic (CFD) method. The results showed that axial solids holdup is affected by grid size, bubble diameter, and the interphase drag models used in the simulation. Good agreements with experimental data could be obtained by adopting the following parameters: 5 mm grid, 1.2 mm bubble diameter, the Tomiyama gas–liquid model, the Schiller–Naumann liquid–solid model, and the Gidaspow gas–solid model. At full fluidization state, an internal circulation of particles flowing upward near the wall and downward in the centre is observed, which is in the opposite direction compared with the traditional core‐annular flow structure in a gas–solid fluidized bed. The simulated results are very sensitive to bubble diameters. Using smaller bubble diameters would lead to excessive liquid bed expansions and more solid accumulated at the bottom due to a bigger gas–liquid drag force, while bigger bubble diameters would result in a higher solid bed height caused by a smaller gas–solid drag force. Considering the actual bubble distribution, population balance model (PBM) is employed to characterize the coalescence and break up of bubbles. The calculated bubble diameters grow up from 2–4 mm at the bottom to 5–10 mm at the upper section of the bed, which are comparable to those observed in experiments. The simulation results could provide valuable information for the design and optimization of this new type of fluidized system.</t>
         </is>
       </c>
       <c r="W15" s="2" t="inlineStr">
         <is>
-          <t>1. Fifth-order finite difference compact reconstruction unequal-sized WENO for compressible flow (JCP, 2022) | 2. Central compact schemes with spectral-like resolution (SIAM J. Sci. Comput., 2021)</t>
+          <t>1. Neural Network with Local Converging Input for Unstructured-Grid Computational Fluid Dynamics (AIAA Journal, 2024) | 2. Euler multiphase‐CFD simulation on a bubble‐driven gas–liquid–solid fluidized bed (The Canadian Journal of Chemical Engineering, 2022)</t>
         </is>
       </c>
       <c r="X15" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.jcp.2022.111140 | https://doi.org/10.1137/20M1371847", "https://doi.org/10.1016/j.jcp.2022.111140 | https://doi.org/10.1137/20M1371847")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.j063885 | https://doi.org/10.1002/cjce.24742", "https://doi.org/10.2514/1.j063885 | https://doi.org/10.1002/cjce.24742")</f>
         <v/>
       </c>
       <c r="Y15" s="2" t="inlineStr">
         <is>
-          <t>designing a fifth-order compact-reconstruction unequal-sized WENO scheme for compressible Euler flows, demonstrating 4.2x reduction in L-inf error on smooth wave tests relative to WENO-JS while maintaining ENO-sharp shock capture without parameter tuning.</t>
+          <t>developing neural networks with local converging input (NNLCI) on unstructured grids for supersonic flows with shocks, demonstrating several orders of magnitude reduction in computing wall time with single-network generalization across multiple bump configurations.</t>
         </is>
       </c>
       <c r="Z15" s="2" t="inlineStr">
@@ -3923,64 +3919,64 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>High-fidelity LES of supercritical-pressure reacting flows -- combining real-fluid thermodynamics, finite-rate chemistry, and subgrid turbulence closures to resolve transcritical LOX/CH4 injection, flame stabilization, and combustion instability in rocket and gas-turbine combustors.</t>
+          <t>Lagrangian coherent structures (LCS), finite-time Lyapunov exponent (FTLE) ridges, and adjoint-based receptivity/biorthogonal decomposition in compressible turbulent reacting shear layers.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>LES (Peng-Robinson real-fluid EOS), Finite-rate GRI-Mech 3.0 chemistry, Dynamic Smagorinsky subgrid, Transcritical jet DNS, RAPTOR high-performance CFD solver</t>
+          <t>Direct Numerical Simulation (DNS), Forward/backward FTLE ridges, Hyperbolic geodesic LCS, Cauchy-Green deformation tensors, Direct/adjoint biorthogonal eigenmode projection</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Large eddy simulation of a supercritical LOX/CH4 round jet flame</t>
+          <t>Planar Lagrangian transport and scalar-gradient organization in a turbulent reacting shear layer</t>
         </is>
       </c>
       <c r="P2" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2022.112183", "https://doi.org/10.1016/j.combustflame.2022.112183")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2606.20352", "https://doi.org/10.48550/arxiv.2606.20352")</f>
         <v/>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>performing real-fluid LES with Peng-Robinson EOS in a supercritical LOX/CH4 jet flame at 6 MPa, demonstrating that transcritical pseudoboiling produces a LOX core of L_c/D = 4.8 and anchors the diffusion flame within 2 jet diameters at the pseudoboiling interface.</t>
+          <t>analyzing 3D DNS of a supersonic reacting H2-air temporal mixing layer via hyperbolic geodesic LCS and FTLE ridges, demonstrating that forward/backward ridge intersections govern localized scalar-gradient enrichment and strain-dominated transport skeletons.</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>LES of a turbulent supercritical LOX/CH4 round jet flame at 6 MPa using RAPTOR with Peng-Robinson real-fluid EOS. The pseudoboiling transition of LOX injected at 120 K into supercritical methane at 300 K produces a dense LOX core of L_c/D = 4.8. Flame stabilization occurs within 2 jet diameters at the highest-density-gradient pseudoboiling interface.</t>
+          <t>We analyze planar Lagrangian transport and scalar-gradient organization in a supersonic, reacting hydrogen-air temporal mixing layer using time-resolved mid-plane data from a three-dimensional direct numerical simulation. The analysis combines forward/backward finite-time Lyapunov exponent (FTLE) fields, operational FTLE-ridge skeletons, Cauchy-Green deformation measures, shear-LCS metrics, and planar hyperbolic geodesic-LCS extraction to examine how finite-time stretching structures the reacting shear layer. The time-resolved FTLE ridges identify repelling and attracting finite-time transport skeletons in the constrained two-dimensional slice, from which ridge geometry, intersection occupancy, persistence, and scalar-conditioned transport are quantified. Hyperbolic geodesic LCS are extracted from Cauchy-Green tensors reconstructed from planar flow maps as strainlines seeded at high-$λ_{\max}$ normal maxima, providing a variational counterpart to the operational FTLE-ridge skeleton. We then relate the transport skeleton to temperature, mixture fraction, and a reaction intermediate. The results show localized forward/backward ridge overlap, strong scalar-gradient enrichment, fini...</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>Analysis of Mixing, Thermodynamic, and Combustion Characteristics of Turbulent Supercritical Flows</t>
+          <t>Receptivity and Biorthogonal Decomposition in a Reacting Temporal Mixing Layer</t>
         </is>
       </c>
       <c r="T2" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.J059845", "https://doi.org/10.2514/1.J059845")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2606.20819", "https://doi.org/10.48550/arxiv.2606.20819")</f>
         <v/>
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>combining DNS and LES with Peng-Robinson real-fluid EOS across three supercritical configurations at 6-10 MPa, demonstrating that density stratification suppresses scalar dissipation rate by 23% near the critical point and sustains sub-centimeter density gradients through the reacting zone.</t>
+          <t>applying energy-weighted adjoint projections and biorthogonal decomposition to a compressible reacting mixing layer, demonstrating that finite-thickness base states sustain unstable Kelvin-Helmholtz modes across low wavenumbers where vortex-sheet approximations remain neutral.</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>DNS and LES with Peng-Robinson EOS study three supercritical configurations: a N2 jet, LOX/H2 shear layer, and LOX/CH4 injector at 10 MPa. Density stratification produces 23% reduction in scalar dissipation rate at the critical point. Sub-centimeter density gradients persist through the reaction zone in the LOX/CH4 injector LES.</t>
+          <t>We examine receptivity and biorthogonal decomposition in a reacting temporal mixing layer using direct and adjoint eigenmodes of a finite-thickness compressible linearized operator built from the mean reacting base state. The analysis focuses on the Kelvin--Helmholtz branch and asks how the reacting base state modifies the selected temporal instability, where localized forcing most efficiently excites it, and how strongly the associated modal family is represented in time-resolved planar simulation data. Receptivity maps are constructed for mass, momentum, thermal, and mixture-fraction forcing channels using an energy-weighted adjoint projection, with biorthogonality enforced by the corresponding direct--adjoint inner product. A complementary biorthogonal decomposition provides modal amplitudes and cumulative few-mode reconstructions at the fundamental streamwise wavenumber. The finite-thickness branch is interpreted against a compressible vortex-sheet reference built from the outer-stream states. The reacting layer supports an unstable finite-thickness Kelvin--Helmholtz family over low-to-moderate wavenumbers even though the discontinuous reference is essentially neutral. Mass ...</t>
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>1. LES of a supercritical LOX/CH4 round jet flame (Combustion and Flame, 2022) | 2. Analysis of Mixing, Thermodynamic, and Combustion Characteristics of Turbulent Supercritical Flows (AIAA J., 2021)</t>
+          <t>1. Planar Lagrangian transport and scalar-gradient organization in a turbulent reacting shear layer (arXiv, 2026) | 2. Receptivity and Biorthogonal Decomposition in a Reacting Temporal Mixing Layer (arXiv, 2026)</t>
         </is>
       </c>
       <c r="X2" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2022.112183 | https://doi.org/10.2514/1.J059845", "https://doi.org/10.1016/j.combustflame.2022.112183 | https://doi.org/10.2514/1.J059845")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2606.20352 | https://doi.org/10.48550/arxiv.2606.20819", "https://doi.org/10.48550/arxiv.2606.20352 | https://doi.org/10.48550/arxiv.2606.20819")</f>
         <v/>
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>performing real-fluid LES with Peng-Robinson EOS in a supercritical LOX/CH4 jet flame at 6 MPa, demonstrating that transcritical pseudoboiling produces a LOX core of L_c/D = 4.8 and anchors the diffusion flame within 2 jet diameters at the pseudoboiling interface.</t>
+          <t>analyzing 3D DNS of a supersonic reacting H2-air temporal mixing layer via hyperbolic geodesic LCS and FTLE ridges, demonstrating that forward/backward ridge intersections govern localized scalar-gradient enrichment and strain-dominated transport skeletons.</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -4119,64 +4115,64 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>First-principles LES and DNS of supercritical combustion, rotating detonation engine (RDE) wave dynamics, and LOX/CH4 propellant injection physics -- resolving real-fluid thermodynamic non-idealities and turbulence-chemistry coupling at rocket-engine operating pressures.</t>
+          <t>Supersonic combustion dynamics in dual-combustion ramjet (DCR) engines, chemical explosive mode analysis (CEMA), and detonative tangential combustion instability mode transitions in liquid and gas rocket combustors.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>LES (real-fluid EOS, cubic Peng-Robinson EOS), DNS of supercritical jets, Modified Benedict-Webb-Rubin (MBWR) EOS, Finite-rate GRI-Mech 3.0 chemistry, RDE wave solvers</t>
+          <t>Chemical Explosive Mode Analysis (CEMA), STFT / Dynamic Mode Decomposition (DMD), Proper Orthogonal Decomposition (POD), Compressible reacting LES, High-order shock-capturing CFD</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Rotating detonation engine with a hollow annular channel: Effects of inlet geometry on wave dynamics</t>
+          <t>Supersonic Combustion and Flow Evolution in Dual-Combustion Ramjet Engine</t>
         </is>
       </c>
       <c r="P3" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2021.111763", "https://doi.org/10.1016/j.combustflame.2021.111763")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.b40184", "https://doi.org/10.2514/1.b40184")</f>
         <v/>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>performing 3D LES with finite-rate H2-O2 kinetics in a hollow annular RDE, demonstrating that inlet slot aspect ratio controls reactant layer thickness and shifts rotating detonation wave speed between 1820 and 2240 m/s, altering wave deficit by up to 15.4% from Chapman-Jouguet.</t>
+          <t>conducting numerical experiments of supersonic combustion in a DCR engine using CEMA and Damkohler number analysis, demonstrating that thermal choking establishes a thermal throat in the constant-area section and elevates pressure, temperature, and nozzle exit Mach number.</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>The rotating detonation engine (RDE) with a hollow annular channel is investigated using 3D LES with detailed H2-O2 kinetics. Slot aspect ratio variations of 1:4 to 4:1 produce wave speeds ranging from 1820 to 2240 m/s, with wave deficits from 8.2% to 15.4% relative to the idealized Chapman-Jouguet value. Inlet geometry controls the freshly mixed reactant layer thickness ahead of the detonation wave, directly setting wave speed and heat release peak.</t>
+          <t>This work presents a numerical investigation of supersonic combustion dynamics and flow evolution in a dual-combustion ramjet (DCR) engine. Two series of parametric numerical experiments were conducted for the DCR combustor configuration by varying the length of the constant-area section [Formula: see text] and the divergence angle [Formula: see text] of the expansion section. The operating conditions were selected to mimic realistic flight scenarios. Two distinct combustion modes were identified, based on the occurrence of thermal choking. To analyze the combustion characteristics of these modes, chemical explosive mode analysis was performed, along with an evaluation of the Damköhler number. In the thermally choked combustion mode, both pressure and temperature were significantly elevated compared to the supersonic shear-layer combustion mode. This increase is attributed to the coupling between pressure and heat release, which enhances combustion efficiency. A thermal throat forms at the end of the constant-area section, while the divergent section functions as a supersonic nozzle. The exit Mach number in thermally choked cases is higher than its counterpart in supersonic shea...</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>Supercritical cryogenic LOX/GH2 combustion in a single-element shear-coaxial injector</t>
+          <t>Resonant phenomena in detonative tangential combustion instability in a rocket combustor</t>
         </is>
       </c>
       <c r="T3" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.B38219", "https://doi.org/10.2514/1.B38219")</f>
+        <f>HYPERLINK("https://doi.org/10.1063/5.0268442", "https://doi.org/10.1063/5.0268442")</f>
         <v/>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>conducting LES with MBWR real-fluid EOS in a LOX/GH2 shear-coaxial injector at 6-12 MPa, demonstrating that transcritical injection eliminates surface tension, produces high-density oxygen fingers in hydrogen coflow, and increases flame standoff length by 38% with rising chamber pressure.</t>
+          <t>applying STFT, DMD, and POD spectral decomposition to detonative tangential combustion instability in a rocket combustor, demonstrating that limit-cycle instabilities originate from thermofluidic wave resonance rather than pure acoustic natural frequencies and exhibit characteristic frequency-shifting harmonics.</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>Supercritical cryogenic LOX/GH2 combustion in a shear-coaxial injector at 6-12 MPa is investigated using LES with MBWR real-fluid EOS. LES reveals that above the critical point, continuous fluid mixing eliminates surface tension and produces high-density LOX fingers that stretch into hydrogen coflow. Flame standoff length increases by 38% as chamber pressure rises from 6 to 12 MPa.</t>
+          <t>In addition to investigating the flow field of detonative tangential combustion instability [Sung, B.-K., Kasahara, J., and Choi, J.-Y., Combust. Flame 275 114092 (2025)], spectral analysis was performed using Short-time Fourier Transform (STFT), Dynamic Mode Decomposition (DMD), and Proper Orthogonal Decomposition (POD) to gain a deeper understanding of the instability modes. By comparing the limit-cycle frequencies with the acoustic natural frequencies, it was confirmed that the detonative tangential combustion instability cannot be analyzed solely based on natural frequencies, as it corresponds to thermofluidic phenomena rather than thermoacoustic instability. The STFT provided time-dependent frequencies and revealed a frequency shift phenomenon during instability mode transitions. Using DMD, the corresponding dominant mode shapes were identified. The POD analysis corroborated the DMD results, and by examining the eigenvectors of the energetic POD modes, the mode undergoing the frequency shift was identified. During limit cycle operation, frequency harmonics emerged as the frequencies of each mode became integer multiples of the most energetic mode, further indicating that de...</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>1. Rotating detonation engine hollow annular channel: Effects of inlet geometry on wave dynamics (Combustion and Flame, 2022) | 2. Supercritical cryogenic LOX/GH2 combustion in a single-element shear-coaxial injector (JPP, 2021)</t>
+          <t>1. Supersonic Combustion and Flow Evolution in Dual-Combustion Ramjet Engine (Journal of Propulsion and Power, 2025) | 2. Resonant phenomena in detonative tangential combustion instability in a rocket combustor (Physics of Fluids, 2025)</t>
         </is>
       </c>
       <c r="X3" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2021.111763 | https://doi.org/10.2514/1.B38219", "https://doi.org/10.1016/j.combustflame.2021.111763 | https://doi.org/10.2514/1.B38219")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.b40184 | https://doi.org/10.1063/5.0268442", "https://doi.org/10.2514/1.b40184 | https://doi.org/10.1063/5.0268442")</f>
         <v/>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>performing 3D LES with finite-rate H2-O2 kinetics in a hollow annular RDE, demonstrating that inlet slot aspect ratio controls reactant layer thickness and shifts rotating detonation wave speed between 1820 and 2240 m/s, altering wave deficit by up to 15.4% from Chapman-Jouguet.</t>
+          <t>conducting numerical experiments of supersonic combustion in a DCR engine using CEMA and Damkohler number analysis, demonstrating that thermal choking establishes a thermal throat in the constant-area section and elevates pressure, temperature, and nozzle exit Mach number.</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
@@ -4319,64 +4315,64 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Simultaneous high-speed 3D laser diagnostics -- tomographic PIV, dual-pump CARS thermometry, and kHz OH-PLIF -- to map turbulence-chemistry interactions, flame kernel growth, and thermoacoustic feedback in swirl-stabilized gas-turbine combustors.</t>
+          <t>High-speed laser diagnostics for high-pressure turbulent reacting flows, ducted fuel injection (DFI) soot mitigation, and lean blowoff stability mechanisms in lean premixed prevaporized (LPP) supersonic transport combustors.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Dual-pump CARS (N2/O2 thermometry), High-speed stereoscopic PIV, kHz OH-PLIF, Tomographic PIV, High-speed Schlieren</t>
+          <t>Filtered Rayleigh Scattering (FRS), High-speed PIV/PLIF, Ducted Fuel Injection (DFI), Optical high-pressure combustor rigs (700 K, 9 bar), Laser extinction soot diagnostics</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Experimental investigation of turbulence-chemistry interaction in a gas turbine model combustor using simultaneous high-speed CARS and PIV</t>
+          <t>Impact of pilot injections on ducted fuel injection performance</t>
         </is>
       </c>
       <c r="P4" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2023.112754", "https://doi.org/10.1016/j.combustflame.2023.112754")</f>
+        <f>HYPERLINK("https://doi.org/10.1177/14680874261426780", "https://doi.org/10.1177/14680874261426780")</f>
         <v/>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>deploying simultaneous 5 kHz dual-pump CARS and stereo-PIV in a swirl combustor, demonstrating that local extinction events co-locate with strain-rate regions where Ka &gt; 50 and that re-ignition traces preferentially the trailing edges of high-scalar-dissipation tubes.</t>
+          <t>investigating the coupling of ducted fuel injection (DFI) with pilot injections in high-pressure diesel combustion, demonstrating that DFI reduces flame spatially integrated natural luminosity (SINL) by 30-70% and pilot injection mitigates peak SINL by a further 16%.</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>Simultaneous dual-pump CARS thermometry and stereoscopic PIV measurements at 5 kHz are applied to characterize turbulence-chemistry interaction in a gas turbine model combustor under atmospheric and elevated pressure conditions. Results demonstrate strongly non-equilibrium scalar mixing in the flame brush: local extinction events co-locate with high-strain-rate regions where turbulent Karlovitz numbers exceed Ka = 50, while re-ignition preferentially occurs at the trailing edges of high-scalar-dissipation tubes, indicating that distributed reaction zones operate transiently in thin-flame mode.</t>
+          <t>This experimental and numerical study evaluates how ducted fuel injection (DFI) and pilot injections interact to impact soot formation and the premixed heat release pressure spike in diesel combustion. Experiments showed that pilot injections reduced the premixed heat release spike of a free spray by approximately 70%, while DFI configurations only experienced a decrease of approximately 25%. Similarly, pilot injections reduced the initial lift-off length (LOL) of the main injection of a free-spray by approximately 30%, while DFI’s initial LOL had little to no change when pilot injections were utilized. Regardless of whether a standalone-main or pilot-main strategy was used, DFI was able to reduce the spatially integrated natural luminosity (SINL) of the flame relative to a free spray, indicating a likely reduction in soot formation. Both duct configurations studied produced steady SINL signals which were approximately 30% and 70% of the free-spray’s, respectively. For DFI, pilot injections further reduced the peak SINL compared to a standalone main by approximately 16%. The decrease in peak SINL correlated with increased spray head penetration rates. The numerical study reveale...</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>Simultaneous high-speed OH-PLIF and stereoscopic PIV of turbulent premixed flames at elevated pressure</t>
+          <t>Lean Blowoff Limits and Emissions Measurements in a Lean Premixed Prevaporized Combustor with Variable Reactant Inhomogeneity</t>
         </is>
       </c>
       <c r="T4" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.proci.2020.06.149", "https://doi.org/10.1016/j.proci.2020.06.149")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0384", "https://doi.org/10.2514/6.2026-0384")</f>
         <v/>
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>conducting simultaneous kHz OH-PLIF and SPIV across 1-5 atm in a swirl combustor, demonstrating that elevated pressure compresses the reaction layer and increases mean tangential strain rates by 3.2x while transitioning flame-wrinkling from Ka-dominated to curvature-dominated kinematic regimes.</t>
+          <t>characterizing lean blowoff (LBO) limits and emissions in an LPP combustor operating at 700 K and 9 bar on Jet A and SAF, demonstrating that moderate prevaporization and premixing are required to anchor main flames and curb NOx emission spikes.</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>Simultaneous kHz-rate OH-PLIF and SPIV measurements were performed in turbulent premixed swirling flames at elevated pressures up to 5 atm. Elevated pressure compresses the reaction layer, increases Damkohler number, and transitions flame-wrinkling dynamics from Ka-dominated to curvature-dominated modes. Strain-rate statistics at 5 atm show that global mean tangential strain rates increase by a factor of 3.2 relative to atmospheric cases.</t>
+          <t>Lean premixed prevaporized (LPP) combustor designs and sustainable aviation fuels (SAF) show great promise for the development of next-generation low-emission civil supersonic transport (CST) aircraft engines. In this work, exhaust emissions sampling and optical diagnostic measurements were conducted in an LPP model combustor with variable reactant inhomogeneity. The LPP combustor features a novel premixer design, which facilitates control of the level of fuel vaporization and fuel-air mixedness entering the combustor. Measurements of lean blowoff (LBO) limits and gaseous emissions trends were obtained through the optically accessible combustor liner and custom exhaust sampling probe. The combustor was operated at elevated temperature (700 K) and pressure (9 bar) conditions to simulate the combustor inlet conditions of CST aircraft engines. A conventional Jet A fuel was used as the baseline fuel, to which a SAF was compared. Results show that a moderate level of prevaporization and premixing was sufficient to properly stabilize the premixed main flames. With reduced prevaporization and premixing, the main flames did not properly stabilize and NOx emissions were increased. With i...</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>1. Turbulence-chemistry interaction in a GT model combustor via simultaneous high-speed CARS and PIV (Combustion and Flame, 2023) | 2. Simultaneous high-speed OH-PLIF and stereo-PIV of turbulent premixed flames at elevated pressure (Proc. Combustion Institute, 2021)</t>
+          <t>1. Impact of pilot injections on ducted fuel injection performance (International Journal of Engine Research, 2026) | 2. Lean Blowoff Limits and Emissions Measurements in a Lean Premixed Prevaporized Combustor with Variable Reactant Inhomogeneity (2026)</t>
         </is>
       </c>
       <c r="X4" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2023.112754 | https://doi.org/10.1016/j.proci.2020.06.149", "https://doi.org/10.1016/j.combustflame.2023.112754 | https://doi.org/10.1016/j.proci.2020.06.149")</f>
+        <f>HYPERLINK("https://doi.org/10.1177/14680874261426780 | https://doi.org/10.2514/6.2026-0384", "https://doi.org/10.1177/14680874261426780 | https://doi.org/10.2514/6.2026-0384")</f>
         <v/>
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>deploying simultaneous 5 kHz dual-pump CARS and stereo-PIV in a swirl combustor, demonstrating that local extinction events co-locate with strain-rate regions where Ka &gt; 50 and that re-ignition traces preferentially the trailing edges of high-scalar-dissipation tubes.</t>
+          <t>investigating the coupling of ducted fuel injection (DFI) with pilot injections in high-pressure diesel combustion, demonstrating that DFI reduces flame spatially integrated natural luminosity (SINL) by 30-70% and pilot injection mitigates peak SINL by a further 16%.</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr">
@@ -4519,64 +4515,64 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Quantitative laser diagnostics for high-enthalpy reacting flows -- PLIF-based scalar measurements, dual-pump CARS thermometry, and two-photon LIF for atomic species in high-pressure combustion, shock tunnels, and detonation chambers.</t>
+          <t>Advanced planar laser-induced fluorescence (PLIF) diagnostics for elevated-pressure reacting flows, lean blowoff proximity sensing, and multi-species optical imaging in swirl-stabilized spray flames.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Planar Laser-Induced Fluorescence (PLIF), Dual-pump CARS, Two-photon atomic LIF, High-speed intensified CCD, Shock tube/detonation chamber diagnostics</t>
+          <t>Single-laser CH/OH/fuel PLIF, Longpass intra-vibrational band optical filtering, High-pressure combustor rigs (9 bar), Lean blowout acoustic/optical sensing</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Quantitative PLIF imaging of OH* chemiluminescence in detonation-driven flows</t>
+          <t>Lean Blowoff Limits and Emissions Measurements in a Lean Premixed Prevaporized Combustor with Variable Reactant Inhomogeneity</t>
         </is>
       </c>
       <c r="P5" s="3">
-        <f>HYPERLINK("https://doi.org/10.1088/1361-6501/ac4b21", "https://doi.org/10.1088/1361-6501/ac4b21")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0384", "https://doi.org/10.2514/6.2026-0384")</f>
         <v/>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>applying quantitative OH* PLIF with dual-pump CARS quenching correction behind H2-air detonation fronts, demonstrating that post-detonation OH* overshoots equilibrium concentration by 2.3x due to ZND induction-zone kinetic excess, fully resolved at 200 um spatial resolution.</t>
+          <t>evaluating lean blowoff limits and emissions in an LPP combustor operating at 700 K and 9 bar under variable reactant inhomogeneity, demonstrating that prevaporization uniformity dictates flame stabilization and prevents severe NOx emission surges.</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>A quantitative PLIF diagnostic for excited-state OH* is developed and applied to detonation-driven supersonic combustion flows. The diagnostic accounts for collisional quenching corrections using simultaneous dual-pump CARS measurements. Applied to a H2-air detonation tube, OH* PLIF images resolve the thin reaction zone behind the detonation front with 200 um spatial resolution. OH* signal peaks at 2.3x the equilibrium post-detonation value, indicating strong kinetic overshoot driven by ZND induction zone chemistry.</t>
+          <t>Lean premixed prevaporized (LPP) combustor designs and sustainable aviation fuels (SAF) show great promise for the development of next-generation low-emission civil supersonic transport (CST) aircraft engines. In this work, exhaust emissions sampling and optical diagnostic measurements were conducted in an LPP model combustor with variable reactant inhomogeneity. The LPP combustor features a novel premixer design, which facilitates control of the level of fuel vaporization and fuel-air mixedness entering the combustor. Measurements of lean blowoff (LBO) limits and gaseous emissions trends were obtained through the optically accessible combustor liner and custom exhaust sampling probe. The combustor was operated at elevated temperature (700 K) and pressure (9 bar) conditions to simulate the combustor inlet conditions of CST aircraft engines. A conventional Jet A fuel was used as the baseline fuel, to which a SAF was compared. Results show that a moderate level of prevaporization and premixing was sufficient to properly stabilize the premixed main flames. With reduced prevaporization and premixing, the main flames did not properly stabilize and NOx emissions were increased. With i...</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>Two-temperature analysis of non-equilibrium N2 vibrational excitation in hypersonic arcjet flows</t>
+          <t>Single-laser CH, OH and fuel PLIF in a pressurized swirl-stabilized spray flame</t>
         </is>
       </c>
       <c r="T5" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.T6072", "https://doi.org/10.2514/1.T6072")</f>
+        <f>HYPERLINK("https://doi.org/10.1016/j.proci.2026.106104", "https://doi.org/10.1016/j.proci.2026.106104")</f>
         <v/>
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>measuring two-photon LIF vibrational temperatures across a Mach 5-7 arcjet freestream, demonstrating N2 vibrational temperatures exceed translational by 1800-2400 K and Park finite-rate model under-predicts vibrational relaxation in the expansion fan by 28%.</t>
+          <t>demonstrating single-laser simultaneous CH, OH, and fuel PLIF in a pressurized swirl-stabilized spray flame at 310.7 nm, revealing that pressure-induced collisional broadening allows clean separation of thin CH reaction zones from dense liquid spray droplet fluorescence.</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>Non-equilibrium vibrational excitation of N2 in a high-enthalpy arcjet flow simulating Mars entry conditions is investigated using two-photon LIF and optical emission spectroscopy. Measured vibrational temperatures exceed translational temperatures by 1800-2400 K across Mach 5-7 test conditions. Agreement with LAURA CFD predictions using Park rate model is within 12% in the freestream but degrades to 28% in the expansion fan region.</t>
+          <t>This paper explores the use of planar laser-induced fluorescence (PLIF) with excitation wavelengths in the R-branch of the CH C 2 Σ + − X 2 Π ( 0,0 ) in a liquid-fueled combustor at elevated pressures. Following the atmospheric pressure work of Hammack et al. Appl. Phys. B 124:34 (2018), longpass intra-vibrational band filtering was used to isolate CH PLIF, OH PLIF, and fuel signals from the laser scattering. CH PLIF images were obtained by targeting CH R-branch transitions at 310.69 nm and 311.18 nm. Interference from fuel fluorescence was mitigated through the use of a low-aromatic content synthetic aviation fuel, though it was still significant where liquid was present. Nevertheless, the CH layers in the reaction zone were distinguishable from the droplet signal even in the dense spray near the fuel injector. OH PLIF images could be obtained without CH interference using the same setup, but targeting the OH Q-branch transitions of the A − X ( 0,0 ) band at 310.75 nm. Furthermore, due to pressure-induced collisional broadening, simultaneous CH and OH PLIF could be imaged on a single frame when the laser wavelength was tuned in the vicinity of either CH R-branch transition. The...</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>1. Quantitative PLIF imaging of OH* chemiluminescence in detonation-driven flows (MST, 2022) | 2. Two-temperature analysis of non-equilibrium N2 in hypersonic arcjet flows (JTHT, 2021)</t>
+          <t>1. Lean Blowoff Limits and Emissions Measurements in a Lean Premixed Prevaporized Combustor with Variable Reactant Inhomogeneity (2026) | 2. Single-laser CH, OH and fuel PLIF in a pressurized swirl-stabilized spray flame (Proceedings of the Combustion Institute, 2026)</t>
         </is>
       </c>
       <c r="X5" s="3">
-        <f>HYPERLINK("https://doi.org/10.1088/1361-6501/ac4b21 | https://doi.org/10.2514/1.T6072", "https://doi.org/10.1088/1361-6501/ac4b21 | https://doi.org/10.2514/1.T6072")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0384 | https://doi.org/10.1016/j.proci.2026.106104", "https://doi.org/10.2514/6.2026-0384 | https://doi.org/10.1016/j.proci.2026.106104")</f>
         <v/>
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>applying quantitative OH* PLIF with dual-pump CARS quenching correction behind H2-air detonation fronts, demonstrating that post-detonation OH* overshoots equilibrium concentration by 2.3x due to ZND induction-zone kinetic excess, fully resolved at 200 um spatial resolution.</t>
+          <t>evaluating lean blowoff limits and emissions in an LPP combustor operating at 700 K and 9 bar under variable reactant inhomogeneity, demonstrating that prevaporization uniformity dictates flame stabilization and prevents severe NOx emission surges.</t>
         </is>
       </c>
       <c r="Z5" s="2" t="inlineStr">
@@ -4719,64 +4715,64 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>High-fidelity RANS/hybrid RANS-LES aeromechanics simulation of helicopter rotors and wind turbines -- capturing dynamic stall vortex shedding, rotor-wake interaction, and blade-vortex interaction noise to reduce vibration and acoustic emissions in next-generation rotorcraft.</t>
+          <t>Aeroacoustics DNS of high-amplitude acoustic transmission and inverse airfoil design for roughness-tolerant low-drag wind and hydrokinetic turbine blades.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Hybrid RANS-LES (DDES), Overset Chimera grids, Dynamic mesh motion, CAMRAD II structural coupling, Gradient boosted trees (dynamic stall onset ML)</t>
+          <t>Direct Numerical Simulation (DNS) aeroacoustics, Impedance tube testing (120-150 dB), Inverse airfoil aerodynamic design, Blade Element Momentum (BEM) turbine codes</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Dynamic Stall Onset Prediction and Modeling Using Machine Learning on CFD-Generated Datasets</t>
+          <t>Transmission of high-amplitude sound through leakages of ill-fitting earplugs</t>
         </is>
       </c>
       <c r="P6" s="3">
-        <f>HYPERLINK("https://doi.org/10.4050/JAHS.68.032001", "https://doi.org/10.4050/JAHS.68.032001")</f>
+        <f>HYPERLINK("https://doi.org/10.1177/1475472x261473636", "https://doi.org/10.1177/1475472x261473636")</f>
         <v/>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>training gradient-boosted classifiers on 4.1M URANS time steps across 15,000 airfoil conditions, demonstrating 94.2% accuracy in predicting dynamic stall onset 3 convective time units in advance and reducing full-rotor vibration estimation error from 31% to 9%.</t>
+          <t>combining impedance-tube experiments with DNS of high-amplitude acoustic transmission (120-150 dB) across 1-5 kHz, demonstrating that ill-fitting earplug leakages reduce transmission loss by ~18 dB at 120 dB incident SPL.</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>Machine learning models trained on 4.1 million time steps from URANS simulations across 15,000 operating conditions achieve 94.2% accuracy in predicting dynamic stall onset 3 convective time units in advance. The ML-based predictor integrated into a blade element momentum model reduces dynamic stall-induced vibration estimation error from 31% to 9% relative to pure BEMT.</t>
+          <t>Exposure to high sound pressure levels (SPL) is a leading cause of noiseinduced hearing loss, and earplugs are a primary means of protection. The effectiveness of earplug protection depends on the seal formed in the ear canal. An ill-fitting earplug leaves air gaps that leak sound and degrade attenuation. The acoustics of these leak paths and their dissipation mechanisms under high-amplitude sound remain poorly characterized. This study quantifies sound transmission through modeled earplug leakage with rigid-wall idealization and identifies the governing dissipation mechanisms by combining impedance-tube experiments and direct numerical simulation (DNS). The methods were first verified against stand-alone slit resonators and orifices, for which extensive published data are available, and then used to measure the transmission loss (TL) and acoustic power absorption coefficient of modeled earplug–canal configurations over 1–5 kHz at overall incident SPLs of 120–150 dB. Leakage from an ill-fitting silicone rubber earplug reduced its TL by approximately 18 dB relative to a sealed configuration at an overall incident sound pressure levels (OISPL) of 120 dB, and the leakage-path TL in...</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>Computational Investigation of Rotor-Fuselage Interactional Aerodynamics Using Hybrid RANS-LES</t>
+          <t>Design and Use of Roughness-Tolerant Low Drag Airfoils for Wind Turbine and Hydrokinetic Turbine Applications</t>
         </is>
       </c>
       <c r="T6" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.J060183", "https://doi.org/10.2514/1.J060183")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0480", "https://doi.org/10.2514/6.2026-0480")</f>
         <v/>
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>simulating rotor-fuselage interactional aerodynamics via DDES on overset grids at advance ratio mu = 0.15, demonstrating that recirculation below the hub increases rotor torque by 4.7% and produces wake-fuselage surface pressure fluctuations of 0.08 Cp matching experimental data.</t>
+          <t>applying inverse design to develop roughness-tolerant airfoils with laminar drag buckets across wide lift coefficients, demonstrating preserved profile efficiency under surface dirt and icing degradation in wind and tidal turbines.</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>The interactional aerodynamics between a helicopter main rotor and fuselage is investigated using DDES on overset grids. Rotor-fuselage interaction produces a recirculation region below the hub that increases rotor torque requirement by 4.7%. Unsteady wake-fuselage impingement creates surface pressure fluctuations of 0.08 Cp, consistent with Georgia Tech Aeroflite wind tunnel measurements.</t>
+          <t>Wind turbines and hydrokinetic turbines are designed to use laminar airfoils that provide maximum power at the rated speed. During day-to-day operations, the blade surface may be degraded due to accumulation of dirt and icing on the pressure side, in addition to development of scratches or other surface imperfections. As a result, the profile power losses would increase, reducing the available power over a broad range of operating conditions. In this work, an inverse design approach has been employed to generate roughness tolerant airfoils that exhibit a laminar drag bucket for a broad range of lift coefficients. Two-dimensional drag polars are presented for smooth and rough airfoils and compared to NACA airfoils of comparable thickness. A limited number of three-dimensional studies based on combined blade element-momentum theory are also presented for several wind and tidal turbines for a broad range of rated power conditions.</t>
         </is>
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>1. Dynamic Stall Onset Prediction Using Machine Learning on CFD Datasets (JAHS, 2023) | 2. Computational Investigation of Rotor-Fuselage Interactional Aerodynamics Using Hybrid RANS-LES (AIAA J., 2021)</t>
+          <t>1. Transmission of high-amplitude sound through leakages of ill-fitting earplugs (International Journal of Aeroacoustics, 2026) | 2. Design and Use of Roughness-Tolerant Low Drag Airfoils for Wind Turbine and Hydrokinetic Turbine Applications (2026)</t>
         </is>
       </c>
       <c r="X6" s="3">
-        <f>HYPERLINK("https://doi.org/10.4050/JAHS.68.032001 | https://doi.org/10.2514/1.J060183", "https://doi.org/10.4050/JAHS.68.032001 | https://doi.org/10.2514/1.J060183")</f>
+        <f>HYPERLINK("https://doi.org/10.1177/1475472x261473636 | https://doi.org/10.2514/6.2026-0480", "https://doi.org/10.1177/1475472x261473636 | https://doi.org/10.2514/6.2026-0480")</f>
         <v/>
       </c>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>training gradient-boosted classifiers on 4.1M URANS time steps across 15,000 airfoil conditions, demonstrating 94.2% accuracy in predicting dynamic stall onset 3 convective time units in advance and reducing full-rotor vibration estimation error from 31% to 9%.</t>
+          <t>combining impedance-tube experiments with DNS of high-amplitude acoustic transmission (120-150 dB) across 1-5 kHz, demonstrating that ill-fitting earplug leakages reduce transmission loss by ~18 dB at 120 dB incident SPL.</t>
         </is>
       </c>
       <c r="Z6" s="2" t="inlineStr">
@@ -4919,64 +4915,64 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Hall-effect thruster plume physics, near-anode ionization instabilities, and plasma-neutral coupling in electric propulsion -- combining laser-induced fluorescence velocimetry, Langmuir probe arrays, and particle-in-cell simulations to push CubeSat and deep-space thruster efficiency boundaries.</t>
+          <t>Hall-effect thruster plasma physics, heaterless hollow cathode operation on alternative propellants (krypton/argon), and laser Thomson scattering electron dynamics in magnetically shielded thrusters.</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Laser-Induced Fluorescence (LIF) velocimetry (Xe II lines), Langmuir and Faraday probes, Retarding Potential Analyzer (RPA), E×B probe, Particle-in-Cell (PIC) simulations</t>
+          <t>Laser Thomson Scattering, Steady-state I-V cathode characterization, Magnetically shielded Hall thruster testing (H9 9 kW), Vacuum Test Facilities (VTF-2)</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Azimuthal Ion Velocity Measurements in a Hall Thruster via Laser-Induced Fluorescence</t>
+          <t>Characterization of a heaterless 60 A hollow cathode on krypton and argon</t>
         </is>
       </c>
       <c r="P7" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.B38688", "https://doi.org/10.2514/1.B38688")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s44205-026-00221-w", "https://doi.org/10.1007/s44205-026-00221-w")</f>
         <v/>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>measuring azimuthal Xe II ion velocities via dual-geometry LIF in a Hall thruster near-field plume, demonstrating that azimuthal swirl reaches 2.1-3.8 km/s (11-19% of exit velocity) and correlates with 15-20 kHz breathing mode oscillations that reduce effective specific impulse.</t>
+          <t>characterizing a 60 A heaterless hollow cathode on krypton and argon in the 9 kW H9 thruster, demonstrating that magnetic fields systematically increase steady-state discharge voltage by up to +159% (+67.5 V) on argon at fixed current rather than reducing it.</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>Azimuthal ion velocity measurements in the near-field plume of a Hall-effect thruster are reported using LIF velocimetry of Xe II lines. Peak swirl velocities of 2.1-3.8 km/s correspond to 11-19% of total ion exit velocity. These azimuthal components correlate with low-frequency breathing mode oscillations at 15-20 kHz and indicate non-trivial angular momentum deposition that degrades effective thruster specific impulse.</t>
+          <t>Abstract We present a steady-state current-voltage (IV) characterization of a heaterless version of the 9 kW-class H9 Hall thruster cathode. This work was conducted at Georgia Tech’s High-Power Electric Propulsion Laboratory (HPEPL) at operational background pressures of 0.22–0.70 µTorr on krypton and 0.11–0.24 µTorr on argon, with a base pressure of 9.1 × 10 − 8 Torr. The characterization mapped steady-state voltage behavior from 5 to 45 A of discharge current on krypton and 5 to 30 A on argon (with paired magnetized and unmagnetized data over 5 to 35 A on krypton and 5 to 20 A on argon), in both magnetized and unmagnetized configurations. The magnetized configuration produced a higher discharge voltage than the unmagnetized configuration at every paired (current, flow) operating point on both propellants. On krypton, the magnetized-unmagnetized voltage gap ranged from near zero at the highest cathode flow and lowest current to + 39.6 V (+ 148%) at 30 A and 12.39 sccm. On argon, the gap ranged from + 6.0 V at 15 A and 12.39 sccm to + 67.5 V (+ 159%) at 20 A and 15.89 sccm. In both cases, the gap widened with discharge current and narrowed with cathode flow. These results verify reproducible ignition at every tested flow rate, confirm uninterrupted steady-state heaterless operation on krypton and argon, and quantify how the applied magnetic field shifts the steady-state operating point at fixed discharge current. The key finding is that the applied magnetic field increases the steady-state discharge voltage at fixed current rather than reducing it, and the effect is systematically larger on argon than on krypton at matched operating conditions.</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>Near-Field Plume Characterization of a 200-W Hall Thruster via Electrostatic Probes</t>
+          <t>Effect of body bias on near-field electron behavior in a magnetically shielded Hall thruster</t>
         </is>
       </c>
       <c r="T7" s="3">
-        <f>HYPERLINK("https://doi.org/10.1007/s44205-023-00045-z", "https://doi.org/10.1007/s44205-023-00045-z")</f>
+        <f>HYPERLINK("https://doi.org/10.1063/5.0340395", "https://doi.org/10.1063/5.0340395")</f>
         <v/>
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>deploying 2D electrostatic probe arrays in a 200-W Hall thruster near-field plume, demonstrating that bimodal IEDFs at 5 cm downstream directly evidence charge-exchange collisions that broaden plume divergence by 6.8 degrees beyond the accelerated-ion beam.</t>
+          <t>deploying spatially resolved laser Thomson scattering in the near-field of the 9 kW H9 Hall thruster at 40 A, demonstrating that +2 V body bias inverts electron density topology between the cathode centerline (3.4e19 m^-3) and channel centerline (9.0e17 m^-3).</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>A comprehensive electrostatic probe characterization of the near-field plume of a 200-W Hall thruster is reported. The IEDF at 5 cm downstream reveals a bimodal structure with a cold (&lt;10 eV) charge-exchange peak and a hot (120-180 eV) direct-acceleration peak, providing direct evidence for near-field charge exchange collisions that broaden plume divergence by 6.8 degrees.</t>
+          <t>This work investigates the influence of thruster body bias on near-field electron behavior in a magnetically shielded Hall effect thruster (HET) through spatially resolved laser Thomson scattering diagnostics. Experiments were conducted on the 9 kW class H9 magnetically shielded HET operating at 40 A discharge current and 150 V discharge voltage on krypton propellant in the Georgia Tech Vacuum Test Facility 2. Three electrical configurations were examined: floating (body electrically isolated), cathode-tied (body at cathode potential, approximately −10.3 V relative to facility ground), and +2 V bias (body biased +2 V relative to ground). Spatially resolved measurements of electron density, electron temperature, and radial electron bulk velocity were obtained at up to 23 locations (a 15-point radial grid and up to eight axial stations along the cathode centerline) spanning the cathode near-field from the cathode centerline to the discharge channel centerline. A configuration-dependent spatial density inversion reveals distinct circuit topologies: at z/r0 = 0.029, cathode-tied elevates ne at the cathode centerline (4.4 × 1019 m−3) while exhibiting the lowest channel-centerline density (6.6 × 1017 m−3), whereas the +2 V configuration shows the opposite pattern (3.4 × 1019 and 9.0 × 1017 m−3, respectively). The +2 V configuration exhibits the lowest Te at the inner front pole cover, consistent with magnetization-limited, energy-selective electron collection. Electron pressure does not serve as a reliable proxy for electrostatic potential in this near-field region due to unmeasured anomalous transport terms.</t>
         </is>
       </c>
       <c r="W7" s="2" t="inlineStr">
         <is>
-          <t>1. Azimuthal Ion Velocity Measurements in a Hall Thruster via Laser-Induced Fluorescence (JPP, 2022) | 2. Near-Field Plume Characterization of a 200-W Hall Thruster via Electrostatic Probes (JEP, 2023)</t>
+          <t>1. Characterization of a heaterless 60 A hollow cathode on krypton and argon (Journal of Electric Propulsion, 2026) | 2. Effect of body bias on near-field electron behavior in a magnetically shielded Hall thruster (Journal of Applied Physics, 2026)</t>
         </is>
       </c>
       <c r="X7" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.B38688 | https://doi.org/10.1007/s44205-023-00045-z", "https://doi.org/10.2514/1.B38688 | https://doi.org/10.1007/s44205-023-00045-z")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s44205-026-00221-w | https://doi.org/10.1063/5.0340395", "https://doi.org/10.1007/s44205-026-00221-w | https://doi.org/10.1063/5.0340395")</f>
         <v/>
       </c>
       <c r="Y7" s="2" t="inlineStr">
         <is>
-          <t>measuring azimuthal Xe II ion velocities via dual-geometry LIF in a Hall thruster near-field plume, demonstrating that azimuthal swirl reaches 2.1-3.8 km/s (11-19% of exit velocity) and correlates with 15-20 kHz breathing mode oscillations that reduce effective specific impulse.</t>
+          <t>characterizing a 60 A heaterless hollow cathode on krypton and argon in the 9 kW H9 thruster, demonstrating that magnetic fields systematically increase steady-state discharge voltage by up to +159% (+67.5 V) on argon at fixed current rather than reducing it.</t>
         </is>
       </c>
       <c r="Z7" s="2" t="inlineStr">
@@ -5103,64 +5099,64 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>LES-driven combustion instability modeling, turbulent premixed flame propagation, and plasma-assisted ignition in gas-turbine and scramjet combustors — advancing high-fidelity reacting-flow simulation from laboratory-scale flames to full annular combustion chambers.</t>
+          <t>Large eddy simulations (LES) of turbulent combustion, hybrid transported-tabulated chemistry (HTTC), and soot aerosol dynamics in rich-burn quick-mix lean-burn (RQL) and rotating detonation combustors.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Large Eddy Simulation (LES) with LDK subgrid closure, PRISM tabulated chemistry, Spray Lagrangian tracking, DNS of premixed flame kernels</t>
+          <t>Large Eddy Simulation (LES), Hybrid Transported-Tabulated Chemistry (HTTC), Dynamic subgrid closures, PAH-based soot modeling, Partially stirred reactor (PaSR)</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Subgrid combustion modeling for large eddy simulation of spray combustion in turbulent swirling flows</t>
+          <t>Application of Hybrid Transported-Tabulated Chemistry for Efficient Large-Eddy Simulation of Turbulent Combustion</t>
         </is>
       </c>
       <c r="P8" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2021.111634", "https://doi.org/10.1016/j.combustflame.2021.111634")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s10494-026-00794-4", "https://doi.org/10.1007/s10494-026-00794-4")</f>
         <v/>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>coupling Lagrangian spray dynamics with LES dynamic subgrid combustion in a bluff-body swirl combustor, demonstrating that droplet evaporation controls inner-recirculation-zone flame anchoring and produces unsteady heat-release fluctuations at Strouhal numbers consistent with observed thermoacoustic instabilities.</t>
+          <t>implementing a hybrid transported-tabulated chemistry (HTTC) strategy in LES of turbulent combustion with 29 species and 141 steps, demonstrating up to 11-fold computational speedup while maintaining high fidelity in predicting extinction and re-ignition dynamics.</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>A subgrid combustion model for large eddy simulation of spray combustion in turbulent swirling flows is developed and validated. The model is based on the localized dynamic K-equation (LDK) subgrid kinetic energy closure combined with a progress variable approach for turbulent premixed combustion. Two-phase spray effects are modeled using a Lagrangian particle tracking approach coupled to the LES gas-phase solver. The combined model is applied to a bluff-body stabilized swirl combustor and validated against experimental measurements of velocity, temperature, and species concentrations. Simulations reveal that liquid fuel droplet evaporation and transport profoundly alter local flame structure and stabilization mechanisms, particularly near the inner recirculation zone where unsteady flame-vortex interactions dominate heat release distribution.</t>
+          <t>Abstract The performance of a hybrid transported-tabulated chemistry (HTTC) strategy is evaluated for large-eddy simulations (LES) of turbulent combustion with detailed finite-rate kinetics. The computational cost of LES is reduced in the HTTC approach by segregating the species list into major and minor species, with the former transported and the latter tabulated. Apart from reducing the number of transported species, the HTTC approach and its variants decrease computational cost by enabling efficient computation of thermodynamics and transport properties and by relieving the stiffness of chemical source terms. The calculations can be up to 11 times faster with stiff kinetics (29 species, 141 steps), as the HTTC approach eliminates the need to integrate and transport the minor species, which typically have short chemical times. The original HTTC and other variants are assessed for their accuracy, efficiency, and robustness for LES by considering two temporally evolving challenging test cases: a freely propagating turbulent premixed flame in the thin reaction zone regime and a turbulent non-premixed jet flame exhibiting local extinction and re-ignition. Modifications to the original HTTC approach are considered and evaluated to account for the effect of subgrid-scale turbulence. Both a priori and a posteriori analyses are conducted to evaluate the accuracy of the HTTC approach. The turbulent premixed flame test shows noticeable yet small differences between the calculated and tabulated concentrations of minor species. This results in reasonable predictions of reaction rates and overall combustion process with HTTC. The difference between calculated and tabulated minor species concentrations is larger for the turbulent non-premixed flame case; however, the minor species concentrations are generally much lower for it, and therefore, extinction-re-ignition physics is still predicted well with HTTC.</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>Effects of multi-fuel blending on combustion characteristics of turbulent premixed swirling flames</t>
+          <t>Large-Eddy Simulations of Soot Formation and Dispersion in Rich-Burn Quick-Mix Lean-Burn (RQL) Spray Combustor</t>
         </is>
       </c>
       <c r="T8" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.proci.2022.07.034", "https://doi.org/10.1016/j.proci.2022.07.034")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2025-2484", "https://doi.org/10.2514/6.2025-2484")</f>
         <v/>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>performing LES with PRISM tabulated chemistry across methane-hydrogen blends (0-60% H2 by volume) in a swirl combustor, demonstrating that hydrogen enrichment amplifies local laminar flame speed by up to 48% and activates preferential diffusion wrinkling that reshapes thermoacoustic coupling frequencies.</t>
+          <t>performing LES with a Lagrangian spray and PAH soot kinetics in an RQL combustor at 6.8 atm, demonstrating that shifting global equivalence ratio from 0.12 to 0.2 markedly increases primary-zone soot volume fraction through localized flame-spray-soot interactions.</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t>The effects of fuel composition on turbulent premixed combustion characteristics of swirling flames are investigated using high-fidelity large eddy simulations (LES). Three fuel blends of methane and hydrogen (0%, 30%, and 60% H2 by volume) are studied in a gas turbine model combustor at atmospheric pressure. The LES employs a dynamic localized combustion model with detailed chemistry tabulation via PRISM. Increased hydrogen fraction accelerates local flame propagation by up to 48%, narrows the reaction zone, and triggers preferential diffusion-driven flame wrinkling at small scales, with direct consequence for NOx formation pathways.</t>
+          <t>The influence of varying fuel/air ratios on the primary zone soot formation characteristics of the liquid-fueled rich-quench-lean (RQL) combustor is investigated numerically. Large- eddy simulations (LES) of two global equivalence ratios (��) corresponding to 0.12 and 0.2 respectively are conducted at an overall pressure of 6.8 atm. The employed LES modeling framework includes Lagrangian treatment for liquid-fuel spray, finite-rate chemistry for gas- phase combustion, a polycyclic aromatic hydrocarbon (PAH)-based soot model, a partially stirred reactor model for turbulence-soot-chemistry interactions, and an optically thin radiation model. The soot and gas-phase chemistry modeling framework is verified against the experimental measurements from canonical premixed and non-premixed flames of gaseous ethylene fuels. The LES simulations of the RQL combustor qualitatively demonstrate the trend of increasing soot volume fractions (SVFs) under the two conditions investigated in this work. Further analysis of local flame-soot-spray interactions and soot source terms is reported to explain the observed differences.</t>
         </is>
       </c>
       <c r="W8" s="2" t="inlineStr">
         <is>
-          <t>1. Subgrid combustion modeling for LES of spray combustion in turbulent swirling flows (Combustion and Flame, 2022) | 2. Effects of multi-fuel blending on combustion of turbulent premixed swirling flames (Proc. Combustion Institute, 2023)</t>
+          <t>1. Application of Hybrid Transported-Tabulated Chemistry for Efficient Large-Eddy Simulation of Turbulent Combustion (Flow Turbulence and Combustion, 2026) | 2. Large-Eddy Simulations of Soot Formation and Dispersion in Rich-Burn Quick-Mix Lean-Burn (RQL) Spray Combustor (2025)</t>
         </is>
       </c>
       <c r="X8" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2021.111634 | https://doi.org/10.1016/j.proci.2022.07.034", "https://doi.org/10.1016/j.combustflame.2021.111634 | https://doi.org/10.1016/j.proci.2022.07.034")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s10494-026-00794-4 | https://doi.org/10.2514/6.2025-2484", "https://doi.org/10.1007/s10494-026-00794-4 | https://doi.org/10.2514/6.2025-2484")</f>
         <v/>
       </c>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>coupling Lagrangian spray dynamics with LES dynamic subgrid combustion in a bluff-body swirl combustor, demonstrating that droplet evaporation controls inner-recirculation-zone flame anchoring and produces unsteady heat-release fluctuations at Strouhal numbers consistent with observed thermoacoustic instabilities.</t>
+          <t>implementing a hybrid transported-tabulated chemistry (HTTC) strategy in LES of turbulent combustion with 29 species and 141 steps, demonstrating up to 11-fold computational speedup while maintaining high fidelity in predicting extinction and re-ignition dynamics.</t>
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr">
@@ -5299,64 +5295,64 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Thermoacoustic instability theory, turbulent flame linear response functions, and hydrodynamic wavemaker identification in low-NOx combustors -- building physics-based predictive frameworks for acoustic-flame coupling in next-generation gas turbines and hydrogen-fueled engines.</t>
+          <t>Combustion dynamics, swirl burner flame stability, low-carbon ammonia (NH3) rich-relaxation-quench-lean (RRQL) combustion systems, and turbulence sensitivity of NOx/CO emissions in hydrogen-methane blends.</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>High-speed OH-PLIF, Acoustic forcing rigs (transverse/longitudinal), Phase-locked PIV, Global flame transfer function measurement, Wavemaker stability analysis</t>
+          <t>High-speed OH*/NH2* chemiluminescence, Modular swirl burners, Gas-phase emissions sampling (NOx, N2O, NH3, CO), Turbulence-flame interaction rigs</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Flame Transfer Function Measurement of a Transversely Excited Swirling Flame</t>
+          <t>Toward the Development of an RRQL System—Part I: Swirl Pattern Effect on Exhaust Emissions and Chemiluminescence Distribution for NH3–Air Premixed Swirl Flames</t>
         </is>
       </c>
       <c r="P9" s="3">
-        <f>HYPERLINK("https://doi.org/10.1115/1.4053164", "https://doi.org/10.1115/1.4053164")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/1.4069796", "https://doi.org/10.1115/1.4069796")</f>
         <v/>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>measuring transverse flame transfer functions via phase-locked OH-PLIF in a swirl-stabilized combustor, demonstrating that transverse excitation produces peak gain at the swirler geometric resonance rather than the convective residence time, directly altering annular combustor thermoacoustic stability predictions.</t>
+          <t>investigating swirl geometry effects on flame morphology and emissions in rich premixed NH3-air flames for an RRQL system, demonstrating that compact flames minimize wall quenching and enable post-flame relaxation to suppress NOx and NH3 emissions.</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>This paper presents measurements of the flame transfer function (FTF) of a swirl-stabilized flame excited by transverse acoustic forcing. Using phase-locked OH-PLIF and acoustic pressure measurements, the FTF relating heat release rate fluctuations to transverse velocity perturbations is characterized over 100-600 Hz. Results show that the transverse FTF exhibits a substantially different gain-phase structure than the longitudinal FTF, with peak gain at frequencies near the swirler geometric resonance rather than the convective time scale.</t>
+          <t>Abstract Ammonia (NH3) is a carbon–free energy source and hydrogen carrier, but its fuel–bound nitrogen can lead to significant nitrogen oxides (NOx) emissions. Staged combustion strategies, such as rich–quench–lean, can achieve low NOx emissions. However, improper design may result in high NOx levels when operating with a rich head end without a sufficient post–flame relaxation time. Previous work has shown that a rich–relaxation–quench–lean (RRQL) configuration can minimize NOx emissions in the rich head end (Cole et al., 2024, “Rich Ammonia Flame Shapes and NO Relaxation: Facility Development and Characterization,” ASME Paper No. GT2024–122369). This study focuses on how different swirl geometries affect exhaust emissions and flame morphology in rich, premixed NH3–air flames, for the design of a rich relaxation head end of an RRQL combustor. Experiments were conducted using a modular swirl burner and measuring NOx, N2O, and NH3 emissions, and recording natural flame luminosity and NH2* and OH* chemiluminescence images. Swirler design affects emissions by influencing flame length (with shorter flames allowing for more postflame relaxation time) and flame–wall interactions (influencing NH3 and N2O emissions). A compact flame with minimal wall interactions allows for increased NOx relaxation, while minimal wall interactions prevent heat losses and instabilities, which minimize NH3 and N2O emissions at a richer equivalence ratio, potentially enhancing H2 production during the relaxation phase without increasing overall primary stage NOx emissions, thereby improving system efficiency. Detailed spatial evolution of NOx, N2O, and NH3 emissions further supports the RRQL as a promising combustor design for NH3 combustion, if the rich head end is designed properly.</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Hydrodynamic stability of reacting swirling jets</t>
+          <t>Measurements of CO and NOx Emissions From Premixed Turbulent Methane/Hydrogen Flames</t>
         </is>
       </c>
       <c r="T9" s="3">
-        <f>HYPERLINK("https://doi.org/10.1017/jfm.2021.433", "https://doi.org/10.1017/jfm.2021.433")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/1.4069625", "https://doi.org/10.1115/1.4069625")</f>
         <v/>
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>performing global wavemaker stability analysis of reacting swirling jets across varying equivalence ratios, demonstrating that combustion heat release simultaneously destabilizes the axisymmetric (m=0) centrifugal mode and suppresses the precessing vortex core (m=+-1) helical instability branch.</t>
+          <t>measuring the sensitivity of NO and CO emissions from turbulent premixed H2/CH4 flames across varying turbulence intensities, demonstrating that H2 enrichment sharply accelerates CO relaxation toward equilibrium while turbulence intensity yields negligible impact on NO at constant CO.</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
         <is>
-          <t>The hydrodynamic stability of reacting swirling jets is investigated using global stability analysis and wavemaker identification. Structural sensitivity analysis reveals a confined wavemaker region near the central recirculation zone boundary. Two competing instability branches are identified: an axisymmetric (m=0) branch driven by centrifugal destabilization and a helical (m=+-1) branch associated with the precessing vortex core (PVC). Increased heat release from combustion destabilizes the m=0 mode and simultaneously stabilizes the PVC branch.</t>
+          <t>Abstract This paper presents measurements of the sensitivity of NO and CO emissions from H2/CH4 combustion to variations in turbulence intensity. Existing studies of exhaust emissions either focus on laminar modeling and measurements or report device-level measurements from practical combustors. However, there are limited fundamental studies of emissions characteristics of turbulent systems, the focus of this study. Because of the strong stretch sensitivity of these mixtures, local temperatures/reaction rates along the turbulent front can differ markedly from mixture-averaged properties, and they are very sensitive to turbulence. Single-point emissions measurements are presented for turbulent premixed H2/CH4 flames from a contoured nozzle Bunsen burner with variable turbulence. Emissions are measured at varying residence times and incoming flow turbulence intensities. Data show the clear benefit of H2 blending on CO emissions, both due to the expected reduction in C atoms, but also due to faster relaxation of flame generated CO toward equilibrium. It also shows negligible impact of turbulence intensity on NO emissions at constant CO for CH4.</t>
         </is>
       </c>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>1. Flame Transfer Function of a Transversely Excited Swirling Flame (JEGTP, 2022) | 2. Hydrodynamic stability of reacting swirling jets (Journal of Fluid Mechanics, 2021)</t>
+          <t>1. Toward the Development of an RRQL System—Part I: Swirl Pattern Effect on Exhaust Emissions and Chemiluminescence Distribution for NH3–Air Premixed Swirl Flames (Journal of Engineering for Gas Turbines and Power, 2025) | 2. Measurements of CO and NOx Emissions From Premixed Turbulent Methane/Hydrogen Flames (Journal of Engineering for Gas Turbines and Power, 2025)</t>
         </is>
       </c>
       <c r="X9" s="3">
-        <f>HYPERLINK("https://doi.org/10.1115/1.4053164 | https://doi.org/10.1017/jfm.2021.433", "https://doi.org/10.1115/1.4053164 | https://doi.org/10.1017/jfm.2021.433")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/1.4069796 | https://doi.org/10.1115/1.4069625", "https://doi.org/10.1115/1.4069796 | https://doi.org/10.1115/1.4069625")</f>
         <v/>
       </c>
       <c r="Y9" s="2" t="inlineStr">
         <is>
-          <t>measuring transverse flame transfer functions via phase-locked OH-PLIF in a swirl-stabilized combustor, demonstrating that transverse excitation produces peak gain at the swirler geometric resonance rather than the convective residence time, directly altering annular combustor thermoacoustic stability predictions.</t>
+          <t>investigating swirl geometry effects on flame morphology and emissions in rich premixed NH3-air flames for an RRQL system, demonstrating that compact flames minimize wall quenching and enable post-flame relaxation to suppress NOx and NH3 emissions.</t>
         </is>
       </c>
       <c r="Z9" s="2" t="inlineStr">
@@ -5479,64 +5475,64 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Computational soft-matter and mesoscale fluid mechanics -- lattice Boltzmann / immersed boundary simulations of active elastic filaments, magnetically controlled microswimmers, elastic capsule deformation in microchannel flow, and interfacial transport in patterned soft-wetting surfaces.</t>
+          <t>Quantum lattice Boltzmann methods (QLBM) for phase-change heat transfer and mesoscale modeling of responsive hydrogel interfaces and fluid-structure interaction.</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Lattice-Boltzmann Method (LBM), Immersed Boundary Method (IBM), Elastic network membrane model, Magnetic dipole actuator model, Finite element structural coupling</t>
+          <t>Quantum Lattice Boltzmann Method (QLBM), Dissipative Particle Dynamics (DPD), Quantum circuit state storage (53 qubits), Immersed Boundary Method (IBM)</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Magnetic soft robot locomotion across unstructured terrains</t>
+          <t>Neutron Reflectometry and Compression of Graded Hydrogel Surfaces</t>
         </is>
       </c>
       <c r="P10" s="3">
-        <f>HYPERLINK("https://doi.org/10.1002/adma.202307002", "https://doi.org/10.1002/adma.202307002")</f>
+        <f>HYPERLINK("https://doi.org/10.1002/admi.70580", "https://doi.org/10.1002/admi.70580")</f>
         <v/>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>simulating magnetic soft robot locomotion with IBM-coupled elastic shell mechanics across terrain roughness Ra/L = 0-0.3, demonstrating undulatory gaits outperform rolling by 2.8x on irregular substrates with gait switching at critical roughness threshold Ra/L = 0.12.</t>
+          <t>investigating depth-wise graded hydrogel layers via neutron reflectometry and DPD mesoscale simulations, demonstrating that near-surface polymer network collapse under compression dictates contact stress modulation and effective elastic modulus.</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>IBM-coupled elastic shell finite element mechanics simulates magnetic soft robot locomotion across substrates with random height perturbations up to 30% of body length. Undulatory gaits outperform rolling gaits by 2.8x on irregular substrates. Gait switching occurs at a terrain roughness threshold of Ra/L = 0.12.</t>
+          <t>ABSTRACT Polyacrylamide hydrogels with depth‐wise gradients in polymer density (i.e., surface gel layers) are ideal synthetic models to understand stress modulation in hierarchical, compositionally‐graded biological tissues, including articular cartilage, in part, due to their similarities in water content and network structure. This work investigated surface gel layer thickness and crosslinker mobility (e.g., covalent crosslinks vs. physical entanglements) in polyacrylamide hydrogels and their impact on mechanical properties via confocal microscopy, indentation and compression measurements, neutron reflectivity, and mesoscale modeling. Hydrogels polymerized against oxygen‐permeable polydimethylsiloxane exhibited thicker surface gel layers and significantly lower elastic modulus compared to hydrogels polymerized against oxygen‐impermeable glass. Physical entanglements lowered the hydrogel elastic modulus within the surface gel layer and throughout the bulk. Neutron reflectivity revealed the collapse of near‐surface polymer networks under compressive loads, in good agreement with dissipative particle dynamics (DPD) simulations. Our results suggested that both the hydrogel elastic...</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>Elastic capsules in shear flow near a planar wall: Numerical simulation</t>
+          <t>Quantum lattice Boltzmann algorithm for heat transfer with phase change</t>
         </is>
       </c>
       <c r="T10" s="3">
-        <f>HYPERLINK("https://doi.org/10.1063/5.0078753", "https://doi.org/10.1063/5.0078753")</f>
+        <f>HYPERLINK("https://doi.org/10.1088/2058-9565/ae7b7c", "https://doi.org/10.1088/2058-9565/ae7b7c")</f>
         <v/>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>simulating elastic capsule wall migration via IB-LBM at Ca=0.1-0.5 and h/a=0.1-2.0, demonstrating near-wall membrane amplifies principal strain by 45-68% relative to far-field and lateral migration velocity scales as Ca*(h/a)^-3.</t>
+          <t>implementing a quantum lattice Boltzmann method (QLBM) on 17 lattice nodes using 53 qubits for phase-change heat transfer, demonstrating accurate moving interface tracking with temperature RMS errors of order 0.01 relative to classical analytical solutions.</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>IB-LBM simulates elastic capsule dynamics in shear flow near a rigid wall. Near-wall membrane deformation is amplified by 45-68% relative to far-field, with maximum principal strain of 0.42 at Ca=0.5, h/a=0.15. Lateral migration velocity scales as Ca*(h/a)^-3.</t>
+          <t>Abstract Heat transfer involving phase change is computationally intensive due to moving phase boundaries, nonlinear computations, and time step restrictions. This paper presents a quantum lattice Boltzmann method (QLBM) for simulating heat transfer with phase change. The approach leverages the statistical nature of the lattice Boltzmann method (LBM) while addressing the challenges of discontinuous phase transitions in quantum computing. The method implements an interface-tracking strategy that partitions the problem into separate solid and liquid domains, enabling the algorithm to handle the discontinuity in the enthalpy–temperature relationship. We store phase change information in the quantum circuit to reduce information exchange between classical and quantum hardware, a bottleneck in many quantum applications. Results from the implementation agree with both classical LBM and analytical solutions, demonstrating QLBM as an effective approach for analyzing thermal systems with phase transitions. Simulations using 17 lattice nodes with 53 qubits demonstrate temperature root-mean-square errors of order 0.01 when compared against classical solutions. The method accurately tracks ...</t>
         </is>
       </c>
       <c r="W10" s="2" t="inlineStr">
         <is>
-          <t>1. Magnetic soft robot locomotion across unstructured terrains (Advanced Materials, 2023) | 2. Elastic capsules in shear flow near a planar wall: Numerical simulation (Biomicrofluidics, 2022)</t>
+          <t>1. Neutron Reflectometry and Compression of Graded Hydrogel Surfaces (Advanced Materials Interfaces, 2026) | 2. Quantum lattice Boltzmann algorithm for heat transfer with phase change (Quantum Science and Technology, 2026)</t>
         </is>
       </c>
       <c r="X10" s="3">
-        <f>HYPERLINK("https://doi.org/10.1002/adma.202307002 | https://doi.org/10.1063/5.0078753", "https://doi.org/10.1002/adma.202307002 | https://doi.org/10.1063/5.0078753")</f>
+        <f>HYPERLINK("https://doi.org/10.1002/admi.70580 | https://doi.org/10.1088/2058-9565/ae7b7c", "https://doi.org/10.1002/admi.70580 | https://doi.org/10.1088/2058-9565/ae7b7c")</f>
         <v/>
       </c>
       <c r="Y10" s="2" t="inlineStr">
         <is>
-          <t>simulating magnetic soft robot locomotion with IBM-coupled elastic shell mechanics across terrain roughness Ra/L = 0-0.3, demonstrating undulatory gaits outperform rolling by 2.8x on irregular substrates with gait switching at critical roughness threshold Ra/L = 0.12.</t>
+          <t>investigating depth-wise graded hydrogel layers via neutron reflectometry and DPD mesoscale simulations, demonstrating that near-surface polymer network collapse under compression dictates contact stress modulation and effective elastic modulus.</t>
         </is>
       </c>
       <c r="Z10" s="2" t="inlineStr">
@@ -5544,11 +5540,7 @@
           <t>Skip To Keyboard Navigation Toggle navigation George W. Woodruff School of Mechanical Engineering Main navigation Home About Ch...</t>
         </is>
       </c>
-      <c r="AA10" s="2" t="inlineStr">
-        <is>
-          <t>"Neutron Reflectometry and Compression of Graded Hydrogel Surfaces" [Advanced Materials Interfaces] (2026) [DOI: https://doi.org/10.1002/admi.70580] | "Quantum lattice Boltzmann algorithm for heat transfer with phase change" [Quantum Science and Technology] (2026) [DOI: https://doi.org/10.1088/2058-9565/ae7b7c] | "Undulatory hydrodynamics of tapered elastic plates in viscous fluid" [Journal of Fluid Mechanics] (2026) [DOI: https://doi.org/10.1017/jfm.2026.11157] | "MEASUREMENT TECHNIQUE MEASUREMENT OF ABSORBED DOSE IN WATER DURING IRRADIATION IN CARBON ION AND PROTON BEAMS USING THERMAL LUMINESCENCE DOSIMETERS номер в ФИФ: ФР.1.38.2025.52532" (2026) [DOI: https://doi.org/10.13140/rg.2.2.36020.51847] | "Mesoscale Modeling of Hydrogels Under Frictional Shear Stress" [Macromolecules] (2025) [DOI: https://doi.org/10.1021/acs.macromol.5c01748]</t>
-        </is>
-      </c>
+      <c r="AA10" s="2" t="inlineStr"/>
       <c r="AB10" s="2" t="inlineStr">
         <is>
           <t>"Deformations in Si−Li Anodes Upon Electrochemical Alloying in Nano-Confined Space" [Journal of the American Chemical Society] (2010, 324 cites) [DOI: https://doi.org/10.1021/ja1031997] | "Ultrasoft microgels displaying emergent platelet-like behaviours" [Nature Materials] (2014, 221 cites) [DOI: https://doi.org/10.1038/nmat4066] | "Harnessing Janus Nanoparticles to Create Controllable Pores in Membranes" [ACS Nano] (2008, 198 cites) [DOI: https://doi.org/10.1021/nn8000998]</t>
@@ -5679,64 +5671,64 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Lattice-Boltzmann and fluctuating lattice-Boltzmann methods for multiphase suspension flows, deformable capsule dynamics in microcirculation, and turbulent fiber suspensions -- bridging colloidal-scale stochastic physics with engineering-scale flow predictions.</t>
+          <t>Direct numerical simulation (DNS) and experimental scaling of bubble interactions in decaying dynamic turbulence, Hinze-scale evolution, and microbubble mass-transfer control.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Lattice-Boltzmann Method (LBM), Fluctuating Lattice-Boltzmann (FLB), Immersed Boundary Method (IBM), Spectral Element DNS, Capsule membrane finite-element models</t>
+          <t>DNS of bubble-laden homogeneous isotropic turbulence, Particle Shadow Velocimetry (PSV), High-speed back-lit shadowgraphy, Lattice Boltzmann suspension modeling</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>Lattice Boltzmann simulation of the dynamics of capsule suspensions in shear flow</t>
+          <t>On the scaling of bubble interactions in dynamic turbulence: theoretical, numerical, and experimental study</t>
         </is>
       </c>
       <c r="P11" s="3">
-        <f>HYPERLINK("https://doi.org/10.1103/PhysRevFluids.7.054302", "https://doi.org/10.1103/PhysRevFluids.7.054302")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2607.25251", "https://doi.org/10.48550/arxiv.2607.25251")</f>
         <v/>
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>coupling LBM with finite-element capsule membrane models for volume fractions up to 0.40, demonstrating hydrodynamic capsule interactions produce shear-induced diffusivity of 3.2e-3 and drive a 340% viscosity increase from dilute to concentrated regimes.</t>
+          <t>investigating bubbly decaying homogeneous isotropic turbulence via DNS and experiments, demonstrating that when dissipation decays rapidly the Hinze scale overtakes bubble diameter, driving a transition from super-Hinze to capillary-dominated sub-Hinze scaling.</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>LBM coupled with finite-element membrane models studies capsule suspensions in shear flow at volume fractions up to 0.40. Shear-induced diffusion coefficient D_s/gamma_dot*a^2 = 3.2e-3, comparable to experimental hard-sphere measurements. Bulk suspension viscosity increases by 340% from dilute to concentrated regime at the same capillary number.</t>
+          <t>This study investigates dilute bubbly decaying homogeneous isotropic turbulence at high Reynolds number using theory, direct numerical simulation, and experiments. The turbulent kinetic energy and dissipation rate follow power-law decay, while the bubble population reorganizes relative to the evolving Hinze scale. When the dissipation decays sufficiently rapidly, the Hinze scale grows faster than the characteristic bubble diameter, driving the population from super-Hinze toward sub-Hinze sizes. The system passes through a mixed regime in which coalescence dominates but breakup remains active, followed by a pure-coalescence regime. Residual breakup in the mixed regime increases the number of small bubbles and enhances coalescence, leading to faster growth of the characteristic bubble size. DNS of dilute bubble-laden turbulence shows decay exponents close to single-phase turbulence and a bubble-size distribution that shifts toward smaller diameter relative to the Hinze scale. Before the transition, the distribution exhibits two power-law ranges associated with capillary effects and inertial breakup; after the transition, it approaches a single capillary-dominated scaling. Theory a...</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>Fluctuating lattice Boltzmann method for complex fluids and dense suspensions</t>
+          <t>Mass-Transfer Control With Microbubbles in Highly Turbulent Decaying Flows</t>
         </is>
       </c>
       <c r="T11" s="3">
-        <f>HYPERLINK("https://doi.org/10.1017/jfm.2021.432", "https://doi.org/10.1017/jfm.2021.432")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2604.24520", "https://doi.org/10.48550/arxiv.2604.24520")</f>
         <v/>
       </c>
       <c r="U11" s="2" t="inlineStr">
         <is>
-          <t>extending fluctuating LBM to dense suspensions at volume fractions 0.35-0.55, demonstrating sub-diffusive caging dynamics with MSD ~ t^0.72 and predicting viscosity divergence at 0.63 consistent with Krieger-Dougherty theory.</t>
+          <t>combining extreme turbulence (Re_lambda ~ 10^3) with minute surfactant addition (~0.01% CMC) in a straight duct, demonstrating that interfacial tuning arrests bubble coalescence and dictates micron-scale bubble size distributions.</t>
         </is>
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>The fluctuating LBM is extended to dense suspensions with thermodynamically consistent Langevin noise. At volume fractions 0.35-0.55, the model captures sub-diffusive dynamics with MSD scaling as t^0.72, consistent with colloidal glass transition theories. Suspension viscosity diverges at volume fraction 0.63, consistent with Krieger-Dougherty theory.</t>
+          <t>We hypothesize that combining extreme turbulence with a minute reduction in surface tension $σ$ (surface tension of the liquid) using surfactant provides a simple and scalable route for controlling micron scale bubble size in gas--liquid systems. To test this, we generate high-intensity turbulence using a multiphase pump [turbulent intensity $\ge 40\%$; Taylor Reynolds number $Re_λ=\mathcal{O}(10^3)$; bulk Reynolds number $Re=\mathcal{O}(10^5)$] feeding a straight duct, which produces a decaying turbulent flow where, without additives, bubble coalescence dominates and causes monotonic downstream growth in the mean diameter $d_\mathrm{avg}$ of the bubbles. This growth is governed by the turbulent dissipation rate $\varepsilon$. High-speed imaging, back-lit shadowgraph and particle shadow velocimetry (PSV) quantify bubble statistics ($d_\mathrm{avg}$, and the bubble-size distribution) and turbulence metrics (turbulent kinetic energy $k$, turbulence intensity $\mathcal{I}$, and dissipation rate $\varepsilon$). We then introduce a minute amount ($\sim 0.01\%$ critical micelle concentration) of additive that produces a slight reduction in $σ$, used here only as an interfacial tuning ...</t>
         </is>
       </c>
       <c r="W11" s="2" t="inlineStr">
         <is>
-          <t>1. LBM simulation of capsule suspensions in shear flow (Physical Review Fluids, 2022) | 2. Fluctuating LBM for dense suspensions (Journal of Fluid Mechanics, 2021)</t>
+          <t>1. On the scaling of bubble interactions in dynamic turbulence: theoretical, numerical, and experimental study (arXiv, 2026) | 2. Mass-Transfer Control With Microbubbles in Highly Turbulent Decaying Flows (arXiv, 2026)</t>
         </is>
       </c>
       <c r="X11" s="3">
-        <f>HYPERLINK("https://doi.org/10.1103/PhysRevFluids.7.054302 | https://doi.org/10.1017/jfm.2021.432", "https://doi.org/10.1103/PhysRevFluids.7.054302 | https://doi.org/10.1017/jfm.2021.432")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2607.25251 | https://doi.org/10.48550/arxiv.2604.24520", "https://doi.org/10.48550/arxiv.2607.25251 | https://doi.org/10.48550/arxiv.2604.24520")</f>
         <v/>
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>coupling LBM with finite-element capsule membrane models for volume fractions up to 0.40, demonstrating hydrodynamic capsule interactions produce shear-induced diffusivity of 3.2e-3 and drive a 340% viscosity increase from dilute to concentrated regimes.</t>
+          <t>investigating bubbly decaying homogeneous isotropic turbulence via DNS and experiments, demonstrating that when dissipation decays rapidly the Hinze scale overtakes bubble diameter, driving a transition from super-Hinze to capillary-dominated sub-Hinze scaling.</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr">
@@ -5879,64 +5871,64 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Multi-fidelity rotorcraft aeromechanics -- coupling CAMRAD II with CFD/CSD for dynamic stall, blade-vortex interaction, and coaxial rotor-wake aerodynamics to enable next-generation Urban Air Mobility eVTOL vehicle design.</t>
+          <t>Proprotor-wing interactional aerodynamics across tiltrotor conversion maneuvers, mid-to-high-fidelity CFD coupling (Helios / OVERFLOW / ROAM), and reduced-order wake models for Advanced Air Mobility.</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>CAMRAD II, Overset CFD/CSD loose coupling, Unsteady Vortex Lattice Method (UVLM), GT-Hybrid RANS-LES, Aeroflite wind tunnel PIV validation</t>
+          <t>Helios-OVERFLOW overset CFD, Reduced Order Aerodynamic Model (ROAM), Actuator Line Model (ALM), Immersed Boundary Method (IBM), Power spectral density surface pressure analysis</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Validation of an Unsteady Vortex Lattice Method for Coaxial Rotor Wake Interactions</t>
+          <t>Physics of the Proprotor–Wing Interactional Aerodynamics Across the Tiltrotor Conversion Maneuver</t>
         </is>
       </c>
       <c r="P12" s="3">
-        <f>HYPERLINK("https://doi.org/10.4050/JAHS.67.032007", "https://doi.org/10.4050/JAHS.67.032007")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.c038965", "https://doi.org/10.2514/1.c038965")</f>
         <v/>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>validating a free-wake UVLM for coaxial rotor wake mutual induction against Georgia Tech PIV data, demonstrating 6.4% RMS blade normal force accuracy and capturing the figure-8 loading signature in the lower rotor from upper-rotor tip-vortex impingement.</t>
+          <t>simulating two-way coupled proprotor-wing interaction across tilt angles in 15-degree increments using high-fidelity CFD, demonstrating that wing surface pressure PSD reveals dominant wake excitation frequencies during tiltrotor conversion maneuvers.</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>An unsteady vortex lattice method (UVLM) for coaxial rotor aerodynamics is validated against GT Aeroflite wind tunnel PIV data. The UVLM predicts blade normal force within 6.4% RMS error across the azimuth and reproduces the characteristic figure-8 loading signature in the lower rotor due to upper rotor tip vortex impingement.</t>
+          <t>The conversion maneuver is one of the most complex and hazardous aspects of tiltrotor operations. The complex interactions increase pilot workload and vibratory wing loads, making it imperative to further understand and accurately predict this dynamic operation. An extensively correlated high-fidelity computational fluid dynamics (CFD) model elucidates the physics within these two-way coupled aerodynamic interactions for a generic model-scale tractor proprotor–wing configuration. Quasi-static evaluations are conducted for proprotor tilt angles in fifteen degree increments to capture the conversion from low-speed edgewise flight to cruise. To assess and quantify the coupled proprotor–wing interactions, additional assessments of an isolated wing at two relevant wing angles of attack and an isolated proprotor operating at all tilt angles were conducted. Wing thickness and loading were mildly correlated with the proprotor loads due to the large proprotor–wing separation relative to the proprotor radius. The proprotor-to-wing effects were assessed using a power spectral density of the wing surface pressure within the proprotor wake. This novel approach elucidates the dominant frequen...</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>Multi-fidelity aeromechanical analysis of a UH-60A rotor in forward flight using loosely coupled CFD/CSD</t>
+          <t>Mid-Fidelity Investigation of the Proprotor-Wing Aerodynamic Interactions across the Tiltrotor Conversion Maneuver</t>
         </is>
       </c>
       <c r="T12" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.J059977", "https://doi.org/10.2514/1.J059977")</f>
+        <f>HYPERLINK("https://doi.org/10.4050/f-0082-2026-0243", "https://doi.org/10.4050/f-0082-2026-0243")</f>
         <v/>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>loosely coupling overset RANS with CAMRAD II across UH-60A advance ratios from 0.15 to 0.368, demonstrating rotor performance within 4.5% of flight test data and capturing dynamic stall vibratory 4P loads at high-advance-ratio conditions.</t>
+          <t>evaluating the Helios mid-fidelity ROAM actuator line model against OVERFLOW for proprotor-wing conversion, demonstrating that adaptive mesh refinement (AMR) in the off-body Cartesian domain is essential for capturing proprotor vortex trajectory and wing load distribution.</t>
         </is>
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>Loosely coupled CFD/CSD methodology is applied to the UH-60A main rotor across advance ratios from mu = 0.15 to 0.368. Rotor performance including thrust, torque, and blade pitch angles agree with UH-60A flight test data within 4.5%. Dynamic stall at high advance ratios is captured with qualitative agreement to flight test vibratory loads at 4P frequency.</t>
+          <t>This paper assesses the capabilities and limitations of mid-fidelity computational fluid dynamics (CFD) approaches when resolving the complex aerodynamic interactions for a generic model-scale proprotor-wing configuration across the tiltrotor conversion maneuver. The Helios mid-fidelity Reduced Order Aerodynamic Model (ROAM) is evaluated against prior extensively validated high-fidelity Helios-OVERFLOW assessments for the proprotor-wing configuration. The ROAM actuator line model (ALM), which represents the proprotor blade via source terms injected into the off-body Cartesian domain, is assessed for the isolated proprotor configuration at several mesh resolutions to understand the requirements to accurately resolve the proprotor physics across the conversion maneuver. The impact of adaptive mesh refinement (AMR) on ROAM's ability to resolve the proprotor physics is also investigated. Next, the flow characteristics and wing loads are evaluated using the ROAM immersed boundary method (IBM) for the isolated wing. The sensitivity of the ROAM IBM predictions to mesh resolution and boundary condition selection is quantified in these assessments. Leveraging the findings from the isolat...</t>
         </is>
       </c>
       <c r="W12" s="2" t="inlineStr">
         <is>
-          <t>1. Validation of an Unsteady Vortex Lattice Method for Coaxial Rotor Wake Interactions (JAHS, 2022) | 2. Multi-fidelity aeromechanical analysis of UH-60A rotor using loosely coupled CFD/CSD (AIAA J., 2021)</t>
+          <t>1. Physics of the Proprotor–Wing Interactional Aerodynamics Across the Tiltrotor Conversion Maneuver (Journal of Aircraft, 2026) | 2. Mid-Fidelity Investigation of the Proprotor-Wing Aerodynamic Interactions across the Tiltrotor Conversion Maneuver (2026)</t>
         </is>
       </c>
       <c r="X12" s="3">
-        <f>HYPERLINK("https://doi.org/10.4050/JAHS.67.032007 | https://doi.org/10.2514/1.J059977", "https://doi.org/10.4050/JAHS.67.032007 | https://doi.org/10.2514/1.J059977")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.c038965 | https://doi.org/10.4050/f-0082-2026-0243", "https://doi.org/10.2514/1.c038965 | https://doi.org/10.4050/f-0082-2026-0243")</f>
         <v/>
       </c>
       <c r="Y12" s="2" t="inlineStr">
         <is>
-          <t>validating a free-wake UVLM for coaxial rotor wake mutual induction against Georgia Tech PIV data, demonstrating 6.4% RMS blade normal force accuracy and capturing the figure-8 loading signature in the lower rotor from upper-rotor tip-vortex impingement.</t>
+          <t>simulating two-way coupled proprotor-wing interaction across tilt angles in 15-degree increments using high-fidelity CFD, demonstrating that wing surface pressure PSD reveals dominant wake excitation frequencies during tiltrotor conversion maneuvers.</t>
         </is>
       </c>
       <c r="Z12" s="2" t="inlineStr">
@@ -6607,64 +6599,64 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>High-fidelity LES of supercritical-pressure reacting flows -- combining real-fluid thermodynamics, finite-rate chemistry, and subgrid turbulence closures to resolve transcritical LOX/CH4 injection, flame stabilization, and combustion instability in rocket and gas-turbine combustors.</t>
+          <t>Lagrangian coherent structures (LCS), finite-time Lyapunov exponent (FTLE) ridges, and adjoint-based receptivity/biorthogonal decomposition in compressible turbulent reacting shear layers.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>LES (Peng-Robinson real-fluid EOS), Finite-rate GRI-Mech 3.0 chemistry, Dynamic Smagorinsky subgrid, Transcritical jet DNS, RAPTOR high-performance CFD solver</t>
+          <t>Direct Numerical Simulation (DNS), Forward/backward FTLE ridges, Hyperbolic geodesic LCS, Cauchy-Green deformation tensors, Direct/adjoint biorthogonal eigenmode projection</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Large eddy simulation of a supercritical LOX/CH4 round jet flame</t>
+          <t>Planar Lagrangian transport and scalar-gradient organization in a turbulent reacting shear layer</t>
         </is>
       </c>
       <c r="P2" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2022.112183", "https://doi.org/10.1016/j.combustflame.2022.112183")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2606.20352", "https://doi.org/10.48550/arxiv.2606.20352")</f>
         <v/>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>performing real-fluid LES with Peng-Robinson EOS in a supercritical LOX/CH4 jet flame at 6 MPa, demonstrating that transcritical pseudoboiling produces a LOX core of L_c/D = 4.8 and anchors the diffusion flame within 2 jet diameters at the pseudoboiling interface.</t>
+          <t>analyzing 3D DNS of a supersonic reacting H2-air temporal mixing layer via hyperbolic geodesic LCS and FTLE ridges, demonstrating that forward/backward ridge intersections govern localized scalar-gradient enrichment and strain-dominated transport skeletons.</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>LES of a turbulent supercritical LOX/CH4 round jet flame at 6 MPa using RAPTOR with Peng-Robinson real-fluid EOS. The pseudoboiling transition of LOX injected at 120 K into supercritical methane at 300 K produces a dense LOX core of L_c/D = 4.8. Flame stabilization occurs within 2 jet diameters at the highest-density-gradient pseudoboiling interface.</t>
+          <t>We analyze planar Lagrangian transport and scalar-gradient organization in a supersonic, reacting hydrogen-air temporal mixing layer using time-resolved mid-plane data from a three-dimensional direct numerical simulation. The analysis combines forward/backward finite-time Lyapunov exponent (FTLE) fields, operational FTLE-ridge skeletons, Cauchy-Green deformation measures, shear-LCS metrics, and planar hyperbolic geodesic-LCS extraction to examine how finite-time stretching structures the reacting shear layer. The time-resolved FTLE ridges identify repelling and attracting finite-time transport skeletons in the constrained two-dimensional slice, from which ridge geometry, intersection occupancy, persistence, and scalar-conditioned transport are quantified. Hyperbolic geodesic LCS are extracted from Cauchy-Green tensors reconstructed from planar flow maps as strainlines seeded at high-$λ_{\max}$ normal maxima, providing a variational counterpart to the operational FTLE-ridge skeleton. We then relate the transport skeleton to temperature, mixture fraction, and a reaction intermediate. The results show localized forward/backward ridge overlap, strong scalar-gradient enrichment, fini...</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>Analysis of Mixing, Thermodynamic, and Combustion Characteristics of Turbulent Supercritical Flows</t>
+          <t>Receptivity and Biorthogonal Decomposition in a Reacting Temporal Mixing Layer</t>
         </is>
       </c>
       <c r="T2" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.J059845", "https://doi.org/10.2514/1.J059845")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2606.20819", "https://doi.org/10.48550/arxiv.2606.20819")</f>
         <v/>
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>combining DNS and LES with Peng-Robinson real-fluid EOS across three supercritical configurations at 6-10 MPa, demonstrating that density stratification suppresses scalar dissipation rate by 23% near the critical point and sustains sub-centimeter density gradients through the reacting zone.</t>
+          <t>applying energy-weighted adjoint projections and biorthogonal decomposition to a compressible reacting mixing layer, demonstrating that finite-thickness base states sustain unstable Kelvin-Helmholtz modes across low wavenumbers where vortex-sheet approximations remain neutral.</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>DNS and LES with Peng-Robinson EOS study three supercritical configurations: a N2 jet, LOX/H2 shear layer, and LOX/CH4 injector at 10 MPa. Density stratification produces 23% reduction in scalar dissipation rate at the critical point. Sub-centimeter density gradients persist through the reaction zone in the LOX/CH4 injector LES.</t>
+          <t>We examine receptivity and biorthogonal decomposition in a reacting temporal mixing layer using direct and adjoint eigenmodes of a finite-thickness compressible linearized operator built from the mean reacting base state. The analysis focuses on the Kelvin--Helmholtz branch and asks how the reacting base state modifies the selected temporal instability, where localized forcing most efficiently excites it, and how strongly the associated modal family is represented in time-resolved planar simulation data. Receptivity maps are constructed for mass, momentum, thermal, and mixture-fraction forcing channels using an energy-weighted adjoint projection, with biorthogonality enforced by the corresponding direct--adjoint inner product. A complementary biorthogonal decomposition provides modal amplitudes and cumulative few-mode reconstructions at the fundamental streamwise wavenumber. The finite-thickness branch is interpreted against a compressible vortex-sheet reference built from the outer-stream states. The reacting layer supports an unstable finite-thickness Kelvin--Helmholtz family over low-to-moderate wavenumbers even though the discontinuous reference is essentially neutral. Mass ...</t>
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>1. LES of a supercritical LOX/CH4 round jet flame (Combustion and Flame, 2022) | 2. Analysis of Mixing, Thermodynamic, and Combustion Characteristics of Turbulent Supercritical Flows (AIAA J., 2021)</t>
+          <t>1. Planar Lagrangian transport and scalar-gradient organization in a turbulent reacting shear layer (arXiv, 2026) | 2. Receptivity and Biorthogonal Decomposition in a Reacting Temporal Mixing Layer (arXiv, 2026)</t>
         </is>
       </c>
       <c r="X2" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2022.112183 | https://doi.org/10.2514/1.J059845", "https://doi.org/10.1016/j.combustflame.2022.112183 | https://doi.org/10.2514/1.J059845")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2606.20352 | https://doi.org/10.48550/arxiv.2606.20819", "https://doi.org/10.48550/arxiv.2606.20352 | https://doi.org/10.48550/arxiv.2606.20819")</f>
         <v/>
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>performing real-fluid LES with Peng-Robinson EOS in a supercritical LOX/CH4 jet flame at 6 MPa, demonstrating that transcritical pseudoboiling produces a LOX core of L_c/D = 4.8 and anchors the diffusion flame within 2 jet diameters at the pseudoboiling interface.</t>
+          <t>analyzing 3D DNS of a supersonic reacting H2-air temporal mixing layer via hyperbolic geodesic LCS and FTLE ridges, demonstrating that forward/backward ridge intersections govern localized scalar-gradient enrichment and strain-dominated transport skeletons.</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -6803,64 +6795,64 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>First-principles LES and DNS of supercritical combustion, rotating detonation engine (RDE) wave dynamics, and LOX/CH4 propellant injection physics -- resolving real-fluid thermodynamic non-idealities and turbulence-chemistry coupling at rocket-engine operating pressures.</t>
+          <t>Supersonic combustion dynamics in dual-combustion ramjet (DCR) engines, chemical explosive mode analysis (CEMA), and detonative tangential combustion instability mode transitions in liquid and gas rocket combustors.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>LES (real-fluid EOS, cubic Peng-Robinson EOS), DNS of supercritical jets, Modified Benedict-Webb-Rubin (MBWR) EOS, Finite-rate GRI-Mech 3.0 chemistry, RDE wave solvers</t>
+          <t>Chemical Explosive Mode Analysis (CEMA), STFT / Dynamic Mode Decomposition (DMD), Proper Orthogonal Decomposition (POD), Compressible reacting LES, High-order shock-capturing CFD</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Rotating detonation engine with a hollow annular channel: Effects of inlet geometry on wave dynamics</t>
+          <t>Supersonic Combustion and Flow Evolution in Dual-Combustion Ramjet Engine</t>
         </is>
       </c>
       <c r="P3" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2021.111763", "https://doi.org/10.1016/j.combustflame.2021.111763")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.b40184", "https://doi.org/10.2514/1.b40184")</f>
         <v/>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>performing 3D LES with finite-rate H2-O2 kinetics in a hollow annular RDE, demonstrating that inlet slot aspect ratio controls reactant layer thickness and shifts rotating detonation wave speed between 1820 and 2240 m/s, altering wave deficit by up to 15.4% from Chapman-Jouguet.</t>
+          <t>conducting numerical experiments of supersonic combustion in a DCR engine using CEMA and Damkohler number analysis, demonstrating that thermal choking establishes a thermal throat in the constant-area section and elevates pressure, temperature, and nozzle exit Mach number.</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>The rotating detonation engine (RDE) with a hollow annular channel is investigated using 3D LES with detailed H2-O2 kinetics. Slot aspect ratio variations of 1:4 to 4:1 produce wave speeds ranging from 1820 to 2240 m/s, with wave deficits from 8.2% to 15.4% relative to the idealized Chapman-Jouguet value. Inlet geometry controls the freshly mixed reactant layer thickness ahead of the detonation wave, directly setting wave speed and heat release peak.</t>
+          <t>This work presents a numerical investigation of supersonic combustion dynamics and flow evolution in a dual-combustion ramjet (DCR) engine. Two series of parametric numerical experiments were conducted for the DCR combustor configuration by varying the length of the constant-area section [Formula: see text] and the divergence angle [Formula: see text] of the expansion section. The operating conditions were selected to mimic realistic flight scenarios. Two distinct combustion modes were identified, based on the occurrence of thermal choking. To analyze the combustion characteristics of these modes, chemical explosive mode analysis was performed, along with an evaluation of the Damköhler number. In the thermally choked combustion mode, both pressure and temperature were significantly elevated compared to the supersonic shear-layer combustion mode. This increase is attributed to the coupling between pressure and heat release, which enhances combustion efficiency. A thermal throat forms at the end of the constant-area section, while the divergent section functions as a supersonic nozzle. The exit Mach number in thermally choked cases is higher than its counterpart in supersonic shea...</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>Supercritical cryogenic LOX/GH2 combustion in a single-element shear-coaxial injector</t>
+          <t>Resonant phenomena in detonative tangential combustion instability in a rocket combustor</t>
         </is>
       </c>
       <c r="T3" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.B38219", "https://doi.org/10.2514/1.B38219")</f>
+        <f>HYPERLINK("https://doi.org/10.1063/5.0268442", "https://doi.org/10.1063/5.0268442")</f>
         <v/>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>conducting LES with MBWR real-fluid EOS in a LOX/GH2 shear-coaxial injector at 6-12 MPa, demonstrating that transcritical injection eliminates surface tension, produces high-density oxygen fingers in hydrogen coflow, and increases flame standoff length by 38% with rising chamber pressure.</t>
+          <t>applying STFT, DMD, and POD spectral decomposition to detonative tangential combustion instability in a rocket combustor, demonstrating that limit-cycle instabilities originate from thermofluidic wave resonance rather than pure acoustic natural frequencies and exhibit characteristic frequency-shifting harmonics.</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>Supercritical cryogenic LOX/GH2 combustion in a shear-coaxial injector at 6-12 MPa is investigated using LES with MBWR real-fluid EOS. LES reveals that above the critical point, continuous fluid mixing eliminates surface tension and produces high-density LOX fingers that stretch into hydrogen coflow. Flame standoff length increases by 38% as chamber pressure rises from 6 to 12 MPa.</t>
+          <t>In addition to investigating the flow field of detonative tangential combustion instability [Sung, B.-K., Kasahara, J., and Choi, J.-Y., Combust. Flame 275 114092 (2025)], spectral analysis was performed using Short-time Fourier Transform (STFT), Dynamic Mode Decomposition (DMD), and Proper Orthogonal Decomposition (POD) to gain a deeper understanding of the instability modes. By comparing the limit-cycle frequencies with the acoustic natural frequencies, it was confirmed that the detonative tangential combustion instability cannot be analyzed solely based on natural frequencies, as it corresponds to thermofluidic phenomena rather than thermoacoustic instability. The STFT provided time-dependent frequencies and revealed a frequency shift phenomenon during instability mode transitions. Using DMD, the corresponding dominant mode shapes were identified. The POD analysis corroborated the DMD results, and by examining the eigenvectors of the energetic POD modes, the mode undergoing the frequency shift was identified. During limit cycle operation, frequency harmonics emerged as the frequencies of each mode became integer multiples of the most energetic mode, further indicating that de...</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>1. Rotating detonation engine hollow annular channel: Effects of inlet geometry on wave dynamics (Combustion and Flame, 2022) | 2. Supercritical cryogenic LOX/GH2 combustion in a single-element shear-coaxial injector (JPP, 2021)</t>
+          <t>1. Supersonic Combustion and Flow Evolution in Dual-Combustion Ramjet Engine (Journal of Propulsion and Power, 2025) | 2. Resonant phenomena in detonative tangential combustion instability in a rocket combustor (Physics of Fluids, 2025)</t>
         </is>
       </c>
       <c r="X3" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2021.111763 | https://doi.org/10.2514/1.B38219", "https://doi.org/10.1016/j.combustflame.2021.111763 | https://doi.org/10.2514/1.B38219")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.b40184 | https://doi.org/10.1063/5.0268442", "https://doi.org/10.2514/1.b40184 | https://doi.org/10.1063/5.0268442")</f>
         <v/>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>performing 3D LES with finite-rate H2-O2 kinetics in a hollow annular RDE, demonstrating that inlet slot aspect ratio controls reactant layer thickness and shifts rotating detonation wave speed between 1820 and 2240 m/s, altering wave deficit by up to 15.4% from Chapman-Jouguet.</t>
+          <t>conducting numerical experiments of supersonic combustion in a DCR engine using CEMA and Damkohler number analysis, demonstrating that thermal choking establishes a thermal throat in the constant-area section and elevates pressure, temperature, and nozzle exit Mach number.</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
@@ -7003,64 +6995,64 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Simultaneous high-speed 3D laser diagnostics -- tomographic PIV, dual-pump CARS thermometry, and kHz OH-PLIF -- to map turbulence-chemistry interactions, flame kernel growth, and thermoacoustic feedback in swirl-stabilized gas-turbine combustors.</t>
+          <t>High-speed laser diagnostics for high-pressure turbulent reacting flows, ducted fuel injection (DFI) soot mitigation, and lean blowoff stability mechanisms in lean premixed prevaporized (LPP) supersonic transport combustors.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Dual-pump CARS (N2/O2 thermometry), High-speed stereoscopic PIV, kHz OH-PLIF, Tomographic PIV, High-speed Schlieren</t>
+          <t>Filtered Rayleigh Scattering (FRS), High-speed PIV/PLIF, Ducted Fuel Injection (DFI), Optical high-pressure combustor rigs (700 K, 9 bar), Laser extinction soot diagnostics</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Experimental investigation of turbulence-chemistry interaction in a gas turbine model combustor using simultaneous high-speed CARS and PIV</t>
+          <t>Impact of pilot injections on ducted fuel injection performance</t>
         </is>
       </c>
       <c r="P4" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2023.112754", "https://doi.org/10.1016/j.combustflame.2023.112754")</f>
+        <f>HYPERLINK("https://doi.org/10.1177/14680874261426780", "https://doi.org/10.1177/14680874261426780")</f>
         <v/>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>deploying simultaneous 5 kHz dual-pump CARS and stereo-PIV in a swirl combustor, demonstrating that local extinction events co-locate with strain-rate regions where Ka &gt; 50 and that re-ignition traces preferentially the trailing edges of high-scalar-dissipation tubes.</t>
+          <t>investigating the coupling of ducted fuel injection (DFI) with pilot injections in high-pressure diesel combustion, demonstrating that DFI reduces flame spatially integrated natural luminosity (SINL) by 30-70% and pilot injection mitigates peak SINL by a further 16%.</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>Simultaneous dual-pump CARS thermometry and stereoscopic PIV measurements at 5 kHz are applied to characterize turbulence-chemistry interaction in a gas turbine model combustor under atmospheric and elevated pressure conditions. Results demonstrate strongly non-equilibrium scalar mixing in the flame brush: local extinction events co-locate with high-strain-rate regions where turbulent Karlovitz numbers exceed Ka = 50, while re-ignition preferentially occurs at the trailing edges of high-scalar-dissipation tubes, indicating that distributed reaction zones operate transiently in thin-flame mode.</t>
+          <t>This experimental and numerical study evaluates how ducted fuel injection (DFI) and pilot injections interact to impact soot formation and the premixed heat release pressure spike in diesel combustion. Experiments showed that pilot injections reduced the premixed heat release spike of a free spray by approximately 70%, while DFI configurations only experienced a decrease of approximately 25%. Similarly, pilot injections reduced the initial lift-off length (LOL) of the main injection of a free-spray by approximately 30%, while DFI’s initial LOL had little to no change when pilot injections were utilized. Regardless of whether a standalone-main or pilot-main strategy was used, DFI was able to reduce the spatially integrated natural luminosity (SINL) of the flame relative to a free spray, indicating a likely reduction in soot formation. Both duct configurations studied produced steady SINL signals which were approximately 30% and 70% of the free-spray’s, respectively. For DFI, pilot injections further reduced the peak SINL compared to a standalone main by approximately 16%. The decrease in peak SINL correlated with increased spray head penetration rates. The numerical study reveale...</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>Simultaneous high-speed OH-PLIF and stereoscopic PIV of turbulent premixed flames at elevated pressure</t>
+          <t>Lean Blowoff Limits and Emissions Measurements in a Lean Premixed Prevaporized Combustor with Variable Reactant Inhomogeneity</t>
         </is>
       </c>
       <c r="T4" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.proci.2020.06.149", "https://doi.org/10.1016/j.proci.2020.06.149")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0384", "https://doi.org/10.2514/6.2026-0384")</f>
         <v/>
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>conducting simultaneous kHz OH-PLIF and SPIV across 1-5 atm in a swirl combustor, demonstrating that elevated pressure compresses the reaction layer and increases mean tangential strain rates by 3.2x while transitioning flame-wrinkling from Ka-dominated to curvature-dominated kinematic regimes.</t>
+          <t>characterizing lean blowoff (LBO) limits and emissions in an LPP combustor operating at 700 K and 9 bar on Jet A and SAF, demonstrating that moderate prevaporization and premixing are required to anchor main flames and curb NOx emission spikes.</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>Simultaneous kHz-rate OH-PLIF and SPIV measurements were performed in turbulent premixed swirling flames at elevated pressures up to 5 atm. Elevated pressure compresses the reaction layer, increases Damkohler number, and transitions flame-wrinkling dynamics from Ka-dominated to curvature-dominated modes. Strain-rate statistics at 5 atm show that global mean tangential strain rates increase by a factor of 3.2 relative to atmospheric cases.</t>
+          <t>Lean premixed prevaporized (LPP) combustor designs and sustainable aviation fuels (SAF) show great promise for the development of next-generation low-emission civil supersonic transport (CST) aircraft engines. In this work, exhaust emissions sampling and optical diagnostic measurements were conducted in an LPP model combustor with variable reactant inhomogeneity. The LPP combustor features a novel premixer design, which facilitates control of the level of fuel vaporization and fuel-air mixedness entering the combustor. Measurements of lean blowoff (LBO) limits and gaseous emissions trends were obtained through the optically accessible combustor liner and custom exhaust sampling probe. The combustor was operated at elevated temperature (700 K) and pressure (9 bar) conditions to simulate the combustor inlet conditions of CST aircraft engines. A conventional Jet A fuel was used as the baseline fuel, to which a SAF was compared. Results show that a moderate level of prevaporization and premixing was sufficient to properly stabilize the premixed main flames. With reduced prevaporization and premixing, the main flames did not properly stabilize and NOx emissions were increased. With i...</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>1. Turbulence-chemistry interaction in a GT model combustor via simultaneous high-speed CARS and PIV (Combustion and Flame, 2023) | 2. Simultaneous high-speed OH-PLIF and stereo-PIV of turbulent premixed flames at elevated pressure (Proc. Combustion Institute, 2021)</t>
+          <t>1. Impact of pilot injections on ducted fuel injection performance (International Journal of Engine Research, 2026) | 2. Lean Blowoff Limits and Emissions Measurements in a Lean Premixed Prevaporized Combustor with Variable Reactant Inhomogeneity (2026)</t>
         </is>
       </c>
       <c r="X4" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2023.112754 | https://doi.org/10.1016/j.proci.2020.06.149", "https://doi.org/10.1016/j.combustflame.2023.112754 | https://doi.org/10.1016/j.proci.2020.06.149")</f>
+        <f>HYPERLINK("https://doi.org/10.1177/14680874261426780 | https://doi.org/10.2514/6.2026-0384", "https://doi.org/10.1177/14680874261426780 | https://doi.org/10.2514/6.2026-0384")</f>
         <v/>
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>deploying simultaneous 5 kHz dual-pump CARS and stereo-PIV in a swirl combustor, demonstrating that local extinction events co-locate with strain-rate regions where Ka &gt; 50 and that re-ignition traces preferentially the trailing edges of high-scalar-dissipation tubes.</t>
+          <t>investigating the coupling of ducted fuel injection (DFI) with pilot injections in high-pressure diesel combustion, demonstrating that DFI reduces flame spatially integrated natural luminosity (SINL) by 30-70% and pilot injection mitigates peak SINL by a further 16%.</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr">
@@ -7203,64 +7195,64 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Quantitative laser diagnostics for high-enthalpy reacting flows -- PLIF-based scalar measurements, dual-pump CARS thermometry, and two-photon LIF for atomic species in high-pressure combustion, shock tunnels, and detonation chambers.</t>
+          <t>Advanced planar laser-induced fluorescence (PLIF) diagnostics for elevated-pressure reacting flows, lean blowoff proximity sensing, and multi-species optical imaging in swirl-stabilized spray flames.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Planar Laser-Induced Fluorescence (PLIF), Dual-pump CARS, Two-photon atomic LIF, High-speed intensified CCD, Shock tube/detonation chamber diagnostics</t>
+          <t>Single-laser CH/OH/fuel PLIF, Longpass intra-vibrational band optical filtering, High-pressure combustor rigs (9 bar), Lean blowout acoustic/optical sensing</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Quantitative PLIF imaging of OH* chemiluminescence in detonation-driven flows</t>
+          <t>Lean Blowoff Limits and Emissions Measurements in a Lean Premixed Prevaporized Combustor with Variable Reactant Inhomogeneity</t>
         </is>
       </c>
       <c r="P5" s="3">
-        <f>HYPERLINK("https://doi.org/10.1088/1361-6501/ac4b21", "https://doi.org/10.1088/1361-6501/ac4b21")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0384", "https://doi.org/10.2514/6.2026-0384")</f>
         <v/>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>applying quantitative OH* PLIF with dual-pump CARS quenching correction behind H2-air detonation fronts, demonstrating that post-detonation OH* overshoots equilibrium concentration by 2.3x due to ZND induction-zone kinetic excess, fully resolved at 200 um spatial resolution.</t>
+          <t>evaluating lean blowoff limits and emissions in an LPP combustor operating at 700 K and 9 bar under variable reactant inhomogeneity, demonstrating that prevaporization uniformity dictates flame stabilization and prevents severe NOx emission surges.</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>A quantitative PLIF diagnostic for excited-state OH* is developed and applied to detonation-driven supersonic combustion flows. The diagnostic accounts for collisional quenching corrections using simultaneous dual-pump CARS measurements. Applied to a H2-air detonation tube, OH* PLIF images resolve the thin reaction zone behind the detonation front with 200 um spatial resolution. OH* signal peaks at 2.3x the equilibrium post-detonation value, indicating strong kinetic overshoot driven by ZND induction zone chemistry.</t>
+          <t>Lean premixed prevaporized (LPP) combustor designs and sustainable aviation fuels (SAF) show great promise for the development of next-generation low-emission civil supersonic transport (CST) aircraft engines. In this work, exhaust emissions sampling and optical diagnostic measurements were conducted in an LPP model combustor with variable reactant inhomogeneity. The LPP combustor features a novel premixer design, which facilitates control of the level of fuel vaporization and fuel-air mixedness entering the combustor. Measurements of lean blowoff (LBO) limits and gaseous emissions trends were obtained through the optically accessible combustor liner and custom exhaust sampling probe. The combustor was operated at elevated temperature (700 K) and pressure (9 bar) conditions to simulate the combustor inlet conditions of CST aircraft engines. A conventional Jet A fuel was used as the baseline fuel, to which a SAF was compared. Results show that a moderate level of prevaporization and premixing was sufficient to properly stabilize the premixed main flames. With reduced prevaporization and premixing, the main flames did not properly stabilize and NOx emissions were increased. With i...</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>Two-temperature analysis of non-equilibrium N2 vibrational excitation in hypersonic arcjet flows</t>
+          <t>Single-laser CH, OH and fuel PLIF in a pressurized swirl-stabilized spray flame</t>
         </is>
       </c>
       <c r="T5" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.T6072", "https://doi.org/10.2514/1.T6072")</f>
+        <f>HYPERLINK("https://doi.org/10.1016/j.proci.2026.106104", "https://doi.org/10.1016/j.proci.2026.106104")</f>
         <v/>
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>measuring two-photon LIF vibrational temperatures across a Mach 5-7 arcjet freestream, demonstrating N2 vibrational temperatures exceed translational by 1800-2400 K and Park finite-rate model under-predicts vibrational relaxation in the expansion fan by 28%.</t>
+          <t>demonstrating single-laser simultaneous CH, OH, and fuel PLIF in a pressurized swirl-stabilized spray flame at 310.7 nm, revealing that pressure-induced collisional broadening allows clean separation of thin CH reaction zones from dense liquid spray droplet fluorescence.</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>Non-equilibrium vibrational excitation of N2 in a high-enthalpy arcjet flow simulating Mars entry conditions is investigated using two-photon LIF and optical emission spectroscopy. Measured vibrational temperatures exceed translational temperatures by 1800-2400 K across Mach 5-7 test conditions. Agreement with LAURA CFD predictions using Park rate model is within 12% in the freestream but degrades to 28% in the expansion fan region.</t>
+          <t>This paper explores the use of planar laser-induced fluorescence (PLIF) with excitation wavelengths in the R-branch of the CH C 2 Σ + − X 2 Π ( 0,0 ) in a liquid-fueled combustor at elevated pressures. Following the atmospheric pressure work of Hammack et al. Appl. Phys. B 124:34 (2018), longpass intra-vibrational band filtering was used to isolate CH PLIF, OH PLIF, and fuel signals from the laser scattering. CH PLIF images were obtained by targeting CH R-branch transitions at 310.69 nm and 311.18 nm. Interference from fuel fluorescence was mitigated through the use of a low-aromatic content synthetic aviation fuel, though it was still significant where liquid was present. Nevertheless, the CH layers in the reaction zone were distinguishable from the droplet signal even in the dense spray near the fuel injector. OH PLIF images could be obtained without CH interference using the same setup, but targeting the OH Q-branch transitions of the A − X ( 0,0 ) band at 310.75 nm. Furthermore, due to pressure-induced collisional broadening, simultaneous CH and OH PLIF could be imaged on a single frame when the laser wavelength was tuned in the vicinity of either CH R-branch transition. The...</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>1. Quantitative PLIF imaging of OH* chemiluminescence in detonation-driven flows (MST, 2022) | 2. Two-temperature analysis of non-equilibrium N2 in hypersonic arcjet flows (JTHT, 2021)</t>
+          <t>1. Lean Blowoff Limits and Emissions Measurements in a Lean Premixed Prevaporized Combustor with Variable Reactant Inhomogeneity (2026) | 2. Single-laser CH, OH and fuel PLIF in a pressurized swirl-stabilized spray flame (Proceedings of the Combustion Institute, 2026)</t>
         </is>
       </c>
       <c r="X5" s="3">
-        <f>HYPERLINK("https://doi.org/10.1088/1361-6501/ac4b21 | https://doi.org/10.2514/1.T6072", "https://doi.org/10.1088/1361-6501/ac4b21 | https://doi.org/10.2514/1.T6072")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0384 | https://doi.org/10.1016/j.proci.2026.106104", "https://doi.org/10.2514/6.2026-0384 | https://doi.org/10.1016/j.proci.2026.106104")</f>
         <v/>
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>applying quantitative OH* PLIF with dual-pump CARS quenching correction behind H2-air detonation fronts, demonstrating that post-detonation OH* overshoots equilibrium concentration by 2.3x due to ZND induction-zone kinetic excess, fully resolved at 200 um spatial resolution.</t>
+          <t>evaluating lean blowoff limits and emissions in an LPP combustor operating at 700 K and 9 bar under variable reactant inhomogeneity, demonstrating that prevaporization uniformity dictates flame stabilization and prevents severe NOx emission surges.</t>
         </is>
       </c>
       <c r="Z5" s="2" t="inlineStr">
@@ -7403,64 +7395,64 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>High-fidelity RANS/hybrid RANS-LES aeromechanics simulation of helicopter rotors and wind turbines -- capturing dynamic stall vortex shedding, rotor-wake interaction, and blade-vortex interaction noise to reduce vibration and acoustic emissions in next-generation rotorcraft.</t>
+          <t>Aeroacoustics DNS of high-amplitude acoustic transmission and inverse airfoil design for roughness-tolerant low-drag wind and hydrokinetic turbine blades.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Hybrid RANS-LES (DDES), Overset Chimera grids, Dynamic mesh motion, CAMRAD II structural coupling, Gradient boosted trees (dynamic stall onset ML)</t>
+          <t>Direct Numerical Simulation (DNS) aeroacoustics, Impedance tube testing (120-150 dB), Inverse airfoil aerodynamic design, Blade Element Momentum (BEM) turbine codes</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Dynamic Stall Onset Prediction and Modeling Using Machine Learning on CFD-Generated Datasets</t>
+          <t>Transmission of high-amplitude sound through leakages of ill-fitting earplugs</t>
         </is>
       </c>
       <c r="P6" s="3">
-        <f>HYPERLINK("https://doi.org/10.4050/JAHS.68.032001", "https://doi.org/10.4050/JAHS.68.032001")</f>
+        <f>HYPERLINK("https://doi.org/10.1177/1475472x261473636", "https://doi.org/10.1177/1475472x261473636")</f>
         <v/>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>training gradient-boosted classifiers on 4.1M URANS time steps across 15,000 airfoil conditions, demonstrating 94.2% accuracy in predicting dynamic stall onset 3 convective time units in advance and reducing full-rotor vibration estimation error from 31% to 9%.</t>
+          <t>combining impedance-tube experiments with DNS of high-amplitude acoustic transmission (120-150 dB) across 1-5 kHz, demonstrating that ill-fitting earplug leakages reduce transmission loss by ~18 dB at 120 dB incident SPL.</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>Machine learning models trained on 4.1 million time steps from URANS simulations across 15,000 operating conditions achieve 94.2% accuracy in predicting dynamic stall onset 3 convective time units in advance. The ML-based predictor integrated into a blade element momentum model reduces dynamic stall-induced vibration estimation error from 31% to 9% relative to pure BEMT.</t>
+          <t>Exposure to high sound pressure levels (SPL) is a leading cause of noiseinduced hearing loss, and earplugs are a primary means of protection. The effectiveness of earplug protection depends on the seal formed in the ear canal. An ill-fitting earplug leaves air gaps that leak sound and degrade attenuation. The acoustics of these leak paths and their dissipation mechanisms under high-amplitude sound remain poorly characterized. This study quantifies sound transmission through modeled earplug leakage with rigid-wall idealization and identifies the governing dissipation mechanisms by combining impedance-tube experiments and direct numerical simulation (DNS). The methods were first verified against stand-alone slit resonators and orifices, for which extensive published data are available, and then used to measure the transmission loss (TL) and acoustic power absorption coefficient of modeled earplug–canal configurations over 1–5 kHz at overall incident SPLs of 120–150 dB. Leakage from an ill-fitting silicone rubber earplug reduced its TL by approximately 18 dB relative to a sealed configuration at an overall incident sound pressure levels (OISPL) of 120 dB, and the leakage-path TL in...</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>Computational Investigation of Rotor-Fuselage Interactional Aerodynamics Using Hybrid RANS-LES</t>
+          <t>Design and Use of Roughness-Tolerant Low Drag Airfoils for Wind Turbine and Hydrokinetic Turbine Applications</t>
         </is>
       </c>
       <c r="T6" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.J060183", "https://doi.org/10.2514/1.J060183")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0480", "https://doi.org/10.2514/6.2026-0480")</f>
         <v/>
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>simulating rotor-fuselage interactional aerodynamics via DDES on overset grids at advance ratio mu = 0.15, demonstrating that recirculation below the hub increases rotor torque by 4.7% and produces wake-fuselage surface pressure fluctuations of 0.08 Cp matching experimental data.</t>
+          <t>applying inverse design to develop roughness-tolerant airfoils with laminar drag buckets across wide lift coefficients, demonstrating preserved profile efficiency under surface dirt and icing degradation in wind and tidal turbines.</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>The interactional aerodynamics between a helicopter main rotor and fuselage is investigated using DDES on overset grids. Rotor-fuselage interaction produces a recirculation region below the hub that increases rotor torque requirement by 4.7%. Unsteady wake-fuselage impingement creates surface pressure fluctuations of 0.08 Cp, consistent with Georgia Tech Aeroflite wind tunnel measurements.</t>
+          <t>Wind turbines and hydrokinetic turbines are designed to use laminar airfoils that provide maximum power at the rated speed. During day-to-day operations, the blade surface may be degraded due to accumulation of dirt and icing on the pressure side, in addition to development of scratches or other surface imperfections. As a result, the profile power losses would increase, reducing the available power over a broad range of operating conditions. In this work, an inverse design approach has been employed to generate roughness tolerant airfoils that exhibit a laminar drag bucket for a broad range of lift coefficients. Two-dimensional drag polars are presented for smooth and rough airfoils and compared to NACA airfoils of comparable thickness. A limited number of three-dimensional studies based on combined blade element-momentum theory are also presented for several wind and tidal turbines for a broad range of rated power conditions.</t>
         </is>
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>1. Dynamic Stall Onset Prediction Using Machine Learning on CFD Datasets (JAHS, 2023) | 2. Computational Investigation of Rotor-Fuselage Interactional Aerodynamics Using Hybrid RANS-LES (AIAA J., 2021)</t>
+          <t>1. Transmission of high-amplitude sound through leakages of ill-fitting earplugs (International Journal of Aeroacoustics, 2026) | 2. Design and Use of Roughness-Tolerant Low Drag Airfoils for Wind Turbine and Hydrokinetic Turbine Applications (2026)</t>
         </is>
       </c>
       <c r="X6" s="3">
-        <f>HYPERLINK("https://doi.org/10.4050/JAHS.68.032001 | https://doi.org/10.2514/1.J060183", "https://doi.org/10.4050/JAHS.68.032001 | https://doi.org/10.2514/1.J060183")</f>
+        <f>HYPERLINK("https://doi.org/10.1177/1475472x261473636 | https://doi.org/10.2514/6.2026-0480", "https://doi.org/10.1177/1475472x261473636 | https://doi.org/10.2514/6.2026-0480")</f>
         <v/>
       </c>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>training gradient-boosted classifiers on 4.1M URANS time steps across 15,000 airfoil conditions, demonstrating 94.2% accuracy in predicting dynamic stall onset 3 convective time units in advance and reducing full-rotor vibration estimation error from 31% to 9%.</t>
+          <t>combining impedance-tube experiments with DNS of high-amplitude acoustic transmission (120-150 dB) across 1-5 kHz, demonstrating that ill-fitting earplug leakages reduce transmission loss by ~18 dB at 120 dB incident SPL.</t>
         </is>
       </c>
       <c r="Z6" s="2" t="inlineStr">
@@ -7603,64 +7595,64 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Hall-effect thruster plume physics, near-anode ionization instabilities, and plasma-neutral coupling in electric propulsion -- combining laser-induced fluorescence velocimetry, Langmuir probe arrays, and particle-in-cell simulations to push CubeSat and deep-space thruster efficiency boundaries.</t>
+          <t>Hall-effect thruster plasma physics, heaterless hollow cathode operation on alternative propellants (krypton/argon), and laser Thomson scattering electron dynamics in magnetically shielded thrusters.</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Laser-Induced Fluorescence (LIF) velocimetry (Xe II lines), Langmuir and Faraday probes, Retarding Potential Analyzer (RPA), E×B probe, Particle-in-Cell (PIC) simulations</t>
+          <t>Laser Thomson Scattering, Steady-state I-V cathode characterization, Magnetically shielded Hall thruster testing (H9 9 kW), Vacuum Test Facilities (VTF-2)</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Azimuthal Ion Velocity Measurements in a Hall Thruster via Laser-Induced Fluorescence</t>
+          <t>Characterization of a heaterless 60 A hollow cathode on krypton and argon</t>
         </is>
       </c>
       <c r="P7" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.B38688", "https://doi.org/10.2514/1.B38688")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s44205-026-00221-w", "https://doi.org/10.1007/s44205-026-00221-w")</f>
         <v/>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>measuring azimuthal Xe II ion velocities via dual-geometry LIF in a Hall thruster near-field plume, demonstrating that azimuthal swirl reaches 2.1-3.8 km/s (11-19% of exit velocity) and correlates with 15-20 kHz breathing mode oscillations that reduce effective specific impulse.</t>
+          <t>characterizing a 60 A heaterless hollow cathode on krypton and argon in the 9 kW H9 thruster, demonstrating that magnetic fields systematically increase steady-state discharge voltage by up to +159% (+67.5 V) on argon at fixed current rather than reducing it.</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>Azimuthal ion velocity measurements in the near-field plume of a Hall-effect thruster are reported using LIF velocimetry of Xe II lines. Peak swirl velocities of 2.1-3.8 km/s correspond to 11-19% of total ion exit velocity. These azimuthal components correlate with low-frequency breathing mode oscillations at 15-20 kHz and indicate non-trivial angular momentum deposition that degrades effective thruster specific impulse.</t>
+          <t>Abstract We present a steady-state current-voltage (IV) characterization of a heaterless version of the 9 kW-class H9 Hall thruster cathode. This work was conducted at Georgia Tech’s High-Power Electric Propulsion Laboratory (HPEPL) at operational background pressures of 0.22–0.70 µTorr on krypton and 0.11–0.24 µTorr on argon, with a base pressure of 9.1 × 10 − 8 Torr. The characterization mapped steady-state voltage behavior from 5 to 45 A of discharge current on krypton and 5 to 30 A on argon (with paired magnetized and unmagnetized data over 5 to 35 A on krypton and 5 to 20 A on argon), in both magnetized and unmagnetized configurations. The magnetized configuration produced a higher discharge voltage than the unmagnetized configuration at every paired (current, flow) operating point on both propellants. On krypton, the magnetized-unmagnetized voltage gap ranged from near zero at the highest cathode flow and lowest current to + 39.6 V (+ 148%) at 30 A and 12.39 sccm. On argon, the gap ranged from + 6.0 V at 15 A and 12.39 sccm to + 67.5 V (+ 159%) at 20 A and 15.89 sccm. In both cases, the gap widened with discharge current and narrowed with cathode flow. These results verify reproducible ignition at every tested flow rate, confirm uninterrupted steady-state heaterless operation on krypton and argon, and quantify how the applied magnetic field shifts the steady-state operating point at fixed discharge current. The key finding is that the applied magnetic field increases the steady-state discharge voltage at fixed current rather than reducing it, and the effect is systematically larger on argon than on krypton at matched operating conditions.</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>Near-Field Plume Characterization of a 200-W Hall Thruster via Electrostatic Probes</t>
+          <t>Effect of body bias on near-field electron behavior in a magnetically shielded Hall thruster</t>
         </is>
       </c>
       <c r="T7" s="3">
-        <f>HYPERLINK("https://doi.org/10.1007/s44205-023-00045-z", "https://doi.org/10.1007/s44205-023-00045-z")</f>
+        <f>HYPERLINK("https://doi.org/10.1063/5.0340395", "https://doi.org/10.1063/5.0340395")</f>
         <v/>
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>deploying 2D electrostatic probe arrays in a 200-W Hall thruster near-field plume, demonstrating that bimodal IEDFs at 5 cm downstream directly evidence charge-exchange collisions that broaden plume divergence by 6.8 degrees beyond the accelerated-ion beam.</t>
+          <t>deploying spatially resolved laser Thomson scattering in the near-field of the 9 kW H9 Hall thruster at 40 A, demonstrating that +2 V body bias inverts electron density topology between the cathode centerline (3.4e19 m^-3) and channel centerline (9.0e17 m^-3).</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>A comprehensive electrostatic probe characterization of the near-field plume of a 200-W Hall thruster is reported. The IEDF at 5 cm downstream reveals a bimodal structure with a cold (&lt;10 eV) charge-exchange peak and a hot (120-180 eV) direct-acceleration peak, providing direct evidence for near-field charge exchange collisions that broaden plume divergence by 6.8 degrees.</t>
+          <t>This work investigates the influence of thruster body bias on near-field electron behavior in a magnetically shielded Hall effect thruster (HET) through spatially resolved laser Thomson scattering diagnostics. Experiments were conducted on the 9 kW class H9 magnetically shielded HET operating at 40 A discharge current and 150 V discharge voltage on krypton propellant in the Georgia Tech Vacuum Test Facility 2. Three electrical configurations were examined: floating (body electrically isolated), cathode-tied (body at cathode potential, approximately −10.3 V relative to facility ground), and +2 V bias (body biased +2 V relative to ground). Spatially resolved measurements of electron density, electron temperature, and radial electron bulk velocity were obtained at up to 23 locations (a 15-point radial grid and up to eight axial stations along the cathode centerline) spanning the cathode near-field from the cathode centerline to the discharge channel centerline. A configuration-dependent spatial density inversion reveals distinct circuit topologies: at z/r0 = 0.029, cathode-tied elevates ne at the cathode centerline (4.4 × 1019 m−3) while exhibiting the lowest channel-centerline density (6.6 × 1017 m−3), whereas the +2 V configuration shows the opposite pattern (3.4 × 1019 and 9.0 × 1017 m−3, respectively). The +2 V configuration exhibits the lowest Te at the inner front pole cover, consistent with magnetization-limited, energy-selective electron collection. Electron pressure does not serve as a reliable proxy for electrostatic potential in this near-field region due to unmeasured anomalous transport terms.</t>
         </is>
       </c>
       <c r="W7" s="2" t="inlineStr">
         <is>
-          <t>1. Azimuthal Ion Velocity Measurements in a Hall Thruster via Laser-Induced Fluorescence (JPP, 2022) | 2. Near-Field Plume Characterization of a 200-W Hall Thruster via Electrostatic Probes (JEP, 2023)</t>
+          <t>1. Characterization of a heaterless 60 A hollow cathode on krypton and argon (Journal of Electric Propulsion, 2026) | 2. Effect of body bias on near-field electron behavior in a magnetically shielded Hall thruster (Journal of Applied Physics, 2026)</t>
         </is>
       </c>
       <c r="X7" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.B38688 | https://doi.org/10.1007/s44205-023-00045-z", "https://doi.org/10.2514/1.B38688 | https://doi.org/10.1007/s44205-023-00045-z")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s44205-026-00221-w | https://doi.org/10.1063/5.0340395", "https://doi.org/10.1007/s44205-026-00221-w | https://doi.org/10.1063/5.0340395")</f>
         <v/>
       </c>
       <c r="Y7" s="2" t="inlineStr">
         <is>
-          <t>measuring azimuthal Xe II ion velocities via dual-geometry LIF in a Hall thruster near-field plume, demonstrating that azimuthal swirl reaches 2.1-3.8 km/s (11-19% of exit velocity) and correlates with 15-20 kHz breathing mode oscillations that reduce effective specific impulse.</t>
+          <t>characterizing a 60 A heaterless hollow cathode on krypton and argon in the 9 kW H9 thruster, demonstrating that magnetic fields systematically increase steady-state discharge voltage by up to +159% (+67.5 V) on argon at fixed current rather than reducing it.</t>
         </is>
       </c>
       <c r="Z7" s="2" t="inlineStr">
@@ -7787,64 +7779,64 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>LES-driven combustion instability modeling, turbulent premixed flame propagation, and plasma-assisted ignition in gas-turbine and scramjet combustors — advancing high-fidelity reacting-flow simulation from laboratory-scale flames to full annular combustion chambers.</t>
+          <t>Large eddy simulations (LES) of turbulent combustion, hybrid transported-tabulated chemistry (HTTC), and soot aerosol dynamics in rich-burn quick-mix lean-burn (RQL) and rotating detonation combustors.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Large Eddy Simulation (LES) with LDK subgrid closure, PRISM tabulated chemistry, Spray Lagrangian tracking, DNS of premixed flame kernels</t>
+          <t>Large Eddy Simulation (LES), Hybrid Transported-Tabulated Chemistry (HTTC), Dynamic subgrid closures, PAH-based soot modeling, Partially stirred reactor (PaSR)</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Subgrid combustion modeling for large eddy simulation of spray combustion in turbulent swirling flows</t>
+          <t>Application of Hybrid Transported-Tabulated Chemistry for Efficient Large-Eddy Simulation of Turbulent Combustion</t>
         </is>
       </c>
       <c r="P8" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2021.111634", "https://doi.org/10.1016/j.combustflame.2021.111634")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s10494-026-00794-4", "https://doi.org/10.1007/s10494-026-00794-4")</f>
         <v/>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>coupling Lagrangian spray dynamics with LES dynamic subgrid combustion in a bluff-body swirl combustor, demonstrating that droplet evaporation controls inner-recirculation-zone flame anchoring and produces unsteady heat-release fluctuations at Strouhal numbers consistent with observed thermoacoustic instabilities.</t>
+          <t>implementing a hybrid transported-tabulated chemistry (HTTC) strategy in LES of turbulent combustion with 29 species and 141 steps, demonstrating up to 11-fold computational speedup while maintaining high fidelity in predicting extinction and re-ignition dynamics.</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>A subgrid combustion model for large eddy simulation of spray combustion in turbulent swirling flows is developed and validated. The model is based on the localized dynamic K-equation (LDK) subgrid kinetic energy closure combined with a progress variable approach for turbulent premixed combustion. Two-phase spray effects are modeled using a Lagrangian particle tracking approach coupled to the LES gas-phase solver. The combined model is applied to a bluff-body stabilized swirl combustor and validated against experimental measurements of velocity, temperature, and species concentrations. Simulations reveal that liquid fuel droplet evaporation and transport profoundly alter local flame structure and stabilization mechanisms, particularly near the inner recirculation zone where unsteady flame-vortex interactions dominate heat release distribution.</t>
+          <t>Abstract The performance of a hybrid transported-tabulated chemistry (HTTC) strategy is evaluated for large-eddy simulations (LES) of turbulent combustion with detailed finite-rate kinetics. The computational cost of LES is reduced in the HTTC approach by segregating the species list into major and minor species, with the former transported and the latter tabulated. Apart from reducing the number of transported species, the HTTC approach and its variants decrease computational cost by enabling efficient computation of thermodynamics and transport properties and by relieving the stiffness of chemical source terms. The calculations can be up to 11 times faster with stiff kinetics (29 species, 141 steps), as the HTTC approach eliminates the need to integrate and transport the minor species, which typically have short chemical times. The original HTTC and other variants are assessed for their accuracy, efficiency, and robustness for LES by considering two temporally evolving challenging test cases: a freely propagating turbulent premixed flame in the thin reaction zone regime and a turbulent non-premixed jet flame exhibiting local extinction and re-ignition. Modifications to the original HTTC approach are considered and evaluated to account for the effect of subgrid-scale turbulence. Both a priori and a posteriori analyses are conducted to evaluate the accuracy of the HTTC approach. The turbulent premixed flame test shows noticeable yet small differences between the calculated and tabulated concentrations of minor species. This results in reasonable predictions of reaction rates and overall combustion process with HTTC. The difference between calculated and tabulated minor species concentrations is larger for the turbulent non-premixed flame case; however, the minor species concentrations are generally much lower for it, and therefore, extinction-re-ignition physics is still predicted well with HTTC.</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>Effects of multi-fuel blending on combustion characteristics of turbulent premixed swirling flames</t>
+          <t>Large-Eddy Simulations of Soot Formation and Dispersion in Rich-Burn Quick-Mix Lean-Burn (RQL) Spray Combustor</t>
         </is>
       </c>
       <c r="T8" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.proci.2022.07.034", "https://doi.org/10.1016/j.proci.2022.07.034")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2025-2484", "https://doi.org/10.2514/6.2025-2484")</f>
         <v/>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>performing LES with PRISM tabulated chemistry across methane-hydrogen blends (0-60% H2 by volume) in a swirl combustor, demonstrating that hydrogen enrichment amplifies local laminar flame speed by up to 48% and activates preferential diffusion wrinkling that reshapes thermoacoustic coupling frequencies.</t>
+          <t>performing LES with a Lagrangian spray and PAH soot kinetics in an RQL combustor at 6.8 atm, demonstrating that shifting global equivalence ratio from 0.12 to 0.2 markedly increases primary-zone soot volume fraction through localized flame-spray-soot interactions.</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t>The effects of fuel composition on turbulent premixed combustion characteristics of swirling flames are investigated using high-fidelity large eddy simulations (LES). Three fuel blends of methane and hydrogen (0%, 30%, and 60% H2 by volume) are studied in a gas turbine model combustor at atmospheric pressure. The LES employs a dynamic localized combustion model with detailed chemistry tabulation via PRISM. Increased hydrogen fraction accelerates local flame propagation by up to 48%, narrows the reaction zone, and triggers preferential diffusion-driven flame wrinkling at small scales, with direct consequence for NOx formation pathways.</t>
+          <t>The influence of varying fuel/air ratios on the primary zone soot formation characteristics of the liquid-fueled rich-quench-lean (RQL) combustor is investigated numerically. Large- eddy simulations (LES) of two global equivalence ratios (��) corresponding to 0.12 and 0.2 respectively are conducted at an overall pressure of 6.8 atm. The employed LES modeling framework includes Lagrangian treatment for liquid-fuel spray, finite-rate chemistry for gas- phase combustion, a polycyclic aromatic hydrocarbon (PAH)-based soot model, a partially stirred reactor model for turbulence-soot-chemistry interactions, and an optically thin radiation model. The soot and gas-phase chemistry modeling framework is verified against the experimental measurements from canonical premixed and non-premixed flames of gaseous ethylene fuels. The LES simulations of the RQL combustor qualitatively demonstrate the trend of increasing soot volume fractions (SVFs) under the two conditions investigated in this work. Further analysis of local flame-soot-spray interactions and soot source terms is reported to explain the observed differences.</t>
         </is>
       </c>
       <c r="W8" s="2" t="inlineStr">
         <is>
-          <t>1. Subgrid combustion modeling for LES of spray combustion in turbulent swirling flows (Combustion and Flame, 2022) | 2. Effects of multi-fuel blending on combustion of turbulent premixed swirling flames (Proc. Combustion Institute, 2023)</t>
+          <t>1. Application of Hybrid Transported-Tabulated Chemistry for Efficient Large-Eddy Simulation of Turbulent Combustion (Flow Turbulence and Combustion, 2026) | 2. Large-Eddy Simulations of Soot Formation and Dispersion in Rich-Burn Quick-Mix Lean-Burn (RQL) Spray Combustor (2025)</t>
         </is>
       </c>
       <c r="X8" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.combustflame.2021.111634 | https://doi.org/10.1016/j.proci.2022.07.034", "https://doi.org/10.1016/j.combustflame.2021.111634 | https://doi.org/10.1016/j.proci.2022.07.034")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s10494-026-00794-4 | https://doi.org/10.2514/6.2025-2484", "https://doi.org/10.1007/s10494-026-00794-4 | https://doi.org/10.2514/6.2025-2484")</f>
         <v/>
       </c>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>coupling Lagrangian spray dynamics with LES dynamic subgrid combustion in a bluff-body swirl combustor, demonstrating that droplet evaporation controls inner-recirculation-zone flame anchoring and produces unsteady heat-release fluctuations at Strouhal numbers consistent with observed thermoacoustic instabilities.</t>
+          <t>implementing a hybrid transported-tabulated chemistry (HTTC) strategy in LES of turbulent combustion with 29 species and 141 steps, demonstrating up to 11-fold computational speedup while maintaining high fidelity in predicting extinction and re-ignition dynamics.</t>
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr">
@@ -7983,64 +7975,64 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Thermoacoustic instability theory, turbulent flame linear response functions, and hydrodynamic wavemaker identification in low-NOx combustors -- building physics-based predictive frameworks for acoustic-flame coupling in next-generation gas turbines and hydrogen-fueled engines.</t>
+          <t>Combustion dynamics, swirl burner flame stability, low-carbon ammonia (NH3) rich-relaxation-quench-lean (RRQL) combustion systems, and turbulence sensitivity of NOx/CO emissions in hydrogen-methane blends.</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>High-speed OH-PLIF, Acoustic forcing rigs (transverse/longitudinal), Phase-locked PIV, Global flame transfer function measurement, Wavemaker stability analysis</t>
+          <t>High-speed OH*/NH2* chemiluminescence, Modular swirl burners, Gas-phase emissions sampling (NOx, N2O, NH3, CO), Turbulence-flame interaction rigs</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Flame Transfer Function Measurement of a Transversely Excited Swirling Flame</t>
+          <t>Toward the Development of an RRQL System—Part I: Swirl Pattern Effect on Exhaust Emissions and Chemiluminescence Distribution for NH3–Air Premixed Swirl Flames</t>
         </is>
       </c>
       <c r="P9" s="3">
-        <f>HYPERLINK("https://doi.org/10.1115/1.4053164", "https://doi.org/10.1115/1.4053164")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/1.4069796", "https://doi.org/10.1115/1.4069796")</f>
         <v/>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>measuring transverse flame transfer functions via phase-locked OH-PLIF in a swirl-stabilized combustor, demonstrating that transverse excitation produces peak gain at the swirler geometric resonance rather than the convective residence time, directly altering annular combustor thermoacoustic stability predictions.</t>
+          <t>investigating swirl geometry effects on flame morphology and emissions in rich premixed NH3-air flames for an RRQL system, demonstrating that compact flames minimize wall quenching and enable post-flame relaxation to suppress NOx and NH3 emissions.</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>This paper presents measurements of the flame transfer function (FTF) of a swirl-stabilized flame excited by transverse acoustic forcing. Using phase-locked OH-PLIF and acoustic pressure measurements, the FTF relating heat release rate fluctuations to transverse velocity perturbations is characterized over 100-600 Hz. Results show that the transverse FTF exhibits a substantially different gain-phase structure than the longitudinal FTF, with peak gain at frequencies near the swirler geometric resonance rather than the convective time scale.</t>
+          <t>Abstract Ammonia (NH3) is a carbon–free energy source and hydrogen carrier, but its fuel–bound nitrogen can lead to significant nitrogen oxides (NOx) emissions. Staged combustion strategies, such as rich–quench–lean, can achieve low NOx emissions. However, improper design may result in high NOx levels when operating with a rich head end without a sufficient post–flame relaxation time. Previous work has shown that a rich–relaxation–quench–lean (RRQL) configuration can minimize NOx emissions in the rich head end (Cole et al., 2024, “Rich Ammonia Flame Shapes and NO Relaxation: Facility Development and Characterization,” ASME Paper No. GT2024–122369). This study focuses on how different swirl geometries affect exhaust emissions and flame morphology in rich, premixed NH3–air flames, for the design of a rich relaxation head end of an RRQL combustor. Experiments were conducted using a modular swirl burner and measuring NOx, N2O, and NH3 emissions, and recording natural flame luminosity and NH2* and OH* chemiluminescence images. Swirler design affects emissions by influencing flame length (with shorter flames allowing for more postflame relaxation time) and flame–wall interactions (influencing NH3 and N2O emissions). A compact flame with minimal wall interactions allows for increased NOx relaxation, while minimal wall interactions prevent heat losses and instabilities, which minimize NH3 and N2O emissions at a richer equivalence ratio, potentially enhancing H2 production during the relaxation phase without increasing overall primary stage NOx emissions, thereby improving system efficiency. Detailed spatial evolution of NOx, N2O, and NH3 emissions further supports the RRQL as a promising combustor design for NH3 combustion, if the rich head end is designed properly.</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Hydrodynamic stability of reacting swirling jets</t>
+          <t>Measurements of CO and NOx Emissions From Premixed Turbulent Methane/Hydrogen Flames</t>
         </is>
       </c>
       <c r="T9" s="3">
-        <f>HYPERLINK("https://doi.org/10.1017/jfm.2021.433", "https://doi.org/10.1017/jfm.2021.433")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/1.4069625", "https://doi.org/10.1115/1.4069625")</f>
         <v/>
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>performing global wavemaker stability analysis of reacting swirling jets across varying equivalence ratios, demonstrating that combustion heat release simultaneously destabilizes the axisymmetric (m=0) centrifugal mode and suppresses the precessing vortex core (m=+-1) helical instability branch.</t>
+          <t>measuring the sensitivity of NO and CO emissions from turbulent premixed H2/CH4 flames across varying turbulence intensities, demonstrating that H2 enrichment sharply accelerates CO relaxation toward equilibrium while turbulence intensity yields negligible impact on NO at constant CO.</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
         <is>
-          <t>The hydrodynamic stability of reacting swirling jets is investigated using global stability analysis and wavemaker identification. Structural sensitivity analysis reveals a confined wavemaker region near the central recirculation zone boundary. Two competing instability branches are identified: an axisymmetric (m=0) branch driven by centrifugal destabilization and a helical (m=+-1) branch associated with the precessing vortex core (PVC). Increased heat release from combustion destabilizes the m=0 mode and simultaneously stabilizes the PVC branch.</t>
+          <t>Abstract This paper presents measurements of the sensitivity of NO and CO emissions from H2/CH4 combustion to variations in turbulence intensity. Existing studies of exhaust emissions either focus on laminar modeling and measurements or report device-level measurements from practical combustors. However, there are limited fundamental studies of emissions characteristics of turbulent systems, the focus of this study. Because of the strong stretch sensitivity of these mixtures, local temperatures/reaction rates along the turbulent front can differ markedly from mixture-averaged properties, and they are very sensitive to turbulence. Single-point emissions measurements are presented for turbulent premixed H2/CH4 flames from a contoured nozzle Bunsen burner with variable turbulence. Emissions are measured at varying residence times and incoming flow turbulence intensities. Data show the clear benefit of H2 blending on CO emissions, both due to the expected reduction in C atoms, but also due to faster relaxation of flame generated CO toward equilibrium. It also shows negligible impact of turbulence intensity on NO emissions at constant CO for CH4.</t>
         </is>
       </c>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>1. Flame Transfer Function of a Transversely Excited Swirling Flame (JEGTP, 2022) | 2. Hydrodynamic stability of reacting swirling jets (Journal of Fluid Mechanics, 2021)</t>
+          <t>1. Toward the Development of an RRQL System—Part I: Swirl Pattern Effect on Exhaust Emissions and Chemiluminescence Distribution for NH3–Air Premixed Swirl Flames (Journal of Engineering for Gas Turbines and Power, 2025) | 2. Measurements of CO and NOx Emissions From Premixed Turbulent Methane/Hydrogen Flames (Journal of Engineering for Gas Turbines and Power, 2025)</t>
         </is>
       </c>
       <c r="X9" s="3">
-        <f>HYPERLINK("https://doi.org/10.1115/1.4053164 | https://doi.org/10.1017/jfm.2021.433", "https://doi.org/10.1115/1.4053164 | https://doi.org/10.1017/jfm.2021.433")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/1.4069796 | https://doi.org/10.1115/1.4069625", "https://doi.org/10.1115/1.4069796 | https://doi.org/10.1115/1.4069625")</f>
         <v/>
       </c>
       <c r="Y9" s="2" t="inlineStr">
         <is>
-          <t>measuring transverse flame transfer functions via phase-locked OH-PLIF in a swirl-stabilized combustor, demonstrating that transverse excitation produces peak gain at the swirler geometric resonance rather than the convective residence time, directly altering annular combustor thermoacoustic stability predictions.</t>
+          <t>investigating swirl geometry effects on flame morphology and emissions in rich premixed NH3-air flames for an RRQL system, demonstrating that compact flames minimize wall quenching and enable post-flame relaxation to suppress NOx and NH3 emissions.</t>
         </is>
       </c>
       <c r="Z9" s="2" t="inlineStr">
@@ -8163,64 +8155,64 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Computational soft-matter and mesoscale fluid mechanics -- lattice Boltzmann / immersed boundary simulations of active elastic filaments, magnetically controlled microswimmers, elastic capsule deformation in microchannel flow, and interfacial transport in patterned soft-wetting surfaces.</t>
+          <t>Quantum lattice Boltzmann methods (QLBM) for phase-change heat transfer and mesoscale modeling of responsive hydrogel interfaces and fluid-structure interaction.</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Lattice-Boltzmann Method (LBM), Immersed Boundary Method (IBM), Elastic network membrane model, Magnetic dipole actuator model, Finite element structural coupling</t>
+          <t>Quantum Lattice Boltzmann Method (QLBM), Dissipative Particle Dynamics (DPD), Quantum circuit state storage (53 qubits), Immersed Boundary Method (IBM)</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Magnetic soft robot locomotion across unstructured terrains</t>
+          <t>Neutron Reflectometry and Compression of Graded Hydrogel Surfaces</t>
         </is>
       </c>
       <c r="P10" s="3">
-        <f>HYPERLINK("https://doi.org/10.1002/adma.202307002", "https://doi.org/10.1002/adma.202307002")</f>
+        <f>HYPERLINK("https://doi.org/10.1002/admi.70580", "https://doi.org/10.1002/admi.70580")</f>
         <v/>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>simulating magnetic soft robot locomotion with IBM-coupled elastic shell mechanics across terrain roughness Ra/L = 0-0.3, demonstrating undulatory gaits outperform rolling by 2.8x on irregular substrates with gait switching at critical roughness threshold Ra/L = 0.12.</t>
+          <t>investigating depth-wise graded hydrogel layers via neutron reflectometry and DPD mesoscale simulations, demonstrating that near-surface polymer network collapse under compression dictates contact stress modulation and effective elastic modulus.</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>IBM-coupled elastic shell finite element mechanics simulates magnetic soft robot locomotion across substrates with random height perturbations up to 30% of body length. Undulatory gaits outperform rolling gaits by 2.8x on irregular substrates. Gait switching occurs at a terrain roughness threshold of Ra/L = 0.12.</t>
+          <t>ABSTRACT Polyacrylamide hydrogels with depth‐wise gradients in polymer density (i.e., surface gel layers) are ideal synthetic models to understand stress modulation in hierarchical, compositionally‐graded biological tissues, including articular cartilage, in part, due to their similarities in water content and network structure. This work investigated surface gel layer thickness and crosslinker mobility (e.g., covalent crosslinks vs. physical entanglements) in polyacrylamide hydrogels and their impact on mechanical properties via confocal microscopy, indentation and compression measurements, neutron reflectivity, and mesoscale modeling. Hydrogels polymerized against oxygen‐permeable polydimethylsiloxane exhibited thicker surface gel layers and significantly lower elastic modulus compared to hydrogels polymerized against oxygen‐impermeable glass. Physical entanglements lowered the hydrogel elastic modulus within the surface gel layer and throughout the bulk. Neutron reflectivity revealed the collapse of near‐surface polymer networks under compressive loads, in good agreement with dissipative particle dynamics (DPD) simulations. Our results suggested that both the hydrogel elastic...</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>Elastic capsules in shear flow near a planar wall: Numerical simulation</t>
+          <t>Quantum lattice Boltzmann algorithm for heat transfer with phase change</t>
         </is>
       </c>
       <c r="T10" s="3">
-        <f>HYPERLINK("https://doi.org/10.1063/5.0078753", "https://doi.org/10.1063/5.0078753")</f>
+        <f>HYPERLINK("https://doi.org/10.1088/2058-9565/ae7b7c", "https://doi.org/10.1088/2058-9565/ae7b7c")</f>
         <v/>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>simulating elastic capsule wall migration via IB-LBM at Ca=0.1-0.5 and h/a=0.1-2.0, demonstrating near-wall membrane amplifies principal strain by 45-68% relative to far-field and lateral migration velocity scales as Ca*(h/a)^-3.</t>
+          <t>implementing a quantum lattice Boltzmann method (QLBM) on 17 lattice nodes using 53 qubits for phase-change heat transfer, demonstrating accurate moving interface tracking with temperature RMS errors of order 0.01 relative to classical analytical solutions.</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>IB-LBM simulates elastic capsule dynamics in shear flow near a rigid wall. Near-wall membrane deformation is amplified by 45-68% relative to far-field, with maximum principal strain of 0.42 at Ca=0.5, h/a=0.15. Lateral migration velocity scales as Ca*(h/a)^-3.</t>
+          <t>Abstract Heat transfer involving phase change is computationally intensive due to moving phase boundaries, nonlinear computations, and time step restrictions. This paper presents a quantum lattice Boltzmann method (QLBM) for simulating heat transfer with phase change. The approach leverages the statistical nature of the lattice Boltzmann method (LBM) while addressing the challenges of discontinuous phase transitions in quantum computing. The method implements an interface-tracking strategy that partitions the problem into separate solid and liquid domains, enabling the algorithm to handle the discontinuity in the enthalpy–temperature relationship. We store phase change information in the quantum circuit to reduce information exchange between classical and quantum hardware, a bottleneck in many quantum applications. Results from the implementation agree with both classical LBM and analytical solutions, demonstrating QLBM as an effective approach for analyzing thermal systems with phase transitions. Simulations using 17 lattice nodes with 53 qubits demonstrate temperature root-mean-square errors of order 0.01 when compared against classical solutions. The method accurately tracks ...</t>
         </is>
       </c>
       <c r="W10" s="2" t="inlineStr">
         <is>
-          <t>1. Magnetic soft robot locomotion across unstructured terrains (Advanced Materials, 2023) | 2. Elastic capsules in shear flow near a planar wall: Numerical simulation (Biomicrofluidics, 2022)</t>
+          <t>1. Neutron Reflectometry and Compression of Graded Hydrogel Surfaces (Advanced Materials Interfaces, 2026) | 2. Quantum lattice Boltzmann algorithm for heat transfer with phase change (Quantum Science and Technology, 2026)</t>
         </is>
       </c>
       <c r="X10" s="3">
-        <f>HYPERLINK("https://doi.org/10.1002/adma.202307002 | https://doi.org/10.1063/5.0078753", "https://doi.org/10.1002/adma.202307002 | https://doi.org/10.1063/5.0078753")</f>
+        <f>HYPERLINK("https://doi.org/10.1002/admi.70580 | https://doi.org/10.1088/2058-9565/ae7b7c", "https://doi.org/10.1002/admi.70580 | https://doi.org/10.1088/2058-9565/ae7b7c")</f>
         <v/>
       </c>
       <c r="Y10" s="2" t="inlineStr">
         <is>
-          <t>simulating magnetic soft robot locomotion with IBM-coupled elastic shell mechanics across terrain roughness Ra/L = 0-0.3, demonstrating undulatory gaits outperform rolling by 2.8x on irregular substrates with gait switching at critical roughness threshold Ra/L = 0.12.</t>
+          <t>investigating depth-wise graded hydrogel layers via neutron reflectometry and DPD mesoscale simulations, demonstrating that near-surface polymer network collapse under compression dictates contact stress modulation and effective elastic modulus.</t>
         </is>
       </c>
       <c r="Z10" s="2" t="inlineStr">
@@ -8228,11 +8220,7 @@
           <t>Skip To Keyboard Navigation Toggle navigation George W. Woodruff School of Mechanical Engineering Main navigation Home About Ch...</t>
         </is>
       </c>
-      <c r="AA10" s="2" t="inlineStr">
-        <is>
-          <t>"Neutron Reflectometry and Compression of Graded Hydrogel Surfaces" [Advanced Materials Interfaces] (2026) [DOI: https://doi.org/10.1002/admi.70580] | "Quantum lattice Boltzmann algorithm for heat transfer with phase change" [Quantum Science and Technology] (2026) [DOI: https://doi.org/10.1088/2058-9565/ae7b7c] | "Undulatory hydrodynamics of tapered elastic plates in viscous fluid" [Journal of Fluid Mechanics] (2026) [DOI: https://doi.org/10.1017/jfm.2026.11157] | "MEASUREMENT TECHNIQUE MEASUREMENT OF ABSORBED DOSE IN WATER DURING IRRADIATION IN CARBON ION AND PROTON BEAMS USING THERMAL LUMINESCENCE DOSIMETERS номер в ФИФ: ФР.1.38.2025.52532" (2026) [DOI: https://doi.org/10.13140/rg.2.2.36020.51847] | "Mesoscale Modeling of Hydrogels Under Frictional Shear Stress" [Macromolecules] (2025) [DOI: https://doi.org/10.1021/acs.macromol.5c01748]</t>
-        </is>
-      </c>
+      <c r="AA10" s="2" t="inlineStr"/>
       <c r="AB10" s="2" t="inlineStr">
         <is>
           <t>"Deformations in Si−Li Anodes Upon Electrochemical Alloying in Nano-Confined Space" [Journal of the American Chemical Society] (2010, 324 cites) [DOI: https://doi.org/10.1021/ja1031997] | "Ultrasoft microgels displaying emergent platelet-like behaviours" [Nature Materials] (2014, 221 cites) [DOI: https://doi.org/10.1038/nmat4066] | "Harnessing Janus Nanoparticles to Create Controllable Pores in Membranes" [ACS Nano] (2008, 198 cites) [DOI: https://doi.org/10.1021/nn8000998]</t>
@@ -8363,64 +8351,64 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Lattice-Boltzmann and fluctuating lattice-Boltzmann methods for multiphase suspension flows, deformable capsule dynamics in microcirculation, and turbulent fiber suspensions -- bridging colloidal-scale stochastic physics with engineering-scale flow predictions.</t>
+          <t>Direct numerical simulation (DNS) and experimental scaling of bubble interactions in decaying dynamic turbulence, Hinze-scale evolution, and microbubble mass-transfer control.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Lattice-Boltzmann Method (LBM), Fluctuating Lattice-Boltzmann (FLB), Immersed Boundary Method (IBM), Spectral Element DNS, Capsule membrane finite-element models</t>
+          <t>DNS of bubble-laden homogeneous isotropic turbulence, Particle Shadow Velocimetry (PSV), High-speed back-lit shadowgraphy, Lattice Boltzmann suspension modeling</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>Lattice Boltzmann simulation of the dynamics of capsule suspensions in shear flow</t>
+          <t>On the scaling of bubble interactions in dynamic turbulence: theoretical, numerical, and experimental study</t>
         </is>
       </c>
       <c r="P11" s="3">
-        <f>HYPERLINK("https://doi.org/10.1103/PhysRevFluids.7.054302", "https://doi.org/10.1103/PhysRevFluids.7.054302")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2607.25251", "https://doi.org/10.48550/arxiv.2607.25251")</f>
         <v/>
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>coupling LBM with finite-element capsule membrane models for volume fractions up to 0.40, demonstrating hydrodynamic capsule interactions produce shear-induced diffusivity of 3.2e-3 and drive a 340% viscosity increase from dilute to concentrated regimes.</t>
+          <t>investigating bubbly decaying homogeneous isotropic turbulence via DNS and experiments, demonstrating that when dissipation decays rapidly the Hinze scale overtakes bubble diameter, driving a transition from super-Hinze to capillary-dominated sub-Hinze scaling.</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>LBM coupled with finite-element membrane models studies capsule suspensions in shear flow at volume fractions up to 0.40. Shear-induced diffusion coefficient D_s/gamma_dot*a^2 = 3.2e-3, comparable to experimental hard-sphere measurements. Bulk suspension viscosity increases by 340% from dilute to concentrated regime at the same capillary number.</t>
+          <t>This study investigates dilute bubbly decaying homogeneous isotropic turbulence at high Reynolds number using theory, direct numerical simulation, and experiments. The turbulent kinetic energy and dissipation rate follow power-law decay, while the bubble population reorganizes relative to the evolving Hinze scale. When the dissipation decays sufficiently rapidly, the Hinze scale grows faster than the characteristic bubble diameter, driving the population from super-Hinze toward sub-Hinze sizes. The system passes through a mixed regime in which coalescence dominates but breakup remains active, followed by a pure-coalescence regime. Residual breakup in the mixed regime increases the number of small bubbles and enhances coalescence, leading to faster growth of the characteristic bubble size. DNS of dilute bubble-laden turbulence shows decay exponents close to single-phase turbulence and a bubble-size distribution that shifts toward smaller diameter relative to the Hinze scale. Before the transition, the distribution exhibits two power-law ranges associated with capillary effects and inertial breakup; after the transition, it approaches a single capillary-dominated scaling. Theory a...</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>Fluctuating lattice Boltzmann method for complex fluids and dense suspensions</t>
+          <t>Mass-Transfer Control With Microbubbles in Highly Turbulent Decaying Flows</t>
         </is>
       </c>
       <c r="T11" s="3">
-        <f>HYPERLINK("https://doi.org/10.1017/jfm.2021.432", "https://doi.org/10.1017/jfm.2021.432")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2604.24520", "https://doi.org/10.48550/arxiv.2604.24520")</f>
         <v/>
       </c>
       <c r="U11" s="2" t="inlineStr">
         <is>
-          <t>extending fluctuating LBM to dense suspensions at volume fractions 0.35-0.55, demonstrating sub-diffusive caging dynamics with MSD ~ t^0.72 and predicting viscosity divergence at 0.63 consistent with Krieger-Dougherty theory.</t>
+          <t>combining extreme turbulence (Re_lambda ~ 10^3) with minute surfactant addition (~0.01% CMC) in a straight duct, demonstrating that interfacial tuning arrests bubble coalescence and dictates micron-scale bubble size distributions.</t>
         </is>
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>The fluctuating LBM is extended to dense suspensions with thermodynamically consistent Langevin noise. At volume fractions 0.35-0.55, the model captures sub-diffusive dynamics with MSD scaling as t^0.72, consistent with colloidal glass transition theories. Suspension viscosity diverges at volume fraction 0.63, consistent with Krieger-Dougherty theory.</t>
+          <t>We hypothesize that combining extreme turbulence with a minute reduction in surface tension $σ$ (surface tension of the liquid) using surfactant provides a simple and scalable route for controlling micron scale bubble size in gas--liquid systems. To test this, we generate high-intensity turbulence using a multiphase pump [turbulent intensity $\ge 40\%$; Taylor Reynolds number $Re_λ=\mathcal{O}(10^3)$; bulk Reynolds number $Re=\mathcal{O}(10^5)$] feeding a straight duct, which produces a decaying turbulent flow where, without additives, bubble coalescence dominates and causes monotonic downstream growth in the mean diameter $d_\mathrm{avg}$ of the bubbles. This growth is governed by the turbulent dissipation rate $\varepsilon$. High-speed imaging, back-lit shadowgraph and particle shadow velocimetry (PSV) quantify bubble statistics ($d_\mathrm{avg}$, and the bubble-size distribution) and turbulence metrics (turbulent kinetic energy $k$, turbulence intensity $\mathcal{I}$, and dissipation rate $\varepsilon$). We then introduce a minute amount ($\sim 0.01\%$ critical micelle concentration) of additive that produces a slight reduction in $σ$, used here only as an interfacial tuning ...</t>
         </is>
       </c>
       <c r="W11" s="2" t="inlineStr">
         <is>
-          <t>1. LBM simulation of capsule suspensions in shear flow (Physical Review Fluids, 2022) | 2. Fluctuating LBM for dense suspensions (Journal of Fluid Mechanics, 2021)</t>
+          <t>1. On the scaling of bubble interactions in dynamic turbulence: theoretical, numerical, and experimental study (arXiv, 2026) | 2. Mass-Transfer Control With Microbubbles in Highly Turbulent Decaying Flows (arXiv, 2026)</t>
         </is>
       </c>
       <c r="X11" s="3">
-        <f>HYPERLINK("https://doi.org/10.1103/PhysRevFluids.7.054302 | https://doi.org/10.1017/jfm.2021.432", "https://doi.org/10.1103/PhysRevFluids.7.054302 | https://doi.org/10.1017/jfm.2021.432")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2607.25251 | https://doi.org/10.48550/arxiv.2604.24520", "https://doi.org/10.48550/arxiv.2607.25251 | https://doi.org/10.48550/arxiv.2604.24520")</f>
         <v/>
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>coupling LBM with finite-element capsule membrane models for volume fractions up to 0.40, demonstrating hydrodynamic capsule interactions produce shear-induced diffusivity of 3.2e-3 and drive a 340% viscosity increase from dilute to concentrated regimes.</t>
+          <t>investigating bubbly decaying homogeneous isotropic turbulence via DNS and experiments, demonstrating that when dissipation decays rapidly the Hinze scale overtakes bubble diameter, driving a transition from super-Hinze to capillary-dominated sub-Hinze scaling.</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr">
@@ -8563,64 +8551,64 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Multi-fidelity rotorcraft aeromechanics -- coupling CAMRAD II with CFD/CSD for dynamic stall, blade-vortex interaction, and coaxial rotor-wake aerodynamics to enable next-generation Urban Air Mobility eVTOL vehicle design.</t>
+          <t>Proprotor-wing interactional aerodynamics across tiltrotor conversion maneuvers, mid-to-high-fidelity CFD coupling (Helios / OVERFLOW / ROAM), and reduced-order wake models for Advanced Air Mobility.</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>CAMRAD II, Overset CFD/CSD loose coupling, Unsteady Vortex Lattice Method (UVLM), GT-Hybrid RANS-LES, Aeroflite wind tunnel PIV validation</t>
+          <t>Helios-OVERFLOW overset CFD, Reduced Order Aerodynamic Model (ROAM), Actuator Line Model (ALM), Immersed Boundary Method (IBM), Power spectral density surface pressure analysis</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Validation of an Unsteady Vortex Lattice Method for Coaxial Rotor Wake Interactions</t>
+          <t>Physics of the Proprotor–Wing Interactional Aerodynamics Across the Tiltrotor Conversion Maneuver</t>
         </is>
       </c>
       <c r="P12" s="3">
-        <f>HYPERLINK("https://doi.org/10.4050/JAHS.67.032007", "https://doi.org/10.4050/JAHS.67.032007")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.c038965", "https://doi.org/10.2514/1.c038965")</f>
         <v/>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>validating a free-wake UVLM for coaxial rotor wake mutual induction against Georgia Tech PIV data, demonstrating 6.4% RMS blade normal force accuracy and capturing the figure-8 loading signature in the lower rotor from upper-rotor tip-vortex impingement.</t>
+          <t>simulating two-way coupled proprotor-wing interaction across tilt angles in 15-degree increments using high-fidelity CFD, demonstrating that wing surface pressure PSD reveals dominant wake excitation frequencies during tiltrotor conversion maneuvers.</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>An unsteady vortex lattice method (UVLM) for coaxial rotor aerodynamics is validated against GT Aeroflite wind tunnel PIV data. The UVLM predicts blade normal force within 6.4% RMS error across the azimuth and reproduces the characteristic figure-8 loading signature in the lower rotor due to upper rotor tip vortex impingement.</t>
+          <t>The conversion maneuver is one of the most complex and hazardous aspects of tiltrotor operations. The complex interactions increase pilot workload and vibratory wing loads, making it imperative to further understand and accurately predict this dynamic operation. An extensively correlated high-fidelity computational fluid dynamics (CFD) model elucidates the physics within these two-way coupled aerodynamic interactions for a generic model-scale tractor proprotor–wing configuration. Quasi-static evaluations are conducted for proprotor tilt angles in fifteen degree increments to capture the conversion from low-speed edgewise flight to cruise. To assess and quantify the coupled proprotor–wing interactions, additional assessments of an isolated wing at two relevant wing angles of attack and an isolated proprotor operating at all tilt angles were conducted. Wing thickness and loading were mildly correlated with the proprotor loads due to the large proprotor–wing separation relative to the proprotor radius. The proprotor-to-wing effects were assessed using a power spectral density of the wing surface pressure within the proprotor wake. This novel approach elucidates the dominant frequen...</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>Multi-fidelity aeromechanical analysis of a UH-60A rotor in forward flight using loosely coupled CFD/CSD</t>
+          <t>Mid-Fidelity Investigation of the Proprotor-Wing Aerodynamic Interactions across the Tiltrotor Conversion Maneuver</t>
         </is>
       </c>
       <c r="T12" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.J059977", "https://doi.org/10.2514/1.J059977")</f>
+        <f>HYPERLINK("https://doi.org/10.4050/f-0082-2026-0243", "https://doi.org/10.4050/f-0082-2026-0243")</f>
         <v/>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>loosely coupling overset RANS with CAMRAD II across UH-60A advance ratios from 0.15 to 0.368, demonstrating rotor performance within 4.5% of flight test data and capturing dynamic stall vibratory 4P loads at high-advance-ratio conditions.</t>
+          <t>evaluating the Helios mid-fidelity ROAM actuator line model against OVERFLOW for proprotor-wing conversion, demonstrating that adaptive mesh refinement (AMR) in the off-body Cartesian domain is essential for capturing proprotor vortex trajectory and wing load distribution.</t>
         </is>
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>Loosely coupled CFD/CSD methodology is applied to the UH-60A main rotor across advance ratios from mu = 0.15 to 0.368. Rotor performance including thrust, torque, and blade pitch angles agree with UH-60A flight test data within 4.5%. Dynamic stall at high advance ratios is captured with qualitative agreement to flight test vibratory loads at 4P frequency.</t>
+          <t>This paper assesses the capabilities and limitations of mid-fidelity computational fluid dynamics (CFD) approaches when resolving the complex aerodynamic interactions for a generic model-scale proprotor-wing configuration across the tiltrotor conversion maneuver. The Helios mid-fidelity Reduced Order Aerodynamic Model (ROAM) is evaluated against prior extensively validated high-fidelity Helios-OVERFLOW assessments for the proprotor-wing configuration. The ROAM actuator line model (ALM), which represents the proprotor blade via source terms injected into the off-body Cartesian domain, is assessed for the isolated proprotor configuration at several mesh resolutions to understand the requirements to accurately resolve the proprotor physics across the conversion maneuver. The impact of adaptive mesh refinement (AMR) on ROAM's ability to resolve the proprotor physics is also investigated. Next, the flow characteristics and wing loads are evaluated using the ROAM immersed boundary method (IBM) for the isolated wing. The sensitivity of the ROAM IBM predictions to mesh resolution and boundary condition selection is quantified in these assessments. Leveraging the findings from the isolat...</t>
         </is>
       </c>
       <c r="W12" s="2" t="inlineStr">
         <is>
-          <t>1. Validation of an Unsteady Vortex Lattice Method for Coaxial Rotor Wake Interactions (JAHS, 2022) | 2. Multi-fidelity aeromechanical analysis of UH-60A rotor using loosely coupled CFD/CSD (AIAA J., 2021)</t>
+          <t>1. Physics of the Proprotor–Wing Interactional Aerodynamics Across the Tiltrotor Conversion Maneuver (Journal of Aircraft, 2026) | 2. Mid-Fidelity Investigation of the Proprotor-Wing Aerodynamic Interactions across the Tiltrotor Conversion Maneuver (2026)</t>
         </is>
       </c>
       <c r="X12" s="3">
-        <f>HYPERLINK("https://doi.org/10.4050/JAHS.67.032007 | https://doi.org/10.2514/1.J059977", "https://doi.org/10.4050/JAHS.67.032007 | https://doi.org/10.2514/1.J059977")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.c038965 | https://doi.org/10.4050/f-0082-2026-0243", "https://doi.org/10.2514/1.c038965 | https://doi.org/10.4050/f-0082-2026-0243")</f>
         <v/>
       </c>
       <c r="Y12" s="2" t="inlineStr">
         <is>
-          <t>validating a free-wake UVLM for coaxial rotor wake mutual induction against Georgia Tech PIV data, demonstrating 6.4% RMS blade normal force accuracy and capturing the figure-8 loading signature in the lower rotor from upper-rotor tip-vortex impingement.</t>
+          <t>simulating two-way coupled proprotor-wing interaction across tilt angles in 15-degree increments using high-fidelity CFD, demonstrating that wing surface pressure PSD reveals dominant wake excitation frequencies during tiltrotor conversion maneuvers.</t>
         </is>
       </c>
       <c r="Z12" s="2" t="inlineStr">
@@ -8759,64 +8747,64 @@
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Stochastic optimal control theory, Hamilton-Jacobi-Bellman PDEs, and adaptive numerical methods for diffusion-dominated transport -- developing efficient solvers for high-dimensional control problems in turbulent mixing, ensemble Kalman filtering, and molecular dynamics.</t>
+          <t>Dynamics-guided weighted weak-form identification of differential equations from noisy trajectories and discrete Mean Field Games (Graph MFG) on finite graphs as initial value optimization.</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Hamilton-Jacobi-Bellman (HJB) finite-difference solvers, Policy iteration, Ensemble Kalman Inversion (EKI), Stochastic Runge-Kutta, Adaptive mesh refinement (h-refinement)</t>
+          <t>Dynamics-guided weighted weak form, Feature voting ensembles, Graph Mean Field Games (Graph MFG), Neural network ODE integrators, Hamilton-Jacobi-Bellman optimization</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Efficient numerical methods for high-dimensional stochastic control with application to turbulent diffusion</t>
+          <t>Identification of Differential Equations by Dynamics-Guided Weighted Weak Form with Voting</t>
         </is>
       </c>
       <c r="P13" s="3">
-        <f>HYPERLINK("https://doi.org/10.1137/21M1409124", "https://doi.org/10.1137/21M1409124")</f>
+        <f>HYPERLINK("https://doi.org/10.4208/cicp.oa-2025-0163", "https://doi.org/10.4208/cicp.oa-2025-0163")</f>
         <v/>
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>solving 6D HJB equations via sparse-grid policy iteration for turbulent scalar mixing control at Re_lambda=150, demonstrating 38% scalar variance reduction using 4.2x fewer grid points through dimension-independent O(h^4*|log h|^(d-1)) convergence.</t>
+          <t>developing dynamics-guided weighted weak formulations with voting strategies for PDE discovery from single noisy trajectories, demonstrating robust recovery of governing differential terms and coefficients by weighting high-dynamic regions.</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>Sparse tensor grid HJB solvers with policy iteration applied to 6D turbulent scalar mixing control at Re_lambda=150. The sparse grid achieves dimension-independent convergence O(h^4*|log h|^(d-1)) vs O(h^2) for standard solvers. Controls reduce scalar variance by 38% using 4.2x fewer grid points than full-tensor discretization.</t>
+          <t>In the identification of differential equations from data, significant progresses have been made with the weak/integral formulation. In this paper, we explore the direction of finding more efficient and robust test functions adaptively given the observed data. While this is a difficult task, we propose weighting a collection of localized test functions for better identification of differential equations from a single trajectory of noisy observations on the differential equation. We find that using high dynamic regions is effective in finding the equation as well as the coefficients, and propose a dynamics indicator per differential term and weight the weak form accordingly. For stable identification against noise, we further introduce a voting strategy to identify the active features from an ensemble of recovered results by selecting the features that frequently occur in different weighting of test functions. Systematic numerical experiments are provided to demonstrate the robustness of our method.</t>
         </is>
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>Adaptive mesh refinement for Hamilton-Jacobi-Bellman equations in continuous-time stochastic control</t>
+          <t>Discrete Mean Field Games on Finite Graphs as Initial Value Optimization</t>
         </is>
       </c>
       <c r="T13" s="3">
-        <f>HYPERLINK("https://doi.org/10.4208/jcm.2009-m2019-0214", "https://doi.org/10.4208/jcm.2009-m2019-0214")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2604.05685", "https://doi.org/10.48550/arxiv.2604.05685")</f>
         <v/>
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
-          <t>applying AMR with gradient-discontinuity indicators to HJB solvers for stochastic control, demonstrating 75-82% reduction in degrees of freedom vs uniform grids while maintaining L-inf error below 1% and recovering optimal O(h^2) convergence at the free boundary.</t>
+          <t>reformulating discrete potential Mean Field Games on finite graphs as initial value optimization problems (Graph MFG-IV), demonstrating reduced search space by utilizing coupled Hamilton-Jacobi ODE integrators without full time-discretization.</t>
         </is>
       </c>
       <c r="V13" s="2" t="inlineStr">
         <is>
-          <t>AMR with a posteriori gradient-discontinuity error estimators for HJB PDE solvers in stochastic control. Applied to LQR with state constraints, stopping-time problem, and pursuit-evasion game. AMR reduces degrees of freedom by 75-82% vs uniform grids while maintaining L-inf error below 1%.</t>
+          <t>In this paper, we propose an initial value fomulation of the discrete mean field games on finite graphs (Graph MFG), and design a neural network based approach to solve it. Graph MFG describes infinite, non-cooperative and interactive homogeneous agents move on node states through the edges to optimize their own goals. Nash Equilibrium of the Graph MFG is characterized by a coupled ordinary differential equations (ODE) system, including the discrete forward continuity equation and the discrete backward Hamilton-Jacobi equation. In this paper, we mainly focus on the potential mean field games (Potential MFG) on finite graphs, which has an infinite-dimensional constrained optimization structure. We reformulate Potential MFG as an initial value finite-dimentional optimization problem with dynamics constrains, names Graph MFG-IV. Specifically, the initial condition of the Hamilton-Jacobi equation is regarded as the unique variable, constrained by the coupled Hamilton-Jacobi and continuity equation system as the ODE integrator. This formulation is a reduced-order model, which avoids time-discretization of the infinite-dimensional path and has a much smaller searching space than the g...</t>
         </is>
       </c>
       <c r="W13" s="2" t="inlineStr">
         <is>
-          <t>1. Efficient numerical methods for high-dimensional stochastic control with application to turbulent diffusion (SIAM J. Control Optim., 2022) | 2. Adaptive mesh refinement for HJB equations in stochastic control (J. Computational Mathematics, 2021)</t>
+          <t>1. Identification of Differential Equations by Dynamics-Guided Weighted Weak Form with Voting (Communications in Computational Physics, 2026) | 2. Discrete Mean Field Games on Finite Graphs as Initial Value Optimization (arXiv, 2026)</t>
         </is>
       </c>
       <c r="X13" s="3">
-        <f>HYPERLINK("https://doi.org/10.1137/21M1409124 | https://doi.org/10.4208/jcm.2009-m2019-0214", "https://doi.org/10.1137/21M1409124 | https://doi.org/10.4208/jcm.2009-m2019-0214")</f>
+        <f>HYPERLINK("https://doi.org/10.4208/cicp.oa-2025-0163 | https://doi.org/10.48550/arxiv.2604.05685", "https://doi.org/10.4208/cicp.oa-2025-0163 | https://doi.org/10.48550/arxiv.2604.05685")</f>
         <v/>
       </c>
       <c r="Y13" s="2" t="inlineStr">
         <is>
-          <t>solving 6D HJB equations via sparse-grid policy iteration for turbulent scalar mixing control at Re_lambda=150, demonstrating 38% scalar variance reduction using 4.2x fewer grid points through dimension-independent O(h^4*|log h|^(d-1)) convergence.</t>
+          <t>developing dynamics-guided weighted weak formulations with voting strategies for PDE discovery from single noisy trajectories, demonstrating robust recovery of governing differential terms and coefficients by weighting high-dynamic regions.</t>
         </is>
       </c>
       <c r="Z13" s="2" t="inlineStr">
@@ -8939,64 +8927,64 @@
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Variational image reconstruction, PDE-based level-set methods, and machine-learning-augmented numerical schemes for fluid interface tracking and multiphase flow image segmentation -- bridging applied harmonic analysis with high-order conservative transport methods.</t>
+          <t>Sampled Local WeakIdent (SLW-Ident) for discovering transitioning governing PDEs from single-set data and unified variational Potts frameworks for weakly supervised image segmentation.</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Variational level-set methods (Chan-Vese), Total variation minimization, PDE-constrained optimization, Physics-informed neural networks (PINNs), ADMM</t>
+          <t>Sampled Local WeakIdent (SLW-Ident), Local patch residual error analysis, Simplex-constrained Potts models, RKHS fuzzy membership functions, Weakly supervised deep learning loss</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>A variational framework for exemplar-based image inpainting integrated with level-set interface tracking</t>
+          <t>Identifying changing partial differential equations using Sampled Local WeakIdent</t>
         </is>
       </c>
       <c r="P14" s="3">
-        <f>HYPERLINK("https://doi.org/10.1137/21M1442626", "https://doi.org/10.1137/21M1442626")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2608.12479", "https://doi.org/10.48550/arxiv.2608.12479")</f>
         <v/>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>coupling exemplar-based TV inpainting with Chan-Vese level-set evolution via ADMM for corrupted multiphase flow images, demonstrating SSIM improvement from 0.74 to 0.91 and boundary localization error reduction to 1.2 pixels through joint rather than sequential optimization.</t>
+          <t>proposing Sampled Local WeakIdent (SLW-Ident) to identify changing governing equations from a single dataset, demonstrating that sampling localized patches and tracking residual errors accurately detects spatial transitions between varying-coefficient PDEs.</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>A variational framework couples exemplar-based TV inpainting with Chan-Vese level-set evolution via ADMM for fluid imaging. Applied to synthetic multiphase flow images with 30% corruption, the joint model achieves SSIM = 0.91 and boundary localization error of 1.2 pixels, vs SSIM = 0.74 for sequential inpainting-then-segmentation.</t>
+          <t>We propose Sampled Local WeakIdent (SLW-Ident), a framework for identifying changing governing equations from a single set of given data. Different from a typical approach of using finite element based approximation to represent varying coefficients, this paper explores a local approach in identification of differential equations. First, we present the power of Local WeakIdent which gives good local identification and is also computationally efficient with a small patch size, yet it can be sensitive to local perturbations. We propose SLW-Ident which stabilizes the identification process and also incorporates global information: we first sample patches in the whole given domain, identify equations for each sampled patch, then use residual error of these equations to find the transitions between different equations. We refer to a region where the support of the identified equation does not change to be a region of one equation. Within each region of one equation, we pick the most frequently identified equation as the identified equation, and find constant as well as varying coefficient PDEs within each region of one equation. This is justified by an uncertainty quantification theo...</t>
         </is>
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>Physics-informed neural networks for multiphase flow interface reconstruction from tomographic measurements</t>
+          <t>A Unified Variational Framework for Deep Weakly Supervised Image Segmentation</t>
         </is>
       </c>
       <c r="T14" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.jcp.2023.112086", "https://doi.org/10.1016/j.jcp.2023.112086")</f>
+        <f>HYPERLINK("https://arxiv.org/abs/2607.19669", "https://arxiv.org/abs/2607.19669")</f>
         <v/>
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>embedding incompressible two-phase NS and VOF physics residuals in PINNs for interface reconstruction from 12 tomographic angles, demonstrating interface curvature MAE of 0.08/cm versus 0.31/cm for unphysical FBP and sub-voxel (0.5 mm RMS) accuracy on experimental bubbly-flow CT data.</t>
+          <t>formulating a simplex-constrained Potts model with RKHS fuzzy membership for weakly supervised image segmentation, demonstrating superior accuracy over partial cross-entropy baselines without requiring dense ground-truth segmentation masks.</t>
         </is>
       </c>
       <c r="V14" s="2" t="inlineStr">
         <is>
-          <t>PINNs embedding two-phase incompressible Navier-Stokes and VOF transport in the loss function reconstruct gas-liquid interfaces from 12 tomographic projections. Interface curvature MAE = 0.08/cm vs 0.31/cm for filtered backprojection. Experimental X-ray CT bubbly flow interface located to within 0.5 mm RMS.</t>
+          <t>We propose a unified variational framework for image segmentation under sparse pixel-level supervision. Our method is based on a simplex-constrained Potts model with a smooth perimeter regularizer, yielding a convex, smooth energy functional that can be used as a training loss in weakly supervised deep learning paradigms or optimized efficiently using iterative methods. Sparse labels are incorporated into the data fidelity term by constructing a fuzzy membership function via a function extension problem in a Reproducing Kernel Hilbert Space (RKHS), which can effectively capture inhomogeneous intensity statistics. The derived discrete loss for training standard networks demonstrates robustness and consistent improvements over non-training and partial cross-entropy (PCE) baselines in experiments, achieving comparable performance without requiring ground-truth segmentation images.</t>
         </is>
       </c>
       <c r="W14" s="2" t="inlineStr">
         <is>
-          <t>1. Variational framework for exemplar-based inpainting integrated with level-set interface tracking (SIAM J. Imaging Sci., 2022) | 2. PINNs for multiphase flow interface reconstruction from tomographic measurements (JCP, 2023)</t>
+          <t>1. Identifying changing partial differential equations using Sampled Local WeakIdent (arXiv, 2026) | 2. A Unified Variational Framework for Deep Weakly Supervised Image Segmentation (arXiv, 2026)</t>
         </is>
       </c>
       <c r="X14" s="3">
-        <f>HYPERLINK("https://doi.org/10.1137/21M1442626 | https://doi.org/10.1016/j.jcp.2023.112086", "https://doi.org/10.1137/21M1442626 | https://doi.org/10.1016/j.jcp.2023.112086")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2608.12479 | https://arxiv.org/abs/2607.19669", "https://doi.org/10.48550/arxiv.2608.12479 | https://arxiv.org/abs/2607.19669")</f>
         <v/>
       </c>
       <c r="Y14" s="2" t="inlineStr">
         <is>
-          <t>coupling exemplar-based TV inpainting with Chan-Vese level-set evolution via ADMM for corrupted multiphase flow images, demonstrating SSIM improvement from 0.74 to 0.91 and boundary localization error reduction to 1.2 pixels through joint rather than sequential optimization.</t>
+          <t>proposing Sampled Local WeakIdent (SLW-Ident) to identify changing governing equations from a single dataset, demonstrating that sampling localized patches and tracking residual errors accurately detects spatial transitions between varying-coefficient PDEs.</t>
         </is>
       </c>
       <c r="Z14" s="2" t="inlineStr">
@@ -9119,64 +9107,64 @@
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>High-order Runge-Kutta discontinuous Galerkin (RKDG) schemes, central compact WENO reconstruction, and entropy-stable finite difference methods for hyperbolic conservation laws -- developing structure-preserving schemes for compressible Euler/Navier-Stokes flows.</t>
+          <t>Neural networks with local converging input (NNLCI) for unstructured-grid supersonic CFD and multiphase Euler CFD simulations of bubble-driven fluidization hydrodynamics.</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Runge-Kutta Discontinuous Galerkin (RKDG), Central compact WENO (CC-WENO), Limiter-free high-order reconstruction, Entropy-stable flux schemes, Gauss-Seidel relaxation</t>
+          <t>Neural Network with Local Converging Input (NNLCI), Unstructured-grid supersonic Euler solvers, Multiphase Eulerian CFD, Population Balance Modeling (PBM)</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>A new fifth-order finite difference compact reconstruction unequal-sized WENO scheme for compressible flow</t>
+          <t>Neural Network with Local Converging Input for Unstructured-Grid Computational Fluid Dynamics</t>
         </is>
       </c>
       <c r="P15" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.jcp.2022.111140", "https://doi.org/10.1016/j.jcp.2022.111140")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.j063885", "https://doi.org/10.2514/1.j063885")</f>
         <v/>
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>designing a fifth-order compact-reconstruction unequal-sized WENO scheme for compressible Euler flows, demonstrating 4.2x reduction in L-inf error on smooth wave tests relative to WENO-JS while maintaining ENO-sharp shock capture without parameter tuning.</t>
+          <t>developing neural networks with local converging input (NNLCI) on unstructured grids for supersonic flows with shocks, demonstrating several orders of magnitude reduction in computing wall time with single-network generalization across multiple bump configurations.</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>A new fifth-order finite difference scheme combining compact reconstruction and unequal-sized WENO stencils is proposed for compressible Euler equations. Compared to standard fifth-order WENO-JS, the new scheme reduces L-inf error by a factor of 4.2 on smooth wave tests while maintaining ENO-sharp shock capture without parameter tuning.</t>
+          <t>In recent years, surrogate models based on deep neural networks have been widely used to solve partial differential equations for fluid flow physics. This kind of model focuses on global interpolation of the training data and thus requires a large network structure. The process is both time consuming and computationally costly. In the present study, we develop a neural network with local converging input (NNLCI) for high-fidelity prediction using unstructured data. The framework uses the local domain of dependence with converging coarse solutions as input, thereby greatly reducing computational resource and training time. As a validation case, the NNLCI method is applied to study two-dimensional inviscid supersonic flows in channels with bumps. Different bump geometries and locations are examined to benchmark the effectiveness and versatility of this new approach. The NNLCI method can accurately and efficiently capture the structure and dynamics of the entire flowfield, including regions with shock discontinuities. For a new bump configuration, the method can perform prediction with only one neural network, eliminating the need for repeated training of multiple networks for different geometries. A saving of computing wall time is achieved by several orders of magnitude against the high-fidelity simulation with the same level of accuracy. The demand on training data is modest, and the training data can be allocated sparsely. These features are especially advantageous compared with conventional global-to-global deep learning methods and physics-informed methods.</t>
         </is>
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>Central compact schemes with spectral-like resolution for computational aeroacoustics</t>
+          <t>Euler multiphase‐CFD simulation on a bubble‐driven gas–liquid–solid fluidized bed</t>
         </is>
       </c>
       <c r="T15" s="3">
-        <f>HYPERLINK("https://doi.org/10.1137/20M1371847", "https://doi.org/10.1137/20M1371847")</f>
+        <f>HYPERLINK("https://doi.org/10.1002/cjce.24742", "https://doi.org/10.1002/cjce.24742")</f>
         <v/>
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>constructing Hermite-based central compact schemes that maintain phase error below 0.1% over 75% of the resolved wavenumber band versus 50% for classical 10th-order explicit schemes, with demonstrated superiority on acoustic pulse propagation and Taylor-Green vortex at Re=1600.</t>
+          <t>simulating gas-liquid-solid fluidized beds via Eulerian multiphase CFD and population balance modeling, demonstrating that bubble coalescence shifts bubble diameters from 2-4 mm at the base to 5-10 mm at the top, dictating axial solids holdup.</t>
         </is>
       </c>
       <c r="V15" s="2" t="inlineStr">
         <is>
-          <t>Central compact finite difference schemes with spectral-like resolution are developed using Hermite-based interpolation. The 10th-order compact scheme maintains phase error below 0.1% over 75% of the resolved wavenumber band, compared to 50% for classical 10th-order explicit schemes, with superiority on acoustic pulse propagation and Taylor-Green vortex at Re=1600.</t>
+          <t>Abstract An integrated flow model was developed to simulate the fluidization hydrodynamics in a new bubble‐driven gas–liquid–solid fluidized bed using the computational fluid dynamic (CFD) method. The results showed that axial solids holdup is affected by grid size, bubble diameter, and the interphase drag models used in the simulation. Good agreements with experimental data could be obtained by adopting the following parameters: 5 mm grid, 1.2 mm bubble diameter, the Tomiyama gas–liquid model, the Schiller–Naumann liquid–solid model, and the Gidaspow gas–solid model. At full fluidization state, an internal circulation of particles flowing upward near the wall and downward in the centre is observed, which is in the opposite direction compared with the traditional core‐annular flow structure in a gas–solid fluidized bed. The simulated results are very sensitive to bubble diameters. Using smaller bubble diameters would lead to excessive liquid bed expansions and more solid accumulated at the bottom due to a bigger gas–liquid drag force, while bigger bubble diameters would result in a higher solid bed height caused by a smaller gas–solid drag force. Considering the actual bubble distribution, population balance model (PBM) is employed to characterize the coalescence and break up of bubbles. The calculated bubble diameters grow up from 2–4 mm at the bottom to 5–10 mm at the upper section of the bed, which are comparable to those observed in experiments. The simulation results could provide valuable information for the design and optimization of this new type of fluidized system.</t>
         </is>
       </c>
       <c r="W15" s="2" t="inlineStr">
         <is>
-          <t>1. Fifth-order finite difference compact reconstruction unequal-sized WENO for compressible flow (JCP, 2022) | 2. Central compact schemes with spectral-like resolution (SIAM J. Sci. Comput., 2021)</t>
+          <t>1. Neural Network with Local Converging Input for Unstructured-Grid Computational Fluid Dynamics (AIAA Journal, 2024) | 2. Euler multiphase‐CFD simulation on a bubble‐driven gas–liquid–solid fluidized bed (The Canadian Journal of Chemical Engineering, 2022)</t>
         </is>
       </c>
       <c r="X15" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.jcp.2022.111140 | https://doi.org/10.1137/20M1371847", "https://doi.org/10.1016/j.jcp.2022.111140 | https://doi.org/10.1137/20M1371847")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.j063885 | https://doi.org/10.1002/cjce.24742", "https://doi.org/10.2514/1.j063885 | https://doi.org/10.1002/cjce.24742")</f>
         <v/>
       </c>
       <c r="Y15" s="2" t="inlineStr">
         <is>
-          <t>designing a fifth-order compact-reconstruction unequal-sized WENO scheme for compressible Euler flows, demonstrating 4.2x reduction in L-inf error on smooth wave tests relative to WENO-JS while maintaining ENO-sharp shock capture without parameter tuning.</t>
+          <t>developing neural networks with local converging input (NNLCI) on unstructured grids for supersonic flows with shocks, demonstrating several orders of magnitude reduction in computing wall time with single-network generalization across multiple bump configurations.</t>
         </is>
       </c>
       <c r="Z15" s="2" t="inlineStr">

</xml_diff>